<commit_message>
impose 'other' not 'non-priority' naming of non ph1/ph2 procedures across all scripts
</commit_message>
<xml_diff>
--- a/04_reports/management_report/serverless_html/resources/SRASA procedure codes and phasing.xlsx
+++ b/04_reports/management_report/serverless_html/resources/SRASA procedure codes and phasing.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\stats\quality\srasa\(11) Scripts\Dylan\snap-srasa\04_reports\management_report\serverless_html\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\stats\quality\srasa\(11) Scripts\Bex\snap-srasa\04_reports\management_report\serverless_html\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8721D83B-8A03-45CB-938D-DA0255D6029C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7648ECA6-30DB-41F5-BD10-804ED9220A4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{1A0DCE31-DBDB-4A7A-8FC4-F05F39A42CDB}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="7" xr2:uid="{1A0DCE31-DBDB-4A7A-8FC4-F05F39A42CDB}"/>
   </bookViews>
   <sheets>
     <sheet name="Colorectal" sheetId="2" r:id="rId1"/>
@@ -20,7 +20,7 @@
     <sheet name="ENT" sheetId="6" r:id="rId5"/>
     <sheet name="Hepatobiliary" sheetId="7" r:id="rId6"/>
     <sheet name="Gastro-intestinal" sheetId="8" r:id="rId7"/>
-    <sheet name="Other" sheetId="9" r:id="rId8"/>
+    <sheet name="General surgery" sheetId="9" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1965" uniqueCount="885">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1965" uniqueCount="886">
   <si>
     <t>M61 Open excision of prostate</t>
   </si>
@@ -2698,6 +2698,9 @@
   </si>
   <si>
     <t>With benign neoplasm diagnosis OR anything excluding routine tonsillitis etc OR just the absence of cancer code (can be applied to over 16s only)</t>
+  </si>
+  <si>
+    <t>Other</t>
   </si>
 </sst>
 </file>
@@ -2900,6 +2903,7 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -2948,7 +2952,6 @@
     <xf numFmtId="0" fontId="1" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3427,19 +3430,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="17" t="s">
         <v>111</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
-      <c r="F1" s="16"/>
-      <c r="G1" s="16"/>
-      <c r="H1" s="16"/>
-      <c r="I1" s="16"/>
-      <c r="J1" s="16"/>
-      <c r="K1" s="16"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
+      <c r="G1" s="17"/>
+      <c r="H1" s="17"/>
+      <c r="I1" s="17"/>
+      <c r="J1" s="17"/>
+      <c r="K1" s="17"/>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
@@ -3474,7 +3477,7 @@
       <c r="E3" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="G3" s="32"/>
+      <c r="G3" s="16"/>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
@@ -3490,7 +3493,7 @@
       <c r="E4" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="G4" s="32"/>
+      <c r="G4" s="16"/>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
@@ -3857,19 +3860,19 @@
       <c r="E30" s="1"/>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A31" s="17" t="s">
+      <c r="A31" s="18" t="s">
         <v>112</v>
       </c>
-      <c r="B31" s="17"/>
-      <c r="C31" s="17"/>
-      <c r="D31" s="17"/>
-      <c r="E31" s="17"/>
-      <c r="F31" s="17"/>
-      <c r="G31" s="17"/>
-      <c r="H31" s="17"/>
-      <c r="I31" s="17"/>
-      <c r="J31" s="17"/>
-      <c r="K31" s="17"/>
+      <c r="B31" s="18"/>
+      <c r="C31" s="18"/>
+      <c r="D31" s="18"/>
+      <c r="E31" s="18"/>
+      <c r="F31" s="18"/>
+      <c r="G31" s="18"/>
+      <c r="H31" s="18"/>
+      <c r="I31" s="18"/>
+      <c r="J31" s="18"/>
+      <c r="K31" s="18"/>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A32" s="2" t="s">
@@ -4119,19 +4122,19 @@
       <c r="E48" s="1"/>
     </row>
     <row r="49" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A49" s="17" t="s">
-        <v>113</v>
-      </c>
-      <c r="B49" s="17"/>
-      <c r="C49" s="17"/>
-      <c r="D49" s="17"/>
-      <c r="E49" s="17"/>
-      <c r="F49" s="17"/>
-      <c r="G49" s="17"/>
-      <c r="H49" s="17"/>
-      <c r="I49" s="17"/>
-      <c r="J49" s="17"/>
-      <c r="K49" s="17"/>
+      <c r="A49" s="18" t="s">
+        <v>885</v>
+      </c>
+      <c r="B49" s="18"/>
+      <c r="C49" s="18"/>
+      <c r="D49" s="18"/>
+      <c r="E49" s="18"/>
+      <c r="F49" s="18"/>
+      <c r="G49" s="18"/>
+      <c r="H49" s="18"/>
+      <c r="I49" s="18"/>
+      <c r="J49" s="18"/>
+      <c r="K49" s="18"/>
     </row>
     <row r="50" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A50" s="2" t="s">
@@ -4691,19 +4694,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="19" t="s">
         <v>111</v>
       </c>
-      <c r="B1" s="18"/>
-      <c r="C1" s="18"/>
-      <c r="D1" s="18"/>
-      <c r="E1" s="18"/>
-      <c r="F1" s="18"/>
-      <c r="G1" s="18"/>
-      <c r="H1" s="18"/>
-      <c r="I1" s="18"/>
-      <c r="J1" s="18"/>
-      <c r="K1" s="18"/>
+      <c r="B1" s="19"/>
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19"/>
+      <c r="F1" s="19"/>
+      <c r="G1" s="19"/>
+      <c r="H1" s="19"/>
+      <c r="I1" s="19"/>
+      <c r="J1" s="19"/>
+      <c r="K1" s="19"/>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
@@ -5183,19 +5186,19 @@
       <c r="E32" s="1"/>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A33" s="19" t="s">
+      <c r="A33" s="20" t="s">
         <v>112</v>
       </c>
-      <c r="B33" s="19"/>
-      <c r="C33" s="19"/>
-      <c r="D33" s="19"/>
-      <c r="E33" s="19"/>
-      <c r="F33" s="19"/>
-      <c r="G33" s="19"/>
-      <c r="H33" s="19"/>
-      <c r="I33" s="19"/>
-      <c r="J33" s="19"/>
-      <c r="K33" s="19"/>
+      <c r="B33" s="20"/>
+      <c r="C33" s="20"/>
+      <c r="D33" s="20"/>
+      <c r="E33" s="20"/>
+      <c r="F33" s="20"/>
+      <c r="G33" s="20"/>
+      <c r="H33" s="20"/>
+      <c r="I33" s="20"/>
+      <c r="J33" s="20"/>
+      <c r="K33" s="20"/>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A34" s="2" t="s">
@@ -5236,19 +5239,19 @@
       <c r="E37" s="1"/>
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A38" s="19" t="s">
-        <v>113</v>
-      </c>
-      <c r="B38" s="19"/>
-      <c r="C38" s="19"/>
-      <c r="D38" s="19"/>
-      <c r="E38" s="19"/>
-      <c r="F38" s="19"/>
-      <c r="G38" s="19"/>
-      <c r="H38" s="19"/>
-      <c r="I38" s="19"/>
-      <c r="J38" s="19"/>
-      <c r="K38" s="19"/>
+      <c r="A38" s="20" t="s">
+        <v>885</v>
+      </c>
+      <c r="B38" s="20"/>
+      <c r="C38" s="20"/>
+      <c r="D38" s="20"/>
+      <c r="E38" s="20"/>
+      <c r="F38" s="20"/>
+      <c r="G38" s="20"/>
+      <c r="H38" s="20"/>
+      <c r="I38" s="20"/>
+      <c r="J38" s="20"/>
+      <c r="K38" s="20"/>
     </row>
     <row r="39" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A39" s="2" t="s">
@@ -5311,19 +5314,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="21" t="s">
         <v>111</v>
       </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20"/>
-      <c r="D1" s="20"/>
-      <c r="E1" s="20"/>
-      <c r="F1" s="20"/>
-      <c r="G1" s="20"/>
-      <c r="H1" s="20"/>
-      <c r="I1" s="20"/>
-      <c r="J1" s="20"/>
-      <c r="K1" s="20"/>
+      <c r="B1" s="21"/>
+      <c r="C1" s="21"/>
+      <c r="D1" s="21"/>
+      <c r="E1" s="21"/>
+      <c r="F1" s="21"/>
+      <c r="G1" s="21"/>
+      <c r="H1" s="21"/>
+      <c r="I1" s="21"/>
+      <c r="J1" s="21"/>
+      <c r="K1" s="21"/>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
@@ -5566,19 +5569,19 @@
       <c r="E19" s="1"/>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A20" s="21" t="s">
+      <c r="A20" s="22" t="s">
         <v>112</v>
       </c>
-      <c r="B20" s="21"/>
-      <c r="C20" s="21"/>
-      <c r="D20" s="21"/>
-      <c r="E20" s="21"/>
-      <c r="F20" s="21"/>
-      <c r="G20" s="21"/>
-      <c r="H20" s="21"/>
-      <c r="I20" s="21"/>
-      <c r="J20" s="21"/>
-      <c r="K20" s="21"/>
+      <c r="B20" s="22"/>
+      <c r="C20" s="22"/>
+      <c r="D20" s="22"/>
+      <c r="E20" s="22"/>
+      <c r="F20" s="22"/>
+      <c r="G20" s="22"/>
+      <c r="H20" s="22"/>
+      <c r="I20" s="22"/>
+      <c r="J20" s="22"/>
+      <c r="K20" s="22"/>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
@@ -5619,19 +5622,19 @@
       <c r="E24" s="1"/>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A25" s="21" t="s">
-        <v>113</v>
-      </c>
-      <c r="B25" s="21"/>
-      <c r="C25" s="21"/>
-      <c r="D25" s="21"/>
-      <c r="E25" s="21"/>
-      <c r="F25" s="21"/>
-      <c r="G25" s="21"/>
-      <c r="H25" s="21"/>
-      <c r="I25" s="21"/>
-      <c r="J25" s="21"/>
-      <c r="K25" s="21"/>
+      <c r="A25" s="22" t="s">
+        <v>885</v>
+      </c>
+      <c r="B25" s="22"/>
+      <c r="C25" s="22"/>
+      <c r="D25" s="22"/>
+      <c r="E25" s="22"/>
+      <c r="F25" s="22"/>
+      <c r="G25" s="22"/>
+      <c r="H25" s="22"/>
+      <c r="I25" s="22"/>
+      <c r="J25" s="22"/>
+      <c r="K25" s="22"/>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
@@ -5761,19 +5764,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A1" s="22" t="s">
+      <c r="A1" s="23" t="s">
         <v>111</v>
       </c>
-      <c r="B1" s="22"/>
-      <c r="C1" s="22"/>
-      <c r="D1" s="22"/>
-      <c r="E1" s="22"/>
-      <c r="F1" s="22"/>
-      <c r="G1" s="22"/>
-      <c r="H1" s="22"/>
-      <c r="I1" s="22"/>
-      <c r="J1" s="22"/>
-      <c r="K1" s="22"/>
+      <c r="B1" s="23"/>
+      <c r="C1" s="23"/>
+      <c r="D1" s="23"/>
+      <c r="E1" s="23"/>
+      <c r="F1" s="23"/>
+      <c r="G1" s="23"/>
+      <c r="H1" s="23"/>
+      <c r="I1" s="23"/>
+      <c r="J1" s="23"/>
+      <c r="K1" s="23"/>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
@@ -5989,19 +5992,19 @@
       <c r="E15" s="1"/>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A16" s="23" t="s">
+      <c r="A16" s="24" t="s">
         <v>112</v>
       </c>
-      <c r="B16" s="23"/>
-      <c r="C16" s="23"/>
-      <c r="D16" s="23"/>
-      <c r="E16" s="23"/>
-      <c r="F16" s="23"/>
-      <c r="G16" s="23"/>
-      <c r="H16" s="23"/>
-      <c r="I16" s="23"/>
-      <c r="J16" s="23"/>
-      <c r="K16" s="23"/>
+      <c r="B16" s="24"/>
+      <c r="C16" s="24"/>
+      <c r="D16" s="24"/>
+      <c r="E16" s="24"/>
+      <c r="F16" s="24"/>
+      <c r="G16" s="24"/>
+      <c r="H16" s="24"/>
+      <c r="I16" s="24"/>
+      <c r="J16" s="24"/>
+      <c r="K16" s="24"/>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
@@ -6253,19 +6256,19 @@
       <c r="E32" s="1"/>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A33" s="23" t="s">
-        <v>113</v>
-      </c>
-      <c r="B33" s="23"/>
-      <c r="C33" s="23"/>
-      <c r="D33" s="23"/>
-      <c r="E33" s="23"/>
-      <c r="F33" s="23"/>
-      <c r="G33" s="23"/>
-      <c r="H33" s="23"/>
-      <c r="I33" s="23"/>
-      <c r="J33" s="23"/>
-      <c r="K33" s="23"/>
+      <c r="A33" s="24" t="s">
+        <v>885</v>
+      </c>
+      <c r="B33" s="24"/>
+      <c r="C33" s="24"/>
+      <c r="D33" s="24"/>
+      <c r="E33" s="24"/>
+      <c r="F33" s="24"/>
+      <c r="G33" s="24"/>
+      <c r="H33" s="24"/>
+      <c r="I33" s="24"/>
+      <c r="J33" s="24"/>
+      <c r="K33" s="24"/>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A34" s="2" t="s">
@@ -6832,19 +6835,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A1" s="24" t="s">
+      <c r="A1" s="25" t="s">
         <v>111</v>
       </c>
-      <c r="B1" s="24"/>
-      <c r="C1" s="24"/>
-      <c r="D1" s="24"/>
-      <c r="E1" s="24"/>
-      <c r="F1" s="24"/>
-      <c r="G1" s="24"/>
-      <c r="H1" s="24"/>
-      <c r="I1" s="24"/>
-      <c r="J1" s="24"/>
-      <c r="K1" s="24"/>
+      <c r="B1" s="25"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
+      <c r="E1" s="25"/>
+      <c r="F1" s="25"/>
+      <c r="G1" s="25"/>
+      <c r="H1" s="25"/>
+      <c r="I1" s="25"/>
+      <c r="J1" s="25"/>
+      <c r="K1" s="25"/>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
@@ -7978,19 +7981,19 @@
       <c r="F71" s="8"/>
     </row>
     <row r="72" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A72" s="25" t="s">
+      <c r="A72" s="26" t="s">
         <v>112</v>
       </c>
-      <c r="B72" s="25"/>
-      <c r="C72" s="25"/>
-      <c r="D72" s="25"/>
-      <c r="E72" s="25"/>
-      <c r="F72" s="25"/>
-      <c r="G72" s="25"/>
-      <c r="H72" s="25"/>
-      <c r="I72" s="25"/>
-      <c r="J72" s="25"/>
-      <c r="K72" s="25"/>
+      <c r="B72" s="26"/>
+      <c r="C72" s="26"/>
+      <c r="D72" s="26"/>
+      <c r="E72" s="26"/>
+      <c r="F72" s="26"/>
+      <c r="G72" s="26"/>
+      <c r="H72" s="26"/>
+      <c r="I72" s="26"/>
+      <c r="J72" s="26"/>
+      <c r="K72" s="26"/>
     </row>
     <row r="73" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A73" s="2" t="s">
@@ -9158,19 +9161,19 @@
       <c r="F144" s="9"/>
     </row>
     <row r="145" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A145" s="25" t="s">
-        <v>113</v>
-      </c>
-      <c r="B145" s="25"/>
-      <c r="C145" s="25"/>
-      <c r="D145" s="25"/>
-      <c r="E145" s="25"/>
-      <c r="F145" s="25"/>
-      <c r="G145" s="25"/>
-      <c r="H145" s="25"/>
-      <c r="I145" s="25"/>
-      <c r="J145" s="25"/>
-      <c r="K145" s="25"/>
+      <c r="A145" s="26" t="s">
+        <v>885</v>
+      </c>
+      <c r="B145" s="26"/>
+      <c r="C145" s="26"/>
+      <c r="D145" s="26"/>
+      <c r="E145" s="26"/>
+      <c r="F145" s="26"/>
+      <c r="G145" s="26"/>
+      <c r="H145" s="26"/>
+      <c r="I145" s="26"/>
+      <c r="J145" s="26"/>
+      <c r="K145" s="26"/>
     </row>
     <row r="146" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A146" s="2" t="s">
@@ -9271,19 +9274,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A1" s="26" t="s">
+      <c r="A1" s="27" t="s">
         <v>111</v>
       </c>
-      <c r="B1" s="26"/>
-      <c r="C1" s="26"/>
-      <c r="D1" s="26"/>
-      <c r="E1" s="26"/>
-      <c r="F1" s="26"/>
-      <c r="G1" s="26"/>
-      <c r="H1" s="26"/>
-      <c r="I1" s="26"/>
-      <c r="J1" s="26"/>
-      <c r="K1" s="26"/>
+      <c r="B1" s="27"/>
+      <c r="C1" s="27"/>
+      <c r="D1" s="27"/>
+      <c r="E1" s="27"/>
+      <c r="F1" s="27"/>
+      <c r="G1" s="27"/>
+      <c r="H1" s="27"/>
+      <c r="I1" s="27"/>
+      <c r="J1" s="27"/>
+      <c r="K1" s="27"/>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
@@ -9324,19 +9327,19 @@
       <c r="E5" s="1"/>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A6" s="27" t="s">
+      <c r="A6" s="28" t="s">
         <v>112</v>
       </c>
-      <c r="B6" s="27"/>
-      <c r="C6" s="27"/>
-      <c r="D6" s="27"/>
-      <c r="E6" s="27"/>
-      <c r="F6" s="27"/>
-      <c r="G6" s="27"/>
-      <c r="H6" s="27"/>
-      <c r="I6" s="27"/>
-      <c r="J6" s="27"/>
-      <c r="K6" s="27"/>
+      <c r="B6" s="28"/>
+      <c r="C6" s="28"/>
+      <c r="D6" s="28"/>
+      <c r="E6" s="28"/>
+      <c r="F6" s="28"/>
+      <c r="G6" s="28"/>
+      <c r="H6" s="28"/>
+      <c r="I6" s="28"/>
+      <c r="J6" s="28"/>
+      <c r="K6" s="28"/>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
@@ -9464,19 +9467,19 @@
       <c r="E15" s="1"/>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A16" s="27" t="s">
-        <v>113</v>
-      </c>
-      <c r="B16" s="27"/>
-      <c r="C16" s="27"/>
-      <c r="D16" s="27"/>
-      <c r="E16" s="27"/>
-      <c r="F16" s="27"/>
-      <c r="G16" s="27"/>
-      <c r="H16" s="27"/>
-      <c r="I16" s="27"/>
-      <c r="J16" s="27"/>
-      <c r="K16" s="27"/>
+      <c r="A16" s="28" t="s">
+        <v>885</v>
+      </c>
+      <c r="B16" s="28"/>
+      <c r="C16" s="28"/>
+      <c r="D16" s="28"/>
+      <c r="E16" s="28"/>
+      <c r="F16" s="28"/>
+      <c r="G16" s="28"/>
+      <c r="H16" s="28"/>
+      <c r="I16" s="28"/>
+      <c r="J16" s="28"/>
+      <c r="K16" s="28"/>
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
@@ -9804,19 +9807,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A1" s="28" t="s">
+      <c r="A1" s="29" t="s">
         <v>111</v>
       </c>
-      <c r="B1" s="28"/>
-      <c r="C1" s="28"/>
-      <c r="D1" s="28"/>
-      <c r="E1" s="28"/>
-      <c r="F1" s="28"/>
-      <c r="G1" s="28"/>
-      <c r="H1" s="28"/>
-      <c r="I1" s="28"/>
-      <c r="J1" s="28"/>
-      <c r="K1" s="28"/>
+      <c r="B1" s="29"/>
+      <c r="C1" s="29"/>
+      <c r="D1" s="29"/>
+      <c r="E1" s="29"/>
+      <c r="F1" s="29"/>
+      <c r="G1" s="29"/>
+      <c r="H1" s="29"/>
+      <c r="I1" s="29"/>
+      <c r="J1" s="29"/>
+      <c r="K1" s="29"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
@@ -9857,19 +9860,19 @@
       <c r="E5" s="1"/>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A6" s="29" t="s">
-        <v>112</v>
-      </c>
-      <c r="B6" s="29"/>
-      <c r="C6" s="29"/>
-      <c r="D6" s="29"/>
-      <c r="E6" s="29"/>
-      <c r="F6" s="29"/>
-      <c r="G6" s="29"/>
-      <c r="H6" s="29"/>
-      <c r="I6" s="29"/>
-      <c r="J6" s="29"/>
-      <c r="K6" s="29"/>
+      <c r="A6" s="30" t="s">
+        <v>885</v>
+      </c>
+      <c r="B6" s="30"/>
+      <c r="C6" s="30"/>
+      <c r="D6" s="30"/>
+      <c r="E6" s="30"/>
+      <c r="F6" s="30"/>
+      <c r="G6" s="30"/>
+      <c r="H6" s="30"/>
+      <c r="I6" s="30"/>
+      <c r="J6" s="30"/>
+      <c r="K6" s="30"/>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
@@ -10429,19 +10432,19 @@
       </c>
     </row>
     <row r="42" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A42" s="29" t="s">
+      <c r="A42" s="30" t="s">
         <v>113</v>
       </c>
-      <c r="B42" s="29"/>
-      <c r="C42" s="29"/>
-      <c r="D42" s="29"/>
-      <c r="E42" s="29"/>
-      <c r="F42" s="29"/>
-      <c r="G42" s="29"/>
-      <c r="H42" s="29"/>
-      <c r="I42" s="29"/>
-      <c r="J42" s="29"/>
-      <c r="K42" s="29"/>
+      <c r="B42" s="30"/>
+      <c r="C42" s="30"/>
+      <c r="D42" s="30"/>
+      <c r="E42" s="30"/>
+      <c r="F42" s="30"/>
+      <c r="G42" s="30"/>
+      <c r="H42" s="30"/>
+      <c r="I42" s="30"/>
+      <c r="J42" s="30"/>
+      <c r="K42" s="30"/>
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A43" s="2" t="s">
@@ -10506,19 +10509,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A1" s="30" t="s">
+      <c r="A1" s="31" t="s">
         <v>111</v>
       </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="30"/>
-      <c r="D1" s="30"/>
-      <c r="E1" s="30"/>
-      <c r="F1" s="30"/>
-      <c r="G1" s="30"/>
-      <c r="H1" s="30"/>
-      <c r="I1" s="30"/>
-      <c r="J1" s="30"/>
-      <c r="K1" s="30"/>
+      <c r="B1" s="31"/>
+      <c r="C1" s="31"/>
+      <c r="D1" s="31"/>
+      <c r="E1" s="31"/>
+      <c r="F1" s="31"/>
+      <c r="G1" s="31"/>
+      <c r="H1" s="31"/>
+      <c r="I1" s="31"/>
+      <c r="J1" s="31"/>
+      <c r="K1" s="31"/>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
@@ -10559,19 +10562,19 @@
       <c r="E5" s="1"/>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A6" s="31" t="s">
+      <c r="A6" s="32" t="s">
         <v>112</v>
       </c>
-      <c r="B6" s="31"/>
-      <c r="C6" s="31"/>
-      <c r="D6" s="31"/>
-      <c r="E6" s="31"/>
-      <c r="F6" s="31"/>
-      <c r="G6" s="31"/>
-      <c r="H6" s="31"/>
-      <c r="I6" s="31"/>
-      <c r="J6" s="31"/>
-      <c r="K6" s="31"/>
+      <c r="B6" s="32"/>
+      <c r="C6" s="32"/>
+      <c r="D6" s="32"/>
+      <c r="E6" s="32"/>
+      <c r="F6" s="32"/>
+      <c r="G6" s="32"/>
+      <c r="H6" s="32"/>
+      <c r="I6" s="32"/>
+      <c r="J6" s="32"/>
+      <c r="K6" s="32"/>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
@@ -10612,19 +10615,19 @@
       <c r="E10" s="1"/>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A11" s="31" t="s">
-        <v>113</v>
-      </c>
-      <c r="B11" s="31"/>
-      <c r="C11" s="31"/>
-      <c r="D11" s="31"/>
-      <c r="E11" s="31"/>
-      <c r="F11" s="31"/>
-      <c r="G11" s="31"/>
-      <c r="H11" s="31"/>
-      <c r="I11" s="31"/>
-      <c r="J11" s="31"/>
-      <c r="K11" s="31"/>
+      <c r="A11" s="32" t="s">
+        <v>885</v>
+      </c>
+      <c r="B11" s="32"/>
+      <c r="C11" s="32"/>
+      <c r="D11" s="32"/>
+      <c r="E11" s="32"/>
+      <c r="F11" s="32"/>
+      <c r="G11" s="32"/>
+      <c r="H11" s="32"/>
+      <c r="I11" s="32"/>
+      <c r="J11" s="32"/>
+      <c r="K11" s="32"/>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">

</xml_diff>

<commit_message>
Update downloadable table with new ENT codes AND more info re: tonsillectomies and m65.3 prostate codes
</commit_message>
<xml_diff>
--- a/04_reports/management_report/serverless_html/resources/SRASA procedure codes and phasing.xlsx
+++ b/04_reports/management_report/serverless_html/resources/SRASA procedure codes and phasing.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rebecm14\Documents\SRASA docs\Procedure codes\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\stats\quality\srasa\(11) Scripts\Bex\snap-srasa\04_reports\management_report\serverless_html\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4DE62A4F-02DA-4116-8A1A-3934FA24C0AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06063F71-934A-417A-BD71-B137E7F2CFB0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="4" xr2:uid="{1A0DCE31-DBDB-4A7A-8FC4-F05F39A42CDB}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1878" uniqueCount="855">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1878" uniqueCount="856">
   <si>
     <t>M61 Open excision of prostate</t>
   </si>
@@ -2586,9 +2586,6 @@
     <t>F48.2 Closure of fistula of salivary gland</t>
   </si>
   <si>
-    <t>REMOVE benign tonsillectomies</t>
-  </si>
-  <si>
     <t xml:space="preserve">F34.1 (bilateral dissection tonsillectomy) does get used occasional for RAS in error but has been left off this list and will be picked up as 'unlisted' </t>
   </si>
   <si>
@@ -2608,6 +2605,12 @@
   </si>
   <si>
     <t>Unspecified kept as it is the most commonly used RAS tonsillectomy code</t>
+  </si>
+  <si>
+    <t>Prostatectomy/TURPS</t>
+  </si>
+  <si>
+    <t>REMOVE benign tonsillectomies - TBD</t>
   </si>
 </sst>
 </file>
@@ -2789,7 +2792,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
@@ -2808,6 +2811,10 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -2856,15 +2863,6 @@
     <xf numFmtId="0" fontId="1" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2960,7 +2958,7 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>83</xdr:row>
+      <xdr:row>73</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="114300" cy="114300"/>
@@ -3016,7 +3014,7 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>83</xdr:row>
+      <xdr:row>73</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="114300" cy="114300"/>
@@ -3399,19 +3397,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="18" t="s">
         <v>111</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
-      <c r="F1" s="16"/>
-      <c r="G1" s="16"/>
-      <c r="H1" s="16"/>
-      <c r="I1" s="16"/>
-      <c r="J1" s="16"/>
-      <c r="K1" s="16"/>
+      <c r="B1" s="18"/>
+      <c r="C1" s="18"/>
+      <c r="D1" s="18"/>
+      <c r="E1" s="18"/>
+      <c r="F1" s="18"/>
+      <c r="G1" s="18"/>
+      <c r="H1" s="18"/>
+      <c r="I1" s="18"/>
+      <c r="J1" s="18"/>
+      <c r="K1" s="18"/>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
@@ -3833,19 +3831,19 @@
       <c r="E30" s="1"/>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A31" s="17" t="s">
+      <c r="A31" s="19" t="s">
         <v>112</v>
       </c>
-      <c r="B31" s="17"/>
-      <c r="C31" s="17"/>
-      <c r="D31" s="17"/>
-      <c r="E31" s="17"/>
-      <c r="F31" s="17"/>
-      <c r="G31" s="17"/>
-      <c r="H31" s="17"/>
-      <c r="I31" s="17"/>
-      <c r="J31" s="17"/>
-      <c r="K31" s="17"/>
+      <c r="B31" s="19"/>
+      <c r="C31" s="19"/>
+      <c r="D31" s="19"/>
+      <c r="E31" s="19"/>
+      <c r="F31" s="19"/>
+      <c r="G31" s="19"/>
+      <c r="H31" s="19"/>
+      <c r="I31" s="19"/>
+      <c r="J31" s="19"/>
+      <c r="K31" s="19"/>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A32" s="2" t="s">
@@ -4095,19 +4093,19 @@
       <c r="E48" s="1"/>
     </row>
     <row r="49" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A49" s="17" t="s">
+      <c r="A49" s="19" t="s">
         <v>776</v>
       </c>
-      <c r="B49" s="17"/>
-      <c r="C49" s="17"/>
-      <c r="D49" s="17"/>
-      <c r="E49" s="17"/>
-      <c r="F49" s="17"/>
-      <c r="G49" s="17"/>
-      <c r="H49" s="17"/>
-      <c r="I49" s="17"/>
-      <c r="J49" s="17"/>
-      <c r="K49" s="17"/>
+      <c r="B49" s="19"/>
+      <c r="C49" s="19"/>
+      <c r="D49" s="19"/>
+      <c r="E49" s="19"/>
+      <c r="F49" s="19"/>
+      <c r="G49" s="19"/>
+      <c r="H49" s="19"/>
+      <c r="I49" s="19"/>
+      <c r="J49" s="19"/>
+      <c r="K49" s="19"/>
     </row>
     <row r="50" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A50" s="2" t="s">
@@ -4667,19 +4665,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="20" t="s">
         <v>111</v>
       </c>
-      <c r="B1" s="18"/>
-      <c r="C1" s="18"/>
-      <c r="D1" s="18"/>
-      <c r="E1" s="18"/>
-      <c r="F1" s="18"/>
-      <c r="G1" s="18"/>
-      <c r="H1" s="18"/>
-      <c r="I1" s="18"/>
-      <c r="J1" s="18"/>
-      <c r="K1" s="18"/>
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="20"/>
+      <c r="E1" s="20"/>
+      <c r="F1" s="20"/>
+      <c r="G1" s="20"/>
+      <c r="H1" s="20"/>
+      <c r="I1" s="20"/>
+      <c r="J1" s="20"/>
+      <c r="K1" s="20"/>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
@@ -5142,10 +5140,10 @@
         <v>771</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>200</v>
+        <v>854</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="E31" s="1" t="s">
         <v>772</v>
@@ -5159,19 +5157,19 @@
       <c r="E32" s="1"/>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A33" s="19" t="s">
+      <c r="A33" s="21" t="s">
         <v>112</v>
       </c>
-      <c r="B33" s="19"/>
-      <c r="C33" s="19"/>
-      <c r="D33" s="19"/>
-      <c r="E33" s="19"/>
-      <c r="F33" s="19"/>
-      <c r="G33" s="19"/>
-      <c r="H33" s="19"/>
-      <c r="I33" s="19"/>
-      <c r="J33" s="19"/>
-      <c r="K33" s="19"/>
+      <c r="B33" s="21"/>
+      <c r="C33" s="21"/>
+      <c r="D33" s="21"/>
+      <c r="E33" s="21"/>
+      <c r="F33" s="21"/>
+      <c r="G33" s="21"/>
+      <c r="H33" s="21"/>
+      <c r="I33" s="21"/>
+      <c r="J33" s="21"/>
+      <c r="K33" s="21"/>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A34" s="2" t="s">
@@ -5212,19 +5210,19 @@
       <c r="E37" s="1"/>
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A38" s="19" t="s">
+      <c r="A38" s="21" t="s">
         <v>776</v>
       </c>
-      <c r="B38" s="19"/>
-      <c r="C38" s="19"/>
-      <c r="D38" s="19"/>
-      <c r="E38" s="19"/>
-      <c r="F38" s="19"/>
-      <c r="G38" s="19"/>
-      <c r="H38" s="19"/>
-      <c r="I38" s="19"/>
-      <c r="J38" s="19"/>
-      <c r="K38" s="19"/>
+      <c r="B38" s="21"/>
+      <c r="C38" s="21"/>
+      <c r="D38" s="21"/>
+      <c r="E38" s="21"/>
+      <c r="F38" s="21"/>
+      <c r="G38" s="21"/>
+      <c r="H38" s="21"/>
+      <c r="I38" s="21"/>
+      <c r="J38" s="21"/>
+      <c r="K38" s="21"/>
     </row>
     <row r="39" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A39" s="2" t="s">
@@ -5287,19 +5285,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="22" t="s">
         <v>111</v>
       </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20"/>
-      <c r="D1" s="20"/>
-      <c r="E1" s="20"/>
-      <c r="F1" s="20"/>
-      <c r="G1" s="20"/>
-      <c r="H1" s="20"/>
-      <c r="I1" s="20"/>
-      <c r="J1" s="20"/>
-      <c r="K1" s="20"/>
+      <c r="B1" s="22"/>
+      <c r="C1" s="22"/>
+      <c r="D1" s="22"/>
+      <c r="E1" s="22"/>
+      <c r="F1" s="22"/>
+      <c r="G1" s="22"/>
+      <c r="H1" s="22"/>
+      <c r="I1" s="22"/>
+      <c r="J1" s="22"/>
+      <c r="K1" s="22"/>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
@@ -5542,19 +5540,19 @@
       <c r="E19" s="1"/>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A20" s="21" t="s">
+      <c r="A20" s="23" t="s">
         <v>112</v>
       </c>
-      <c r="B20" s="21"/>
-      <c r="C20" s="21"/>
-      <c r="D20" s="21"/>
-      <c r="E20" s="21"/>
-      <c r="F20" s="21"/>
-      <c r="G20" s="21"/>
-      <c r="H20" s="21"/>
-      <c r="I20" s="21"/>
-      <c r="J20" s="21"/>
-      <c r="K20" s="21"/>
+      <c r="B20" s="23"/>
+      <c r="C20" s="23"/>
+      <c r="D20" s="23"/>
+      <c r="E20" s="23"/>
+      <c r="F20" s="23"/>
+      <c r="G20" s="23"/>
+      <c r="H20" s="23"/>
+      <c r="I20" s="23"/>
+      <c r="J20" s="23"/>
+      <c r="K20" s="23"/>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
@@ -5595,19 +5593,19 @@
       <c r="E24" s="1"/>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A25" s="21" t="s">
+      <c r="A25" s="23" t="s">
         <v>776</v>
       </c>
-      <c r="B25" s="21"/>
-      <c r="C25" s="21"/>
-      <c r="D25" s="21"/>
-      <c r="E25" s="21"/>
-      <c r="F25" s="21"/>
-      <c r="G25" s="21"/>
-      <c r="H25" s="21"/>
-      <c r="I25" s="21"/>
-      <c r="J25" s="21"/>
-      <c r="K25" s="21"/>
+      <c r="B25" s="23"/>
+      <c r="C25" s="23"/>
+      <c r="D25" s="23"/>
+      <c r="E25" s="23"/>
+      <c r="F25" s="23"/>
+      <c r="G25" s="23"/>
+      <c r="H25" s="23"/>
+      <c r="I25" s="23"/>
+      <c r="J25" s="23"/>
+      <c r="K25" s="23"/>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
@@ -5737,19 +5735,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A1" s="22" t="s">
+      <c r="A1" s="24" t="s">
         <v>111</v>
       </c>
-      <c r="B1" s="22"/>
-      <c r="C1" s="22"/>
-      <c r="D1" s="22"/>
-      <c r="E1" s="22"/>
-      <c r="F1" s="22"/>
-      <c r="G1" s="22"/>
-      <c r="H1" s="22"/>
-      <c r="I1" s="22"/>
-      <c r="J1" s="22"/>
-      <c r="K1" s="22"/>
+      <c r="B1" s="24"/>
+      <c r="C1" s="24"/>
+      <c r="D1" s="24"/>
+      <c r="E1" s="24"/>
+      <c r="F1" s="24"/>
+      <c r="G1" s="24"/>
+      <c r="H1" s="24"/>
+      <c r="I1" s="24"/>
+      <c r="J1" s="24"/>
+      <c r="K1" s="24"/>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
@@ -5965,19 +5963,19 @@
       <c r="E15" s="1"/>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A16" s="23" t="s">
+      <c r="A16" s="25" t="s">
         <v>112</v>
       </c>
-      <c r="B16" s="23"/>
-      <c r="C16" s="23"/>
-      <c r="D16" s="23"/>
-      <c r="E16" s="23"/>
-      <c r="F16" s="23"/>
-      <c r="G16" s="23"/>
-      <c r="H16" s="23"/>
-      <c r="I16" s="23"/>
-      <c r="J16" s="23"/>
-      <c r="K16" s="23"/>
+      <c r="B16" s="25"/>
+      <c r="C16" s="25"/>
+      <c r="D16" s="25"/>
+      <c r="E16" s="25"/>
+      <c r="F16" s="25"/>
+      <c r="G16" s="25"/>
+      <c r="H16" s="25"/>
+      <c r="I16" s="25"/>
+      <c r="J16" s="25"/>
+      <c r="K16" s="25"/>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
@@ -6229,19 +6227,19 @@
       <c r="E32" s="1"/>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A33" s="23" t="s">
+      <c r="A33" s="25" t="s">
         <v>776</v>
       </c>
-      <c r="B33" s="23"/>
-      <c r="C33" s="23"/>
-      <c r="D33" s="23"/>
-      <c r="E33" s="23"/>
-      <c r="F33" s="23"/>
-      <c r="G33" s="23"/>
-      <c r="H33" s="23"/>
-      <c r="I33" s="23"/>
-      <c r="J33" s="23"/>
-      <c r="K33" s="23"/>
+      <c r="B33" s="25"/>
+      <c r="C33" s="25"/>
+      <c r="D33" s="25"/>
+      <c r="E33" s="25"/>
+      <c r="F33" s="25"/>
+      <c r="G33" s="25"/>
+      <c r="H33" s="25"/>
+      <c r="I33" s="25"/>
+      <c r="J33" s="25"/>
+      <c r="K33" s="25"/>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A34" s="2" t="s">
@@ -6770,7 +6768,7 @@
         <v>762</v>
       </c>
       <c r="D67" t="s">
-        <v>850</v>
+        <v>849</v>
       </c>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.3">
@@ -6778,7 +6776,7 @@
         <v>763</v>
       </c>
       <c r="D68" t="s">
-        <v>851</v>
+        <v>850</v>
       </c>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.3">
@@ -6786,7 +6784,7 @@
         <v>764</v>
       </c>
       <c r="D69" t="s">
-        <v>850</v>
+        <v>849</v>
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.3">
@@ -6794,7 +6792,7 @@
         <v>765</v>
       </c>
       <c r="D70" t="s">
-        <v>850</v>
+        <v>849</v>
       </c>
     </row>
   </sheetData>
@@ -6810,7 +6808,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{40C4708D-51A9-4027-A13F-C06B96593285}">
-  <dimension ref="A1:K154"/>
+  <dimension ref="A1:K132"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.33203125" bestFit="1" customWidth="1"/>
@@ -6820,19 +6818,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A1" s="24" t="s">
+      <c r="A1" s="26" t="s">
         <v>111</v>
       </c>
-      <c r="B1" s="24"/>
-      <c r="C1" s="24"/>
-      <c r="D1" s="24"/>
-      <c r="E1" s="24"/>
-      <c r="F1" s="24"/>
-      <c r="G1" s="24"/>
-      <c r="H1" s="24"/>
-      <c r="I1" s="24"/>
-      <c r="J1" s="24"/>
-      <c r="K1" s="24"/>
+      <c r="B1" s="26"/>
+      <c r="C1" s="26"/>
+      <c r="D1" s="26"/>
+      <c r="E1" s="26"/>
+      <c r="F1" s="26"/>
+      <c r="G1" s="26"/>
+      <c r="H1" s="26"/>
+      <c r="I1" s="26"/>
+      <c r="J1" s="26"/>
+      <c r="K1" s="26"/>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
@@ -6852,2211 +6850,2035 @@
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A3" s="34" t="s">
+      <c r="A3" s="1" t="s">
         <v>778</v>
       </c>
-      <c r="B3" s="34" t="s">
+      <c r="B3" s="1" t="s">
         <v>779</v>
       </c>
-      <c r="C3" s="34" t="s">
+      <c r="C3" s="1" t="s">
         <v>780</v>
       </c>
-      <c r="D3" s="34"/>
-      <c r="E3" s="34" t="s">
+      <c r="D3" s="1"/>
+      <c r="E3" s="1" t="s">
         <v>399</v>
       </c>
-      <c r="F3" s="38" t="s">
+      <c r="F3" s="17" t="s">
         <v>415</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A4" s="34" t="s">
+      <c r="A4" s="1" t="s">
         <v>393</v>
       </c>
-      <c r="B4" s="35" t="s">
+      <c r="B4" s="16" t="s">
         <v>396</v>
       </c>
-      <c r="C4" s="34" t="s">
+      <c r="C4" s="1" t="s">
         <v>780</v>
       </c>
-      <c r="D4" s="34"/>
-      <c r="E4" s="34" t="s">
+      <c r="D4" s="1"/>
+      <c r="E4" s="1" t="s">
         <v>399</v>
       </c>
-      <c r="F4" s="36"/>
+      <c r="F4" s="7"/>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A5" s="34" t="s">
+      <c r="A5" s="1" t="s">
         <v>394</v>
       </c>
-      <c r="B5" s="35" t="s">
+      <c r="B5" s="16" t="s">
         <v>397</v>
       </c>
-      <c r="C5" s="34" t="s">
+      <c r="C5" s="1" t="s">
         <v>780</v>
       </c>
-      <c r="D5" s="34"/>
-      <c r="E5" s="34" t="s">
+      <c r="D5" s="1"/>
+      <c r="E5" s="1" t="s">
         <v>399</v>
       </c>
-      <c r="F5" s="36"/>
+      <c r="F5" s="7"/>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A6" s="34" t="s">
+      <c r="A6" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="B6" s="35" t="s">
+      <c r="B6" s="16" t="s">
         <v>398</v>
       </c>
-      <c r="C6" s="34" t="s">
+      <c r="C6" s="1" t="s">
         <v>780</v>
       </c>
-      <c r="D6" s="34" t="s">
+      <c r="D6" s="1" t="s">
+        <v>851</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>399</v>
+      </c>
+      <c r="F6" s="7"/>
+    </row>
+    <row r="7" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A7" s="1" t="s">
+        <v>406</v>
+      </c>
+      <c r="B7" s="16" t="s">
+        <v>400</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>412</v>
+      </c>
+      <c r="D7" s="1"/>
+      <c r="E7" s="1" t="s">
+        <v>413</v>
+      </c>
+      <c r="F7" s="7"/>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A8" s="1" t="s">
+        <v>407</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>401</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>412</v>
+      </c>
+      <c r="D8" s="1"/>
+      <c r="E8" s="1" t="s">
+        <v>413</v>
+      </c>
+      <c r="F8" s="7"/>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A9" s="1" t="s">
+        <v>408</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>402</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>412</v>
+      </c>
+      <c r="D9" s="1"/>
+      <c r="E9" s="1" t="s">
+        <v>414</v>
+      </c>
+      <c r="F9" s="7"/>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A10" s="1" t="s">
+        <v>409</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>403</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>412</v>
+      </c>
+      <c r="D10" s="1"/>
+      <c r="E10" s="1" t="s">
+        <v>414</v>
+      </c>
+      <c r="F10" s="7"/>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A11" s="1" t="s">
+        <v>410</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>404</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>412</v>
+      </c>
+      <c r="D11" s="1"/>
+      <c r="E11" s="1" t="s">
+        <v>414</v>
+      </c>
+      <c r="F11" s="7"/>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A12" s="1" t="s">
+        <v>411</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>405</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>412</v>
+      </c>
+      <c r="D12" s="1"/>
+      <c r="E12" s="1" t="s">
+        <v>414</v>
+      </c>
+      <c r="F12" s="7"/>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A13" s="1" t="s">
+        <v>781</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>782</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>412</v>
+      </c>
+      <c r="D13" s="1"/>
+      <c r="E13" s="1" t="s">
+        <v>420</v>
+      </c>
+      <c r="F13" s="7"/>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A14" s="1" t="s">
+        <v>418</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>416</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>412</v>
+      </c>
+      <c r="D14" s="1"/>
+      <c r="E14" s="1" t="s">
+        <v>420</v>
+      </c>
+      <c r="F14" s="7"/>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A15" s="1" t="s">
+        <v>419</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>417</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>412</v>
+      </c>
+      <c r="D15" s="1"/>
+      <c r="E15" s="1" t="s">
+        <v>420</v>
+      </c>
+      <c r="F15" s="7"/>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A16" s="1" t="s">
+        <v>783</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>784</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>785</v>
+      </c>
+      <c r="D16" s="1"/>
+      <c r="E16" s="1" t="s">
+        <v>786</v>
+      </c>
+      <c r="F16" s="7"/>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A17" s="1" t="s">
+        <v>787</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>788</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>785</v>
+      </c>
+      <c r="D17" s="1"/>
+      <c r="E17" s="1" t="s">
+        <v>786</v>
+      </c>
+      <c r="F17" s="7"/>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A18" s="1" t="s">
+        <v>789</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>790</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>785</v>
+      </c>
+      <c r="D18" s="1"/>
+      <c r="E18" s="1" t="s">
+        <v>786</v>
+      </c>
+      <c r="F18" s="7"/>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A19" s="1" t="s">
+        <v>791</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>792</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>785</v>
+      </c>
+      <c r="D19" s="1"/>
+      <c r="E19" s="1" t="s">
+        <v>786</v>
+      </c>
+      <c r="F19" s="7"/>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A20" s="1" t="s">
+        <v>793</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>794</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>785</v>
+      </c>
+      <c r="D20" s="1"/>
+      <c r="E20" s="1" t="s">
+        <v>786</v>
+      </c>
+      <c r="F20" s="7"/>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A21" s="1" t="s">
+        <v>795</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>796</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>797</v>
+      </c>
+      <c r="D21" s="1"/>
+      <c r="E21" s="1" t="s">
+        <v>786</v>
+      </c>
+      <c r="F21" s="7"/>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A22" s="1" t="s">
+        <v>798</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>799</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>797</v>
+      </c>
+      <c r="D22" s="1"/>
+      <c r="E22" s="1" t="s">
+        <v>800</v>
+      </c>
+      <c r="F22" s="7"/>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A23" s="1" t="s">
+        <v>801</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>802</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>797</v>
+      </c>
+      <c r="D23" s="1"/>
+      <c r="E23" s="1" t="s">
+        <v>800</v>
+      </c>
+      <c r="F23" s="7"/>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A24" s="1" t="s">
+        <v>803</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>804</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>797</v>
+      </c>
+      <c r="D24" s="1"/>
+      <c r="E24" s="1" t="s">
+        <v>800</v>
+      </c>
+      <c r="F24" s="7"/>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A25" s="1" t="s">
+        <v>805</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>806</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>797</v>
+      </c>
+      <c r="D25" s="1"/>
+      <c r="E25" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="F25" s="7"/>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A26" s="1" t="s">
+        <v>808</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>809</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>797</v>
+      </c>
+      <c r="D26" s="1"/>
+      <c r="E26" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="F26" s="7"/>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A27" s="1" t="s">
+        <v>810</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>811</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>797</v>
+      </c>
+      <c r="D27" s="1"/>
+      <c r="E27" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="F27" s="7"/>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A28" s="1" t="s">
+        <v>812</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>813</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>797</v>
+      </c>
+      <c r="D28" s="1"/>
+      <c r="E28" s="1" t="s">
+        <v>814</v>
+      </c>
+      <c r="F28" s="7"/>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A29" s="1" t="s">
+        <v>815</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>816</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>797</v>
+      </c>
+      <c r="D29" s="1"/>
+      <c r="E29" s="1" t="s">
+        <v>814</v>
+      </c>
+      <c r="F29" s="7"/>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A30" s="1" t="s">
+        <v>817</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>818</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>797</v>
+      </c>
+      <c r="D30" s="1"/>
+      <c r="E30" s="1" t="s">
+        <v>814</v>
+      </c>
+      <c r="F30" s="7"/>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A31" s="1" t="s">
+        <v>819</v>
+      </c>
+      <c r="B31" t="s">
+        <v>820</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>797</v>
+      </c>
+      <c r="D31" s="1"/>
+      <c r="E31" s="1" t="s">
+        <v>814</v>
+      </c>
+      <c r="F31" s="7"/>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A32" s="1" t="s">
+        <v>821</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>822</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>823</v>
+      </c>
+      <c r="D32" s="1"/>
+      <c r="E32" s="1" t="s">
+        <v>824</v>
+      </c>
+      <c r="F32" s="7"/>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A33" s="1" t="s">
+        <v>825</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>826</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>823</v>
+      </c>
+      <c r="D33" s="1"/>
+      <c r="E33" s="1" t="s">
+        <v>824</v>
+      </c>
+      <c r="F33" s="7"/>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A34" s="1" t="s">
+        <v>421</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>424</v>
+      </c>
+      <c r="C34" s="1" t="s">
+        <v>427</v>
+      </c>
+      <c r="D34" s="1"/>
+      <c r="E34" s="1" t="s">
+        <v>430</v>
+      </c>
+      <c r="F34" s="7"/>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A35" s="1" t="s">
+        <v>422</v>
+      </c>
+      <c r="B35" t="s">
+        <v>425</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>427</v>
+      </c>
+      <c r="D35" s="1"/>
+      <c r="E35" s="1" t="s">
+        <v>430</v>
+      </c>
+      <c r="F35" s="7"/>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A36" s="1" t="s">
+        <v>423</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>426</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>427</v>
+      </c>
+      <c r="D36" s="1"/>
+      <c r="E36" s="1" t="s">
+        <v>430</v>
+      </c>
+      <c r="F36" s="7"/>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A37" s="1" t="s">
+        <v>428</v>
+      </c>
+      <c r="B37" s="1" t="s">
+        <v>429</v>
+      </c>
+      <c r="C37" s="1" t="s">
+        <v>432</v>
+      </c>
+      <c r="D37" s="1"/>
+      <c r="E37" s="1" t="s">
+        <v>431</v>
+      </c>
+      <c r="F37" s="7"/>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A38" s="1" t="s">
+        <v>433</v>
+      </c>
+      <c r="B38" s="1" t="s">
+        <v>434</v>
+      </c>
+      <c r="C38" s="1" t="s">
+        <v>432</v>
+      </c>
+      <c r="D38" s="1"/>
+      <c r="E38" s="1" t="s">
+        <v>435</v>
+      </c>
+      <c r="F38" s="7"/>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A39" s="1" t="s">
+        <v>827</v>
+      </c>
+      <c r="B39" t="s">
+        <v>828</v>
+      </c>
+      <c r="C39" s="1" t="s">
+        <v>432</v>
+      </c>
+      <c r="D39" s="1"/>
+      <c r="E39" s="1" t="s">
+        <v>435</v>
+      </c>
+      <c r="F39" s="7"/>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A40" s="1" t="s">
+        <v>438</v>
+      </c>
+      <c r="B40" s="1" t="s">
+        <v>436</v>
+      </c>
+      <c r="C40" s="1" t="s">
+        <v>437</v>
+      </c>
+      <c r="D40" s="1"/>
+      <c r="E40" s="1" t="s">
+        <v>439</v>
+      </c>
+      <c r="F40" s="7"/>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A41" s="1" t="s">
+        <v>829</v>
+      </c>
+      <c r="B41" s="1" t="s">
+        <v>830</v>
+      </c>
+      <c r="C41" s="1" t="s">
+        <v>437</v>
+      </c>
+      <c r="D41" s="1"/>
+      <c r="E41" s="1" t="s">
+        <v>831</v>
+      </c>
+      <c r="F41" s="7"/>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A42" s="1" t="s">
+        <v>832</v>
+      </c>
+      <c r="B42" s="1" t="s">
+        <v>833</v>
+      </c>
+      <c r="C42" s="1" t="s">
+        <v>437</v>
+      </c>
+      <c r="D42" s="1"/>
+      <c r="E42" s="1" t="s">
+        <v>831</v>
+      </c>
+      <c r="F42" s="7"/>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A43" s="1" t="s">
+        <v>443</v>
+      </c>
+      <c r="B43" s="1" t="s">
+        <v>440</v>
+      </c>
+      <c r="C43" s="1" t="s">
+        <v>437</v>
+      </c>
+      <c r="D43" s="1"/>
+      <c r="E43" s="1" t="s">
+        <v>445</v>
+      </c>
+      <c r="F43" s="7"/>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A44" s="1" t="s">
+        <v>834</v>
+      </c>
+      <c r="B44" s="1" t="s">
+        <v>835</v>
+      </c>
+      <c r="C44" s="1" t="s">
+        <v>437</v>
+      </c>
+      <c r="D44" s="1"/>
+      <c r="E44" s="1" t="s">
+        <v>445</v>
+      </c>
+      <c r="F44" s="7"/>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A45" s="1" t="s">
+        <v>444</v>
+      </c>
+      <c r="B45" s="1" t="s">
+        <v>442</v>
+      </c>
+      <c r="C45" s="1" t="s">
+        <v>437</v>
+      </c>
+      <c r="D45" s="1"/>
+      <c r="E45" s="1" t="s">
+        <v>445</v>
+      </c>
+      <c r="F45" s="7"/>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A46" s="1" t="s">
+        <v>473</v>
+      </c>
+      <c r="B46" s="1" t="s">
+        <v>441</v>
+      </c>
+      <c r="C46" s="1" t="s">
+        <v>437</v>
+      </c>
+      <c r="D46" s="1"/>
+      <c r="E46" s="1" t="s">
+        <v>445</v>
+      </c>
+      <c r="F46" s="7"/>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A47" s="1" t="s">
+        <v>454</v>
+      </c>
+      <c r="B47" s="1" t="s">
+        <v>446</v>
+      </c>
+      <c r="C47" s="1" t="s">
+        <v>452</v>
+      </c>
+      <c r="D47" s="1" t="s">
+        <v>847</v>
+      </c>
+      <c r="E47" s="1" t="s">
+        <v>453</v>
+      </c>
+      <c r="F47" s="7"/>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A48" s="1" t="s">
+        <v>455</v>
+      </c>
+      <c r="B48" s="1" t="s">
+        <v>447</v>
+      </c>
+      <c r="C48" s="1" t="s">
+        <v>452</v>
+      </c>
+      <c r="D48" s="1"/>
+      <c r="E48" s="1" t="s">
+        <v>453</v>
+      </c>
+      <c r="F48" s="7"/>
+    </row>
+    <row r="49" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A49" s="1" t="s">
+        <v>456</v>
+      </c>
+      <c r="B49" s="1" t="s">
+        <v>448</v>
+      </c>
+      <c r="C49" s="1" t="s">
+        <v>452</v>
+      </c>
+      <c r="D49" s="1"/>
+      <c r="E49" s="1" t="s">
+        <v>453</v>
+      </c>
+      <c r="F49" s="7"/>
+    </row>
+    <row r="50" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A50" s="1" t="s">
+        <v>457</v>
+      </c>
+      <c r="B50" s="1" t="s">
+        <v>449</v>
+      </c>
+      <c r="C50" s="1" t="s">
+        <v>452</v>
+      </c>
+      <c r="D50" s="1"/>
+      <c r="E50" s="1" t="s">
+        <v>453</v>
+      </c>
+      <c r="F50" s="7"/>
+    </row>
+    <row r="51" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A51" s="1" t="s">
+        <v>458</v>
+      </c>
+      <c r="B51" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="C51" s="1" t="s">
+        <v>452</v>
+      </c>
+      <c r="D51" s="1" t="s">
         <v>852</v>
       </c>
-      <c r="E6" s="34" t="s">
+      <c r="E51" s="1" t="s">
+        <v>453</v>
+      </c>
+      <c r="F51" s="7"/>
+    </row>
+    <row r="52" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A52" s="1" t="s">
+        <v>459</v>
+      </c>
+      <c r="B52" s="1" t="s">
+        <v>451</v>
+      </c>
+      <c r="C52" s="1" t="s">
+        <v>452</v>
+      </c>
+      <c r="D52" s="1" t="s">
+        <v>853</v>
+      </c>
+      <c r="E52" s="1" t="s">
+        <v>453</v>
+      </c>
+      <c r="F52" s="7"/>
+    </row>
+    <row r="53" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A53" s="1" t="s">
+        <v>463</v>
+      </c>
+      <c r="B53" s="1" t="s">
+        <v>460</v>
+      </c>
+      <c r="C53" s="1" t="s">
+        <v>462</v>
+      </c>
+      <c r="D53" s="1"/>
+      <c r="E53" s="1" t="s">
+        <v>465</v>
+      </c>
+      <c r="F53" s="7"/>
+    </row>
+    <row r="54" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A54" s="1" t="s">
+        <v>464</v>
+      </c>
+      <c r="B54" t="s">
+        <v>461</v>
+      </c>
+      <c r="C54" s="1" t="s">
+        <v>462</v>
+      </c>
+      <c r="D54" s="1"/>
+      <c r="E54" s="1" t="s">
+        <v>465</v>
+      </c>
+      <c r="F54" s="7"/>
+    </row>
+    <row r="55" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A55" s="1" t="s">
+        <v>469</v>
+      </c>
+      <c r="B55" s="1" t="s">
+        <v>466</v>
+      </c>
+      <c r="C55" s="1" t="s">
+        <v>468</v>
+      </c>
+      <c r="D55" s="1"/>
+      <c r="E55" s="1" t="s">
+        <v>471</v>
+      </c>
+      <c r="F55" s="7"/>
+    </row>
+    <row r="56" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A56" s="1" t="s">
+        <v>470</v>
+      </c>
+      <c r="B56" s="1" t="s">
+        <v>467</v>
+      </c>
+      <c r="C56" s="1" t="s">
+        <v>468</v>
+      </c>
+      <c r="D56" s="1"/>
+      <c r="E56" s="1" t="s">
+        <v>471</v>
+      </c>
+      <c r="F56" s="7"/>
+    </row>
+    <row r="57" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A57" s="1" t="s">
+        <v>836</v>
+      </c>
+      <c r="B57" s="1" t="s">
+        <v>837</v>
+      </c>
+      <c r="C57" s="1" t="s">
+        <v>838</v>
+      </c>
+      <c r="D57" s="1"/>
+      <c r="E57" s="1" t="s">
+        <v>839</v>
+      </c>
+      <c r="F57" s="7"/>
+    </row>
+    <row r="58" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A58" s="1" t="s">
+        <v>840</v>
+      </c>
+      <c r="B58" s="1" t="s">
+        <v>841</v>
+      </c>
+      <c r="C58" s="1" t="s">
+        <v>838</v>
+      </c>
+      <c r="D58" s="1"/>
+      <c r="E58" s="1" t="s">
+        <v>839</v>
+      </c>
+      <c r="F58" s="7"/>
+    </row>
+    <row r="59" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A59" s="1" t="s">
+        <v>842</v>
+      </c>
+      <c r="B59" s="1" t="s">
+        <v>843</v>
+      </c>
+      <c r="C59" s="1" t="s">
+        <v>838</v>
+      </c>
+      <c r="D59" s="1"/>
+      <c r="E59" s="1" t="s">
+        <v>844</v>
+      </c>
+      <c r="F59" s="7"/>
+    </row>
+    <row r="60" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A60" s="1" t="s">
+        <v>845</v>
+      </c>
+      <c r="B60" s="1" t="s">
+        <v>846</v>
+      </c>
+      <c r="C60" s="1" t="s">
+        <v>838</v>
+      </c>
+      <c r="D60" s="1"/>
+      <c r="E60" s="1" t="s">
+        <v>844</v>
+      </c>
+      <c r="F60" s="7"/>
+    </row>
+    <row r="61" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A61" s="1"/>
+      <c r="B61" s="1"/>
+      <c r="C61" s="1"/>
+      <c r="D61" s="1"/>
+      <c r="E61" s="1"/>
+      <c r="F61" s="7"/>
+    </row>
+    <row r="62" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A62" s="27" t="s">
+        <v>112</v>
+      </c>
+      <c r="B62" s="27"/>
+      <c r="C62" s="27"/>
+      <c r="D62" s="27"/>
+      <c r="E62" s="27"/>
+      <c r="F62" s="27"/>
+      <c r="G62" s="27"/>
+      <c r="H62" s="27"/>
+      <c r="I62" s="27"/>
+      <c r="J62" s="27"/>
+      <c r="K62" s="27"/>
+    </row>
+    <row r="63" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A63" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="B63" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="C63" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="D63" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="E63" s="2" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="64" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A64" s="1" t="s">
+        <v>778</v>
+      </c>
+      <c r="B64" s="1" t="s">
+        <v>779</v>
+      </c>
+      <c r="C64" s="1" t="s">
+        <v>780</v>
+      </c>
+      <c r="D64" s="1"/>
+      <c r="E64" s="1" t="s">
         <v>399</v>
       </c>
-      <c r="F6" s="36"/>
-    </row>
-    <row r="7" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A7" s="34" t="s">
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A65" s="1" t="s">
+        <v>393</v>
+      </c>
+      <c r="B65" s="16" t="s">
+        <v>396</v>
+      </c>
+      <c r="C65" s="1" t="s">
+        <v>780</v>
+      </c>
+      <c r="D65" s="1"/>
+      <c r="E65" s="1" t="s">
+        <v>399</v>
+      </c>
+      <c r="F65" s="8" t="s">
+        <v>472</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A66" s="1" t="s">
+        <v>394</v>
+      </c>
+      <c r="B66" s="16" t="s">
+        <v>397</v>
+      </c>
+      <c r="C66" s="1" t="s">
+        <v>780</v>
+      </c>
+      <c r="D66" s="1"/>
+      <c r="E66" s="1" t="s">
+        <v>399</v>
+      </c>
+      <c r="F66" s="8" t="s">
+        <v>773</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A67" s="1" t="s">
+        <v>395</v>
+      </c>
+      <c r="B67" s="16" t="s">
+        <v>398</v>
+      </c>
+      <c r="C67" s="1" t="s">
+        <v>780</v>
+      </c>
+      <c r="D67" s="1"/>
+      <c r="E67" s="1" t="s">
+        <v>399</v>
+      </c>
+      <c r="F67" s="8"/>
+    </row>
+    <row r="68" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A68" s="1" t="s">
         <v>406</v>
       </c>
-      <c r="B7" s="35" t="s">
+      <c r="B68" s="16" t="s">
         <v>400</v>
       </c>
-      <c r="C7" s="34" t="s">
+      <c r="C68" s="1" t="s">
         <v>412</v>
       </c>
-      <c r="D7" s="34"/>
-      <c r="E7" s="34" t="s">
+      <c r="D68" s="1"/>
+      <c r="E68" s="1" t="s">
         <v>413</v>
       </c>
-      <c r="F7" s="36"/>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A8" s="34" t="s">
+      <c r="F68" s="8"/>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A69" s="1" t="s">
         <v>407</v>
       </c>
-      <c r="B8" s="34" t="s">
+      <c r="B69" s="1" t="s">
         <v>401</v>
       </c>
-      <c r="C8" s="34" t="s">
+      <c r="C69" s="1" t="s">
         <v>412</v>
       </c>
-      <c r="D8" s="34"/>
-      <c r="E8" s="34" t="s">
+      <c r="D69" s="1"/>
+      <c r="E69" s="1" t="s">
         <v>413</v>
       </c>
-      <c r="F8" s="36"/>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A9" s="34" t="s">
+      <c r="F69" s="8"/>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A70" s="1" t="s">
         <v>408</v>
       </c>
-      <c r="B9" s="34" t="s">
+      <c r="B70" s="1" t="s">
         <v>402</v>
       </c>
-      <c r="C9" s="34" t="s">
+      <c r="C70" s="1" t="s">
         <v>412</v>
       </c>
-      <c r="D9" s="34"/>
-      <c r="E9" s="34" t="s">
+      <c r="D70" s="1"/>
+      <c r="E70" s="1" t="s">
         <v>414</v>
       </c>
-      <c r="F9" s="36"/>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A10" s="34" t="s">
+      <c r="F70" s="8"/>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A71" s="1" t="s">
         <v>409</v>
       </c>
-      <c r="B10" s="34" t="s">
+      <c r="B71" s="1" t="s">
         <v>403</v>
       </c>
-      <c r="C10" s="34" t="s">
+      <c r="C71" s="1" t="s">
         <v>412</v>
       </c>
-      <c r="D10" s="34"/>
-      <c r="E10" s="34" t="s">
+      <c r="D71" s="1"/>
+      <c r="E71" s="1" t="s">
         <v>414</v>
       </c>
-      <c r="F10" s="36"/>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A11" s="34" t="s">
+      <c r="F71" s="8"/>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A72" s="1" t="s">
         <v>410</v>
       </c>
-      <c r="B11" s="34" t="s">
+      <c r="B72" s="1" t="s">
         <v>404</v>
       </c>
-      <c r="C11" s="34" t="s">
+      <c r="C72" s="1" t="s">
         <v>412</v>
       </c>
-      <c r="D11" s="34"/>
-      <c r="E11" s="34" t="s">
+      <c r="D72" s="1"/>
+      <c r="E72" s="1" t="s">
         <v>414</v>
       </c>
-      <c r="F11" s="36"/>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A12" s="34" t="s">
+      <c r="F72" s="8"/>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A73" s="1" t="s">
         <v>411</v>
       </c>
-      <c r="B12" s="34" t="s">
+      <c r="B73" s="1" t="s">
         <v>405</v>
       </c>
-      <c r="C12" s="34" t="s">
+      <c r="C73" s="1" t="s">
         <v>412</v>
       </c>
-      <c r="D12" s="34"/>
-      <c r="E12" s="34" t="s">
+      <c r="D73" s="1"/>
+      <c r="E73" s="1" t="s">
         <v>414</v>
       </c>
-      <c r="F12" s="36"/>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A13" s="34" t="s">
+      <c r="F73" s="8"/>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A74" s="1" t="s">
         <v>781</v>
       </c>
-      <c r="B13" s="34" t="s">
+      <c r="B74" s="1" t="s">
         <v>782</v>
       </c>
-      <c r="C13" s="34" t="s">
+      <c r="C74" s="1" t="s">
         <v>412</v>
       </c>
-      <c r="D13" s="34"/>
-      <c r="E13" s="34" t="s">
+      <c r="D74" s="1"/>
+      <c r="E74" s="1" t="s">
         <v>420</v>
       </c>
-      <c r="F13" s="36"/>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A14" s="34" t="s">
+      <c r="F74" s="8"/>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A75" s="1" t="s">
         <v>418</v>
       </c>
-      <c r="B14" s="34" t="s">
+      <c r="B75" s="1" t="s">
         <v>416</v>
       </c>
-      <c r="C14" s="34" t="s">
+      <c r="C75" s="1" t="s">
         <v>412</v>
       </c>
-      <c r="D14" s="34"/>
-      <c r="E14" s="34" t="s">
+      <c r="D75" s="1"/>
+      <c r="E75" s="1" t="s">
         <v>420</v>
       </c>
-      <c r="F14" s="36"/>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A15" s="34" t="s">
+      <c r="F75" s="8"/>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A76" s="1" t="s">
         <v>419</v>
       </c>
-      <c r="B15" s="34" t="s">
+      <c r="B76" s="1" t="s">
         <v>417</v>
       </c>
-      <c r="C15" s="34" t="s">
+      <c r="C76" s="1" t="s">
         <v>412</v>
       </c>
-      <c r="D15" s="34"/>
-      <c r="E15" s="34" t="s">
+      <c r="D76" s="1"/>
+      <c r="E76" s="1" t="s">
         <v>420</v>
       </c>
-      <c r="F15" s="36"/>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A16" s="34" t="s">
+      <c r="F76" s="8"/>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A77" s="1" t="s">
         <v>783</v>
       </c>
-      <c r="B16" s="34" t="s">
+      <c r="B77" s="1" t="s">
         <v>784</v>
       </c>
-      <c r="C16" s="34" t="s">
+      <c r="C77" s="1" t="s">
         <v>785</v>
       </c>
-      <c r="D16" s="34"/>
-      <c r="E16" s="34" t="s">
+      <c r="D77" s="1"/>
+      <c r="E77" s="1" t="s">
         <v>786</v>
       </c>
-      <c r="F16" s="36"/>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A17" s="34" t="s">
+      <c r="F77" s="8"/>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A78" s="1" t="s">
         <v>787</v>
       </c>
-      <c r="B17" s="34" t="s">
+      <c r="B78" s="1" t="s">
         <v>788</v>
       </c>
-      <c r="C17" s="34" t="s">
+      <c r="C78" s="1" t="s">
         <v>785</v>
       </c>
-      <c r="D17" s="34"/>
-      <c r="E17" s="34" t="s">
+      <c r="D78" s="1"/>
+      <c r="E78" s="1" t="s">
         <v>786</v>
       </c>
-      <c r="F17" s="36"/>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A18" s="34" t="s">
+      <c r="F78" s="8"/>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A79" s="1" t="s">
         <v>789</v>
       </c>
-      <c r="B18" s="34" t="s">
+      <c r="B79" s="1" t="s">
         <v>790</v>
       </c>
-      <c r="C18" s="34" t="s">
+      <c r="C79" s="1" t="s">
         <v>785</v>
       </c>
-      <c r="D18" s="34"/>
-      <c r="E18" s="34" t="s">
+      <c r="D79" s="1"/>
+      <c r="E79" s="1" t="s">
         <v>786</v>
       </c>
-      <c r="F18" s="36"/>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A19" s="34" t="s">
+      <c r="F79" s="8"/>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A80" s="1" t="s">
         <v>791</v>
       </c>
-      <c r="B19" s="34" t="s">
+      <c r="B80" s="1" t="s">
         <v>792</v>
       </c>
-      <c r="C19" s="34" t="s">
+      <c r="C80" s="1" t="s">
         <v>785</v>
       </c>
-      <c r="D19" s="34"/>
-      <c r="E19" s="34" t="s">
+      <c r="D80" s="1"/>
+      <c r="E80" s="1" t="s">
         <v>786</v>
       </c>
-      <c r="F19" s="36"/>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A20" s="34" t="s">
+      <c r="F80" s="8"/>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A81" s="1" t="s">
         <v>793</v>
       </c>
-      <c r="B20" s="34" t="s">
+      <c r="B81" s="1" t="s">
         <v>794</v>
       </c>
-      <c r="C20" s="34" t="s">
+      <c r="C81" s="1" t="s">
         <v>785</v>
       </c>
-      <c r="D20" s="34"/>
-      <c r="E20" s="34" t="s">
+      <c r="D81" s="1"/>
+      <c r="E81" s="1" t="s">
         <v>786</v>
       </c>
-      <c r="F20" s="36"/>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A21" s="34" t="s">
+      <c r="F81" s="8"/>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A82" s="1" t="s">
         <v>795</v>
       </c>
-      <c r="B21" s="34" t="s">
+      <c r="B82" s="1" t="s">
         <v>796</v>
       </c>
-      <c r="C21" s="34" t="s">
+      <c r="C82" s="1" t="s">
         <v>797</v>
       </c>
-      <c r="D21" s="34"/>
-      <c r="E21" s="34" t="s">
+      <c r="D82" s="1"/>
+      <c r="E82" s="1" t="s">
         <v>786</v>
       </c>
-      <c r="F21" s="36"/>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A22" s="34" t="s">
+      <c r="F82" s="8"/>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A83" s="1" t="s">
         <v>798</v>
       </c>
-      <c r="B22" s="34" t="s">
+      <c r="B83" s="1" t="s">
         <v>799</v>
       </c>
-      <c r="C22" s="34" t="s">
+      <c r="C83" s="1" t="s">
         <v>797</v>
       </c>
-      <c r="D22" s="34"/>
-      <c r="E22" s="34" t="s">
+      <c r="D83" s="1"/>
+      <c r="E83" s="1" t="s">
         <v>800</v>
       </c>
-      <c r="F22" s="36"/>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A23" s="34" t="s">
+      <c r="F83" s="8"/>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A84" s="1" t="s">
         <v>801</v>
       </c>
-      <c r="B23" s="34" t="s">
+      <c r="B84" s="1" t="s">
         <v>802</v>
       </c>
-      <c r="C23" s="34" t="s">
+      <c r="C84" s="1" t="s">
         <v>797</v>
       </c>
-      <c r="D23" s="34"/>
-      <c r="E23" s="34" t="s">
+      <c r="D84" s="1"/>
+      <c r="E84" s="1" t="s">
         <v>800</v>
       </c>
-      <c r="F23" s="36"/>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A24" s="34" t="s">
+      <c r="F84" s="8"/>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A85" s="1" t="s">
         <v>803</v>
       </c>
-      <c r="B24" s="34" t="s">
+      <c r="B85" s="1" t="s">
         <v>804</v>
       </c>
-      <c r="C24" s="34" t="s">
+      <c r="C85" s="1" t="s">
         <v>797</v>
       </c>
-      <c r="D24" s="34"/>
-      <c r="E24" s="34" t="s">
+      <c r="D85" s="1"/>
+      <c r="E85" s="1" t="s">
         <v>800</v>
       </c>
-      <c r="F24" s="36"/>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A25" s="34" t="s">
+      <c r="F85" s="8"/>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A86" s="1" t="s">
         <v>805</v>
       </c>
-      <c r="B25" s="34" t="s">
+      <c r="B86" s="1" t="s">
         <v>806</v>
       </c>
-      <c r="C25" s="34" t="s">
+      <c r="C86" s="1" t="s">
         <v>797</v>
       </c>
-      <c r="D25" s="34"/>
-      <c r="E25" s="34" t="s">
+      <c r="D86" s="1"/>
+      <c r="E86" s="1" t="s">
         <v>807</v>
       </c>
-      <c r="F25" s="36"/>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A26" s="34" t="s">
+      <c r="F86" s="8"/>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A87" s="1" t="s">
         <v>808</v>
       </c>
-      <c r="B26" s="34" t="s">
+      <c r="B87" s="1" t="s">
         <v>809</v>
       </c>
-      <c r="C26" s="34" t="s">
+      <c r="C87" s="1" t="s">
         <v>797</v>
       </c>
-      <c r="D26" s="34"/>
-      <c r="E26" s="34" t="s">
+      <c r="D87" s="1"/>
+      <c r="E87" s="1" t="s">
         <v>807</v>
       </c>
-      <c r="F26" s="36"/>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A27" s="34" t="s">
+      <c r="F87" s="8"/>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A88" s="1" t="s">
         <v>810</v>
       </c>
-      <c r="B27" s="34" t="s">
+      <c r="B88" s="1" t="s">
         <v>811</v>
       </c>
-      <c r="C27" s="34" t="s">
+      <c r="C88" s="1" t="s">
         <v>797</v>
       </c>
-      <c r="D27" s="34"/>
-      <c r="E27" s="34" t="s">
+      <c r="D88" s="1"/>
+      <c r="E88" s="1" t="s">
         <v>807</v>
       </c>
-      <c r="F27" s="36"/>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A28" s="34" t="s">
+      <c r="F88" s="8"/>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A89" s="1" t="s">
         <v>812</v>
       </c>
-      <c r="B28" s="34" t="s">
+      <c r="B89" s="1" t="s">
         <v>813</v>
       </c>
-      <c r="C28" s="34" t="s">
+      <c r="C89" s="1" t="s">
         <v>797</v>
       </c>
-      <c r="D28" s="34"/>
-      <c r="E28" s="34" t="s">
+      <c r="D89" s="1"/>
+      <c r="E89" s="1" t="s">
         <v>814</v>
       </c>
-      <c r="F28" s="36"/>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A29" s="34" t="s">
+      <c r="F89" s="8"/>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A90" s="1" t="s">
         <v>815</v>
       </c>
-      <c r="B29" s="34" t="s">
+      <c r="B90" s="1" t="s">
         <v>816</v>
       </c>
-      <c r="C29" s="34" t="s">
+      <c r="C90" s="1" t="s">
         <v>797</v>
       </c>
-      <c r="D29" s="34"/>
-      <c r="E29" s="34" t="s">
+      <c r="D90" s="1"/>
+      <c r="E90" s="1" t="s">
         <v>814</v>
       </c>
-      <c r="F29" s="36"/>
-    </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A30" s="34" t="s">
+      <c r="F90" s="8"/>
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A91" s="1" t="s">
         <v>817</v>
       </c>
-      <c r="B30" s="34" t="s">
+      <c r="B91" s="1" t="s">
         <v>818</v>
       </c>
-      <c r="C30" s="34" t="s">
+      <c r="C91" s="1" t="s">
         <v>797</v>
       </c>
-      <c r="D30" s="34"/>
-      <c r="E30" s="34" t="s">
+      <c r="D91" s="1"/>
+      <c r="E91" s="1" t="s">
         <v>814</v>
       </c>
-      <c r="F30" s="36"/>
-    </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A31" s="34" t="s">
+      <c r="F91" s="8"/>
+    </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A92" s="1" t="s">
         <v>819</v>
       </c>
-      <c r="B31" s="37" t="s">
+      <c r="B92" t="s">
         <v>820</v>
       </c>
-      <c r="C31" s="34" t="s">
+      <c r="C92" s="1" t="s">
         <v>797</v>
       </c>
-      <c r="D31" s="34"/>
-      <c r="E31" s="34" t="s">
+      <c r="D92" s="1"/>
+      <c r="E92" s="1" t="s">
         <v>814</v>
       </c>
-      <c r="F31" s="36"/>
-    </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A32" s="34" t="s">
+      <c r="F92" s="8"/>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A93" s="1" t="s">
         <v>821</v>
       </c>
-      <c r="B32" s="34" t="s">
+      <c r="B93" s="1" t="s">
         <v>822</v>
       </c>
-      <c r="C32" s="34" t="s">
+      <c r="C93" s="1" t="s">
         <v>823</v>
       </c>
-      <c r="D32" s="34"/>
-      <c r="E32" s="34" t="s">
+      <c r="D93" s="1"/>
+      <c r="E93" s="1" t="s">
         <v>824</v>
       </c>
-      <c r="F32" s="36"/>
-    </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A33" s="34" t="s">
+      <c r="F93" s="8"/>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A94" s="1" t="s">
         <v>825</v>
       </c>
-      <c r="B33" s="34" t="s">
+      <c r="B94" s="1" t="s">
         <v>826</v>
       </c>
-      <c r="C33" s="34" t="s">
+      <c r="C94" s="1" t="s">
         <v>823</v>
       </c>
-      <c r="D33" s="34"/>
-      <c r="E33" s="34" t="s">
+      <c r="D94" s="1"/>
+      <c r="E94" s="1" t="s">
         <v>824</v>
       </c>
-      <c r="F33" s="36"/>
-    </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A34" s="34" t="s">
+      <c r="F94" s="8"/>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A95" s="1" t="s">
         <v>421</v>
       </c>
-      <c r="B34" s="34" t="s">
+      <c r="B95" s="1" t="s">
         <v>424</v>
       </c>
-      <c r="C34" s="34" t="s">
+      <c r="C95" s="1" t="s">
         <v>427</v>
       </c>
-      <c r="D34" s="34"/>
-      <c r="E34" s="34" t="s">
+      <c r="D95" s="1"/>
+      <c r="E95" s="1" t="s">
         <v>430</v>
       </c>
-      <c r="F34" s="36"/>
-    </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A35" s="34" t="s">
+      <c r="F95" s="8"/>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A96" s="1" t="s">
         <v>422</v>
       </c>
-      <c r="B35" s="37" t="s">
+      <c r="B96" t="s">
         <v>425</v>
       </c>
-      <c r="C35" s="34" t="s">
+      <c r="C96" s="1" t="s">
         <v>427</v>
       </c>
-      <c r="D35" s="34"/>
-      <c r="E35" s="34" t="s">
+      <c r="D96" s="1"/>
+      <c r="E96" s="1" t="s">
         <v>430</v>
       </c>
-      <c r="F35" s="36"/>
-    </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A36" s="34" t="s">
+      <c r="F96" s="8"/>
+    </row>
+    <row r="97" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A97" s="1" t="s">
         <v>423</v>
       </c>
-      <c r="B36" s="34" t="s">
+      <c r="B97" s="1" t="s">
         <v>426</v>
       </c>
-      <c r="C36" s="34" t="s">
+      <c r="C97" s="1" t="s">
         <v>427</v>
       </c>
-      <c r="D36" s="34"/>
-      <c r="E36" s="34" t="s">
+      <c r="D97" s="1"/>
+      <c r="E97" s="1" t="s">
         <v>430</v>
       </c>
-      <c r="F36" s="36"/>
-    </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A37" s="34" t="s">
+      <c r="F97" s="8"/>
+    </row>
+    <row r="98" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A98" s="1" t="s">
         <v>428</v>
       </c>
-      <c r="B37" s="34" t="s">
+      <c r="B98" s="1" t="s">
         <v>429</v>
       </c>
-      <c r="C37" s="34" t="s">
+      <c r="C98" s="1" t="s">
         <v>432</v>
       </c>
-      <c r="D37" s="34"/>
-      <c r="E37" s="34" t="s">
+      <c r="D98" s="1"/>
+      <c r="E98" s="1" t="s">
         <v>431</v>
       </c>
-      <c r="F37" s="36"/>
-    </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A38" s="34" t="s">
+      <c r="F98" s="8"/>
+    </row>
+    <row r="99" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A99" s="1" t="s">
         <v>433</v>
       </c>
-      <c r="B38" s="34" t="s">
+      <c r="B99" s="1" t="s">
         <v>434</v>
       </c>
-      <c r="C38" s="34" t="s">
+      <c r="C99" s="1" t="s">
         <v>432</v>
       </c>
-      <c r="D38" s="34"/>
-      <c r="E38" s="34" t="s">
+      <c r="D99" s="1"/>
+      <c r="E99" s="1" t="s">
         <v>435</v>
       </c>
-      <c r="F38" s="36"/>
-    </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A39" s="34" t="s">
+      <c r="F99" s="8"/>
+    </row>
+    <row r="100" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A100" s="1" t="s">
         <v>827</v>
       </c>
-      <c r="B39" s="37" t="s">
+      <c r="B100" t="s">
         <v>828</v>
       </c>
-      <c r="C39" s="34" t="s">
+      <c r="C100" s="1" t="s">
         <v>432</v>
       </c>
-      <c r="D39" s="34"/>
-      <c r="E39" s="34" t="s">
+      <c r="D100" s="1"/>
+      <c r="E100" s="1" t="s">
         <v>435</v>
       </c>
-      <c r="F39" s="36"/>
-    </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A40" s="34" t="s">
+      <c r="F100" s="8"/>
+    </row>
+    <row r="101" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A101" s="1" t="s">
         <v>438</v>
       </c>
-      <c r="B40" s="34" t="s">
+      <c r="B101" s="1" t="s">
         <v>436</v>
       </c>
-      <c r="C40" s="34" t="s">
+      <c r="C101" s="1" t="s">
         <v>437</v>
       </c>
-      <c r="D40" s="34"/>
-      <c r="E40" s="34" t="s">
+      <c r="D101" s="1"/>
+      <c r="E101" s="1" t="s">
         <v>439</v>
       </c>
-      <c r="F40" s="36"/>
-    </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A41" s="34" t="s">
+      <c r="F101" s="8"/>
+    </row>
+    <row r="102" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A102" s="1" t="s">
         <v>829</v>
       </c>
-      <c r="B41" s="34" t="s">
+      <c r="B102" s="1" t="s">
         <v>830</v>
       </c>
-      <c r="C41" s="34" t="s">
+      <c r="C102" s="1" t="s">
         <v>437</v>
       </c>
-      <c r="D41" s="34"/>
-      <c r="E41" s="34" t="s">
+      <c r="D102" s="1"/>
+      <c r="E102" s="1" t="s">
         <v>831</v>
       </c>
-      <c r="F41" s="36"/>
-    </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A42" s="34" t="s">
+      <c r="F102" s="8"/>
+    </row>
+    <row r="103" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A103" s="1" t="s">
         <v>832</v>
       </c>
-      <c r="B42" s="34" t="s">
+      <c r="B103" s="1" t="s">
         <v>833</v>
       </c>
-      <c r="C42" s="34" t="s">
+      <c r="C103" s="1" t="s">
         <v>437</v>
       </c>
-      <c r="D42" s="34"/>
-      <c r="E42" s="34" t="s">
+      <c r="D103" s="1"/>
+      <c r="E103" s="1" t="s">
         <v>831</v>
       </c>
-      <c r="F42" s="36"/>
-    </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A43" s="34" t="s">
+      <c r="F103" s="8"/>
+    </row>
+    <row r="104" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A104" s="1" t="s">
         <v>443</v>
       </c>
-      <c r="B43" s="34" t="s">
+      <c r="B104" s="1" t="s">
         <v>440</v>
       </c>
-      <c r="C43" s="34" t="s">
+      <c r="C104" s="1" t="s">
         <v>437</v>
       </c>
-      <c r="D43" s="34"/>
-      <c r="E43" s="34" t="s">
+      <c r="D104" s="1"/>
+      <c r="E104" s="1" t="s">
         <v>445</v>
       </c>
-      <c r="F43" s="36"/>
-    </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A44" s="34" t="s">
+      <c r="F104" s="8"/>
+    </row>
+    <row r="105" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A105" s="1" t="s">
         <v>834</v>
       </c>
-      <c r="B44" s="34" t="s">
+      <c r="B105" s="1" t="s">
         <v>835</v>
       </c>
-      <c r="C44" s="34" t="s">
+      <c r="C105" s="1" t="s">
         <v>437</v>
       </c>
-      <c r="D44" s="34"/>
-      <c r="E44" s="34" t="s">
+      <c r="D105" s="1"/>
+      <c r="E105" s="1" t="s">
         <v>445</v>
       </c>
-      <c r="F44" s="36"/>
-    </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A45" s="34" t="s">
+      <c r="F105" s="8"/>
+    </row>
+    <row r="106" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A106" s="1" t="s">
         <v>444</v>
       </c>
-      <c r="B45" s="34" t="s">
+      <c r="B106" s="1" t="s">
         <v>442</v>
       </c>
-      <c r="C45" s="34" t="s">
+      <c r="C106" s="1" t="s">
         <v>437</v>
       </c>
-      <c r="D45" s="34"/>
-      <c r="E45" s="34" t="s">
+      <c r="D106" s="1"/>
+      <c r="E106" s="1" t="s">
         <v>445</v>
       </c>
-      <c r="F45" s="36"/>
-    </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A46" s="34" t="s">
+      <c r="F106" s="8"/>
+    </row>
+    <row r="107" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A107" s="1" t="s">
         <v>473</v>
       </c>
-      <c r="B46" s="34" t="s">
+      <c r="B107" s="1" t="s">
         <v>441</v>
       </c>
-      <c r="C46" s="34" t="s">
+      <c r="C107" s="1" t="s">
         <v>437</v>
       </c>
-      <c r="D46" s="34"/>
-      <c r="E46" s="34" t="s">
+      <c r="D107" s="1"/>
+      <c r="E107" s="1" t="s">
         <v>445</v>
       </c>
-      <c r="F46" s="36"/>
-    </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A47" s="34" t="s">
+      <c r="F107" s="8"/>
+    </row>
+    <row r="108" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A108" s="1" t="s">
         <v>454</v>
       </c>
-      <c r="B47" s="34" t="s">
+      <c r="B108" s="1" t="s">
         <v>446</v>
       </c>
-      <c r="C47" s="34" t="s">
+      <c r="C108" s="1" t="s">
         <v>452</v>
       </c>
-      <c r="D47" s="34" t="s">
-        <v>848</v>
-      </c>
-      <c r="E47" s="34" t="s">
+      <c r="D108" s="1" t="s">
+        <v>855</v>
+      </c>
+      <c r="E108" s="1" t="s">
         <v>453</v>
       </c>
-      <c r="F47" s="36"/>
-    </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A48" s="34" t="s">
+      <c r="F108" s="8"/>
+    </row>
+    <row r="109" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A109" s="1" t="s">
         <v>455</v>
       </c>
-      <c r="B48" s="34" t="s">
+      <c r="B109" s="1" t="s">
         <v>447</v>
       </c>
-      <c r="C48" s="34" t="s">
+      <c r="C109" s="1" t="s">
         <v>452</v>
       </c>
-      <c r="D48" s="34"/>
-      <c r="E48" s="34" t="s">
+      <c r="D109" s="1" t="s">
+        <v>855</v>
+      </c>
+      <c r="E109" s="1" t="s">
         <v>453</v>
       </c>
-      <c r="F48" s="36"/>
-    </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A49" s="34" t="s">
+      <c r="F109" s="8"/>
+    </row>
+    <row r="110" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A110" s="1" t="s">
         <v>456</v>
       </c>
-      <c r="B49" s="34" t="s">
+      <c r="B110" s="1" t="s">
         <v>448</v>
       </c>
-      <c r="C49" s="34" t="s">
+      <c r="C110" s="1" t="s">
         <v>452</v>
       </c>
-      <c r="D49" s="34"/>
-      <c r="E49" s="34" t="s">
+      <c r="D110" s="1" t="s">
+        <v>855</v>
+      </c>
+      <c r="E110" s="1" t="s">
         <v>453</v>
       </c>
-      <c r="F49" s="36"/>
-    </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A50" s="34" t="s">
+      <c r="F110" s="8"/>
+    </row>
+    <row r="111" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A111" s="1" t="s">
         <v>457</v>
       </c>
-      <c r="B50" s="34" t="s">
+      <c r="B111" s="1" t="s">
         <v>449</v>
       </c>
-      <c r="C50" s="34" t="s">
+      <c r="C111" s="1" t="s">
         <v>452</v>
       </c>
-      <c r="D50" s="34"/>
-      <c r="E50" s="34" t="s">
+      <c r="D111" s="1" t="s">
+        <v>855</v>
+      </c>
+      <c r="E111" s="1" t="s">
         <v>453</v>
       </c>
-      <c r="F50" s="36"/>
-    </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A51" s="34" t="s">
+      <c r="F111" s="8"/>
+    </row>
+    <row r="112" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A112" s="1" t="s">
         <v>458</v>
       </c>
-      <c r="B51" s="34" t="s">
+      <c r="B112" s="1" t="s">
         <v>450</v>
       </c>
-      <c r="C51" s="34" t="s">
+      <c r="C112" s="1" t="s">
         <v>452</v>
       </c>
-      <c r="D51" s="34" t="s">
-        <v>853</v>
-      </c>
-      <c r="E51" s="34" t="s">
+      <c r="D112" s="1" t="s">
+        <v>855</v>
+      </c>
+      <c r="E112" s="1" t="s">
         <v>453</v>
       </c>
-      <c r="F51" s="36"/>
-    </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A52" s="34" t="s">
+      <c r="F112" s="8"/>
+    </row>
+    <row r="113" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A113" s="1" t="s">
         <v>459</v>
       </c>
-      <c r="B52" s="34" t="s">
+      <c r="B113" s="1" t="s">
         <v>451</v>
       </c>
-      <c r="C52" s="34" t="s">
+      <c r="C113" s="1" t="s">
         <v>452</v>
       </c>
-      <c r="D52" s="34" t="s">
-        <v>854</v>
-      </c>
-      <c r="E52" s="34" t="s">
+      <c r="D113" s="1" t="s">
+        <v>855</v>
+      </c>
+      <c r="E113" s="1" t="s">
         <v>453</v>
       </c>
-      <c r="F52" s="36"/>
-    </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A53" s="34" t="s">
+      <c r="F113" s="8"/>
+    </row>
+    <row r="114" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A114" s="1" t="s">
         <v>463</v>
       </c>
-      <c r="B53" s="34" t="s">
+      <c r="B114" s="1" t="s">
         <v>460</v>
       </c>
-      <c r="C53" s="34" t="s">
+      <c r="C114" s="1" t="s">
         <v>462</v>
       </c>
-      <c r="D53" s="34"/>
-      <c r="E53" s="34" t="s">
+      <c r="D114" s="1" t="s">
+        <v>855</v>
+      </c>
+      <c r="E114" s="1" t="s">
         <v>465</v>
       </c>
-      <c r="F53" s="36"/>
-    </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A54" s="34" t="s">
+      <c r="F114" s="8"/>
+    </row>
+    <row r="115" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A115" s="1" t="s">
         <v>464</v>
       </c>
-      <c r="B54" s="37" t="s">
+      <c r="B115" t="s">
         <v>461</v>
       </c>
-      <c r="C54" s="34" t="s">
+      <c r="C115" s="1" t="s">
         <v>462</v>
       </c>
-      <c r="D54" s="34"/>
-      <c r="E54" s="34" t="s">
+      <c r="D115" s="1" t="s">
+        <v>855</v>
+      </c>
+      <c r="E115" s="1" t="s">
         <v>465</v>
       </c>
-      <c r="F54" s="36"/>
-    </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A55" s="34" t="s">
+      <c r="F115" s="8"/>
+    </row>
+    <row r="116" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A116" s="1" t="s">
         <v>469</v>
       </c>
-      <c r="B55" s="34" t="s">
+      <c r="B116" s="1" t="s">
         <v>466</v>
       </c>
-      <c r="C55" s="34" t="s">
+      <c r="C116" s="1" t="s">
         <v>468</v>
       </c>
-      <c r="D55" s="34"/>
-      <c r="E55" s="34" t="s">
+      <c r="D116" s="1"/>
+      <c r="E116" s="1" t="s">
         <v>471</v>
       </c>
-      <c r="F55" s="36"/>
-    </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A56" s="34" t="s">
+      <c r="F116" s="8"/>
+    </row>
+    <row r="117" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A117" s="1" t="s">
         <v>470</v>
       </c>
-      <c r="B56" s="34" t="s">
+      <c r="B117" s="1" t="s">
         <v>467</v>
       </c>
-      <c r="C56" s="34" t="s">
+      <c r="C117" s="1" t="s">
         <v>468</v>
       </c>
-      <c r="D56" s="34"/>
-      <c r="E56" s="34" t="s">
+      <c r="D117" s="1"/>
+      <c r="E117" s="1" t="s">
         <v>471</v>
       </c>
-      <c r="F56" s="36"/>
-    </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A57" s="34" t="s">
+      <c r="F117" s="8"/>
+    </row>
+    <row r="118" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A118" s="1" t="s">
         <v>836</v>
       </c>
-      <c r="B57" s="34" t="s">
+      <c r="B118" s="1" t="s">
         <v>837</v>
       </c>
-      <c r="C57" s="34" t="s">
+      <c r="C118" s="1" t="s">
         <v>838</v>
       </c>
-      <c r="D57" s="34"/>
-      <c r="E57" s="34" t="s">
+      <c r="D118" s="1"/>
+      <c r="E118" s="1" t="s">
         <v>839</v>
       </c>
-      <c r="F57" s="36"/>
-    </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A58" s="34" t="s">
+      <c r="F118" s="8"/>
+    </row>
+    <row r="119" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A119" s="1" t="s">
         <v>840</v>
       </c>
-      <c r="B58" s="34" t="s">
+      <c r="B119" s="1" t="s">
         <v>841</v>
       </c>
-      <c r="C58" s="34" t="s">
+      <c r="C119" s="1" t="s">
         <v>838</v>
       </c>
-      <c r="D58" s="34"/>
-      <c r="E58" s="34" t="s">
+      <c r="D119" s="1"/>
+      <c r="E119" s="1" t="s">
         <v>839</v>
       </c>
-      <c r="F58" s="36"/>
-    </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A59" s="34" t="s">
+      <c r="F119" s="8"/>
+    </row>
+    <row r="120" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A120" s="1" t="s">
         <v>842</v>
       </c>
-      <c r="B59" s="34" t="s">
+      <c r="B120" s="1" t="s">
         <v>843</v>
       </c>
-      <c r="C59" s="34" t="s">
+      <c r="C120" s="1" t="s">
         <v>838</v>
       </c>
-      <c r="D59" s="34"/>
-      <c r="E59" s="34" t="s">
+      <c r="D120" s="1"/>
+      <c r="E120" s="1" t="s">
         <v>844</v>
       </c>
-      <c r="F59" s="36"/>
-    </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A60" s="34" t="s">
+      <c r="F120" s="8"/>
+    </row>
+    <row r="121" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A121" s="1" t="s">
         <v>845</v>
       </c>
-      <c r="B60" s="34" t="s">
+      <c r="B121" s="1" t="s">
         <v>846</v>
       </c>
-      <c r="C60" s="34" t="s">
+      <c r="C121" s="1" t="s">
         <v>838</v>
       </c>
-      <c r="D60" s="34"/>
-      <c r="E60" s="34" t="s">
+      <c r="D121" s="1"/>
+      <c r="E121" s="1" t="s">
         <v>844</v>
       </c>
-      <c r="F60" s="36"/>
-    </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A61" s="32"/>
-      <c r="B61" s="32"/>
-      <c r="C61" s="32"/>
-      <c r="D61" s="32"/>
-      <c r="E61" s="32"/>
-      <c r="F61" s="7"/>
-    </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A62" s="32"/>
-      <c r="B62" s="32"/>
-      <c r="C62" s="32"/>
-      <c r="D62" s="33"/>
-      <c r="E62" s="32"/>
-      <c r="F62" s="7"/>
-    </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A63" s="32"/>
-      <c r="B63" s="32"/>
-      <c r="C63" s="32"/>
-      <c r="D63" s="32"/>
-      <c r="E63" s="32"/>
-      <c r="F63" s="7"/>
-    </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A64" s="32"/>
-      <c r="B64" s="32"/>
-      <c r="C64" s="32"/>
-      <c r="D64" s="32"/>
-      <c r="E64" s="32"/>
-      <c r="F64" s="7"/>
-    </row>
-    <row r="65" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A65" s="32"/>
-      <c r="B65" s="32"/>
-      <c r="C65" s="32"/>
-      <c r="D65" s="32"/>
-      <c r="E65" s="32"/>
-      <c r="F65" s="7"/>
-    </row>
-    <row r="66" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A66" s="32"/>
-      <c r="B66" s="32"/>
-      <c r="C66" s="32"/>
-      <c r="D66" s="32"/>
-      <c r="E66" s="32"/>
-      <c r="F66" s="7"/>
-    </row>
-    <row r="67" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A67" s="32"/>
-      <c r="B67" s="32"/>
-      <c r="C67" s="32"/>
-      <c r="D67" s="32"/>
-      <c r="E67" s="32"/>
-      <c r="F67" s="7"/>
-    </row>
-    <row r="68" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A68" s="32"/>
-      <c r="B68" s="32"/>
-      <c r="C68" s="32"/>
-      <c r="D68" s="32"/>
-      <c r="E68" s="32"/>
-      <c r="F68" s="7"/>
-    </row>
-    <row r="69" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A69" s="32"/>
-      <c r="B69" s="32"/>
-      <c r="C69" s="32"/>
-      <c r="D69" s="32"/>
-      <c r="E69" s="32"/>
-      <c r="F69" s="7"/>
-    </row>
-    <row r="70" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A70" s="32"/>
-      <c r="B70" s="33"/>
-      <c r="C70" s="32"/>
-      <c r="D70" s="32"/>
-      <c r="E70" s="32"/>
-      <c r="F70" s="7"/>
-    </row>
-    <row r="71" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A71" s="32"/>
-      <c r="B71" s="32"/>
-      <c r="C71" s="32"/>
-      <c r="D71" s="32"/>
-      <c r="E71" s="32"/>
-      <c r="F71" s="7"/>
-    </row>
-    <row r="72" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A72" s="25" t="s">
-        <v>112</v>
-      </c>
-      <c r="B72" s="25"/>
-      <c r="C72" s="25"/>
-      <c r="D72" s="25"/>
-      <c r="E72" s="25"/>
-      <c r="F72" s="25"/>
-      <c r="G72" s="25"/>
-      <c r="H72" s="25"/>
-      <c r="I72" s="25"/>
-      <c r="J72" s="25"/>
-      <c r="K72" s="25"/>
-    </row>
-    <row r="73" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A73" s="2" t="s">
+      <c r="F121" s="8"/>
+    </row>
+    <row r="122" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A122" s="1"/>
+      <c r="B122" s="1"/>
+      <c r="C122" s="1"/>
+      <c r="D122" s="1"/>
+      <c r="E122" s="1"/>
+      <c r="F122" s="8"/>
+    </row>
+    <row r="123" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A123" s="27" t="s">
+        <v>776</v>
+      </c>
+      <c r="B123" s="27"/>
+      <c r="C123" s="27"/>
+      <c r="D123" s="27"/>
+      <c r="E123" s="27"/>
+      <c r="F123" s="27"/>
+      <c r="G123" s="27"/>
+      <c r="H123" s="27"/>
+      <c r="I123" s="27"/>
+      <c r="J123" s="27"/>
+      <c r="K123" s="27"/>
+    </row>
+    <row r="124" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A124" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="B73" s="2" t="s">
+      <c r="B124" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="C73" s="2" t="s">
+      <c r="C124" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="D73" s="2" t="s">
+      <c r="D124" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="E73" s="2" t="s">
+      <c r="E124" s="2" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="74" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A74" s="34" t="s">
-        <v>778</v>
-      </c>
-      <c r="B74" s="34" t="s">
-        <v>779</v>
-      </c>
-      <c r="C74" s="34" t="s">
-        <v>780</v>
-      </c>
-      <c r="D74" s="34"/>
-      <c r="E74" s="34" t="s">
-        <v>399</v>
-      </c>
-    </row>
-    <row r="75" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A75" s="34" t="s">
-        <v>393</v>
-      </c>
-      <c r="B75" s="35" t="s">
-        <v>396</v>
-      </c>
-      <c r="C75" s="34" t="s">
-        <v>780</v>
-      </c>
-      <c r="D75" s="34"/>
-      <c r="E75" s="34" t="s">
-        <v>399</v>
-      </c>
-      <c r="F75" s="8" t="s">
-        <v>472</v>
-      </c>
-    </row>
-    <row r="76" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A76" s="34" t="s">
-        <v>394</v>
-      </c>
-      <c r="B76" s="35" t="s">
-        <v>397</v>
-      </c>
-      <c r="C76" s="34" t="s">
-        <v>780</v>
-      </c>
-      <c r="D76" s="34"/>
-      <c r="E76" s="34" t="s">
-        <v>399</v>
-      </c>
-      <c r="F76" s="8" t="s">
-        <v>773</v>
-      </c>
-    </row>
-    <row r="77" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A77" s="34" t="s">
-        <v>395</v>
-      </c>
-      <c r="B77" s="35" t="s">
-        <v>398</v>
-      </c>
-      <c r="C77" s="34" t="s">
-        <v>780</v>
-      </c>
-      <c r="D77" s="34"/>
-      <c r="E77" s="34" t="s">
-        <v>399</v>
-      </c>
-      <c r="F77" s="8"/>
-    </row>
-    <row r="78" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A78" s="34" t="s">
-        <v>406</v>
-      </c>
-      <c r="B78" s="35" t="s">
-        <v>400</v>
-      </c>
-      <c r="C78" s="34" t="s">
-        <v>412</v>
-      </c>
-      <c r="D78" s="34"/>
-      <c r="E78" s="34" t="s">
-        <v>413</v>
-      </c>
-      <c r="F78" s="8"/>
-    </row>
-    <row r="79" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A79" s="34" t="s">
-        <v>407</v>
-      </c>
-      <c r="B79" s="34" t="s">
-        <v>401</v>
-      </c>
-      <c r="C79" s="34" t="s">
-        <v>412</v>
-      </c>
-      <c r="D79" s="34"/>
-      <c r="E79" s="34" t="s">
-        <v>413</v>
-      </c>
-      <c r="F79" s="8"/>
-    </row>
-    <row r="80" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A80" s="34" t="s">
-        <v>408</v>
-      </c>
-      <c r="B80" s="34" t="s">
-        <v>402</v>
-      </c>
-      <c r="C80" s="34" t="s">
-        <v>412</v>
-      </c>
-      <c r="D80" s="34"/>
-      <c r="E80" s="34" t="s">
-        <v>414</v>
-      </c>
-      <c r="F80" s="8"/>
-    </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A81" s="34" t="s">
-        <v>409</v>
-      </c>
-      <c r="B81" s="34" t="s">
-        <v>403</v>
-      </c>
-      <c r="C81" s="34" t="s">
-        <v>412</v>
-      </c>
-      <c r="D81" s="34"/>
-      <c r="E81" s="34" t="s">
-        <v>414</v>
-      </c>
-      <c r="F81" s="8"/>
-    </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A82" s="34" t="s">
-        <v>410</v>
-      </c>
-      <c r="B82" s="34" t="s">
-        <v>404</v>
-      </c>
-      <c r="C82" s="34" t="s">
-        <v>412</v>
-      </c>
-      <c r="D82" s="34"/>
-      <c r="E82" s="34" t="s">
-        <v>414</v>
-      </c>
-      <c r="F82" s="8"/>
-    </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A83" s="34" t="s">
-        <v>411</v>
-      </c>
-      <c r="B83" s="34" t="s">
-        <v>405</v>
-      </c>
-      <c r="C83" s="34" t="s">
-        <v>412</v>
-      </c>
-      <c r="D83" s="34"/>
-      <c r="E83" s="34" t="s">
-        <v>414</v>
-      </c>
-      <c r="F83" s="8"/>
-    </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A84" s="34" t="s">
-        <v>781</v>
-      </c>
-      <c r="B84" s="34" t="s">
-        <v>782</v>
-      </c>
-      <c r="C84" s="34" t="s">
-        <v>412</v>
-      </c>
-      <c r="D84" s="34"/>
-      <c r="E84" s="34" t="s">
-        <v>420</v>
-      </c>
-      <c r="F84" s="8"/>
-    </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A85" s="34" t="s">
-        <v>418</v>
-      </c>
-      <c r="B85" s="34" t="s">
-        <v>416</v>
-      </c>
-      <c r="C85" s="34" t="s">
-        <v>412</v>
-      </c>
-      <c r="D85" s="34"/>
-      <c r="E85" s="34" t="s">
-        <v>420</v>
-      </c>
-      <c r="F85" s="8"/>
-    </row>
-    <row r="86" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A86" s="34" t="s">
-        <v>419</v>
-      </c>
-      <c r="B86" s="34" t="s">
-        <v>417</v>
-      </c>
-      <c r="C86" s="34" t="s">
-        <v>412</v>
-      </c>
-      <c r="D86" s="34"/>
-      <c r="E86" s="34" t="s">
-        <v>420</v>
-      </c>
-      <c r="F86" s="8"/>
-    </row>
-    <row r="87" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A87" s="34" t="s">
-        <v>783</v>
-      </c>
-      <c r="B87" s="34" t="s">
-        <v>784</v>
-      </c>
-      <c r="C87" s="34" t="s">
-        <v>785</v>
-      </c>
-      <c r="D87" s="34"/>
-      <c r="E87" s="34" t="s">
-        <v>786</v>
-      </c>
-      <c r="F87" s="8"/>
-    </row>
-    <row r="88" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A88" s="34" t="s">
-        <v>787</v>
-      </c>
-      <c r="B88" s="34" t="s">
-        <v>788</v>
-      </c>
-      <c r="C88" s="34" t="s">
-        <v>785</v>
-      </c>
-      <c r="D88" s="34"/>
-      <c r="E88" s="34" t="s">
-        <v>786</v>
-      </c>
-      <c r="F88" s="8"/>
-    </row>
-    <row r="89" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A89" s="34" t="s">
-        <v>789</v>
-      </c>
-      <c r="B89" s="34" t="s">
-        <v>790</v>
-      </c>
-      <c r="C89" s="34" t="s">
-        <v>785</v>
-      </c>
-      <c r="D89" s="34"/>
-      <c r="E89" s="34" t="s">
-        <v>786</v>
-      </c>
-      <c r="F89" s="8"/>
-    </row>
-    <row r="90" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A90" s="34" t="s">
-        <v>791</v>
-      </c>
-      <c r="B90" s="34" t="s">
-        <v>792</v>
-      </c>
-      <c r="C90" s="34" t="s">
-        <v>785</v>
-      </c>
-      <c r="D90" s="34"/>
-      <c r="E90" s="34" t="s">
-        <v>786</v>
-      </c>
-      <c r="F90" s="8"/>
-    </row>
-    <row r="91" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A91" s="34" t="s">
-        <v>793</v>
-      </c>
-      <c r="B91" s="34" t="s">
-        <v>794</v>
-      </c>
-      <c r="C91" s="34" t="s">
-        <v>785</v>
-      </c>
-      <c r="D91" s="34"/>
-      <c r="E91" s="34" t="s">
-        <v>786</v>
-      </c>
-      <c r="F91" s="8"/>
-    </row>
-    <row r="92" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A92" s="34" t="s">
-        <v>795</v>
-      </c>
-      <c r="B92" s="34" t="s">
-        <v>796</v>
-      </c>
-      <c r="C92" s="34" t="s">
-        <v>797</v>
-      </c>
-      <c r="D92" s="34"/>
-      <c r="E92" s="34" t="s">
-        <v>786</v>
-      </c>
-      <c r="F92" s="8"/>
-    </row>
-    <row r="93" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A93" s="34" t="s">
-        <v>798</v>
-      </c>
-      <c r="B93" s="34" t="s">
-        <v>799</v>
-      </c>
-      <c r="C93" s="34" t="s">
-        <v>797</v>
-      </c>
-      <c r="D93" s="34"/>
-      <c r="E93" s="34" t="s">
-        <v>800</v>
-      </c>
-      <c r="F93" s="8"/>
-    </row>
-    <row r="94" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A94" s="34" t="s">
-        <v>801</v>
-      </c>
-      <c r="B94" s="34" t="s">
-        <v>802</v>
-      </c>
-      <c r="C94" s="34" t="s">
-        <v>797</v>
-      </c>
-      <c r="D94" s="34"/>
-      <c r="E94" s="34" t="s">
-        <v>800</v>
-      </c>
-      <c r="F94" s="8"/>
-    </row>
-    <row r="95" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A95" s="34" t="s">
-        <v>803</v>
-      </c>
-      <c r="B95" s="34" t="s">
-        <v>804</v>
-      </c>
-      <c r="C95" s="34" t="s">
-        <v>797</v>
-      </c>
-      <c r="D95" s="34"/>
-      <c r="E95" s="34" t="s">
-        <v>800</v>
-      </c>
-      <c r="F95" s="8"/>
-    </row>
-    <row r="96" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A96" s="34" t="s">
-        <v>805</v>
-      </c>
-      <c r="B96" s="34" t="s">
-        <v>806</v>
-      </c>
-      <c r="C96" s="34" t="s">
-        <v>797</v>
-      </c>
-      <c r="D96" s="34"/>
-      <c r="E96" s="34" t="s">
-        <v>807</v>
-      </c>
-      <c r="F96" s="8"/>
-    </row>
-    <row r="97" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A97" s="34" t="s">
-        <v>808</v>
-      </c>
-      <c r="B97" s="34" t="s">
-        <v>809</v>
-      </c>
-      <c r="C97" s="34" t="s">
-        <v>797</v>
-      </c>
-      <c r="D97" s="34"/>
-      <c r="E97" s="34" t="s">
-        <v>807</v>
-      </c>
-      <c r="F97" s="8"/>
-    </row>
-    <row r="98" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A98" s="34" t="s">
-        <v>810</v>
-      </c>
-      <c r="B98" s="34" t="s">
-        <v>811</v>
-      </c>
-      <c r="C98" s="34" t="s">
-        <v>797</v>
-      </c>
-      <c r="D98" s="34"/>
-      <c r="E98" s="34" t="s">
-        <v>807</v>
-      </c>
-      <c r="F98" s="8"/>
-    </row>
-    <row r="99" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A99" s="34" t="s">
-        <v>812</v>
-      </c>
-      <c r="B99" s="34" t="s">
-        <v>813</v>
-      </c>
-      <c r="C99" s="34" t="s">
-        <v>797</v>
-      </c>
-      <c r="D99" s="34"/>
-      <c r="E99" s="34" t="s">
-        <v>814</v>
-      </c>
-      <c r="F99" s="8"/>
-    </row>
-    <row r="100" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A100" s="34" t="s">
-        <v>815</v>
-      </c>
-      <c r="B100" s="34" t="s">
-        <v>816</v>
-      </c>
-      <c r="C100" s="34" t="s">
-        <v>797</v>
-      </c>
-      <c r="D100" s="34"/>
-      <c r="E100" s="34" t="s">
-        <v>814</v>
-      </c>
-      <c r="F100" s="8"/>
-    </row>
-    <row r="101" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A101" s="34" t="s">
-        <v>817</v>
-      </c>
-      <c r="B101" s="34" t="s">
-        <v>818</v>
-      </c>
-      <c r="C101" s="34" t="s">
-        <v>797</v>
-      </c>
-      <c r="D101" s="34"/>
-      <c r="E101" s="34" t="s">
-        <v>814</v>
-      </c>
-      <c r="F101" s="8"/>
-    </row>
-    <row r="102" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A102" s="34" t="s">
-        <v>819</v>
-      </c>
-      <c r="B102" s="37" t="s">
-        <v>820</v>
-      </c>
-      <c r="C102" s="34" t="s">
-        <v>797</v>
-      </c>
-      <c r="D102" s="34"/>
-      <c r="E102" s="34" t="s">
-        <v>814</v>
-      </c>
-      <c r="F102" s="8"/>
-    </row>
-    <row r="103" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A103" s="34" t="s">
-        <v>821</v>
-      </c>
-      <c r="B103" s="34" t="s">
-        <v>822</v>
-      </c>
-      <c r="C103" s="34" t="s">
-        <v>823</v>
-      </c>
-      <c r="D103" s="34"/>
-      <c r="E103" s="34" t="s">
-        <v>824</v>
-      </c>
-      <c r="F103" s="8"/>
-    </row>
-    <row r="104" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A104" s="34" t="s">
-        <v>825</v>
-      </c>
-      <c r="B104" s="34" t="s">
-        <v>826</v>
-      </c>
-      <c r="C104" s="34" t="s">
-        <v>823</v>
-      </c>
-      <c r="D104" s="34"/>
-      <c r="E104" s="34" t="s">
-        <v>824</v>
-      </c>
-      <c r="F104" s="8"/>
-    </row>
-    <row r="105" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A105" s="34" t="s">
-        <v>421</v>
-      </c>
-      <c r="B105" s="34" t="s">
-        <v>424</v>
-      </c>
-      <c r="C105" s="34" t="s">
-        <v>427</v>
-      </c>
-      <c r="D105" s="34"/>
-      <c r="E105" s="34" t="s">
-        <v>430</v>
-      </c>
-      <c r="F105" s="8"/>
-    </row>
-    <row r="106" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A106" s="34" t="s">
-        <v>422</v>
-      </c>
-      <c r="B106" s="37" t="s">
-        <v>425</v>
-      </c>
-      <c r="C106" s="34" t="s">
-        <v>427</v>
-      </c>
-      <c r="D106" s="34"/>
-      <c r="E106" s="34" t="s">
-        <v>430</v>
-      </c>
-      <c r="F106" s="8"/>
-    </row>
-    <row r="107" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A107" s="34" t="s">
-        <v>423</v>
-      </c>
-      <c r="B107" s="34" t="s">
-        <v>426</v>
-      </c>
-      <c r="C107" s="34" t="s">
-        <v>427</v>
-      </c>
-      <c r="D107" s="34"/>
-      <c r="E107" s="34" t="s">
-        <v>430</v>
-      </c>
-      <c r="F107" s="8"/>
-    </row>
-    <row r="108" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A108" s="34" t="s">
-        <v>428</v>
-      </c>
-      <c r="B108" s="34" t="s">
-        <v>429</v>
-      </c>
-      <c r="C108" s="34" t="s">
-        <v>432</v>
-      </c>
-      <c r="D108" s="34"/>
-      <c r="E108" s="34" t="s">
-        <v>431</v>
-      </c>
-      <c r="F108" s="8"/>
-    </row>
-    <row r="109" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A109" s="34" t="s">
-        <v>433</v>
-      </c>
-      <c r="B109" s="34" t="s">
-        <v>434</v>
-      </c>
-      <c r="C109" s="34" t="s">
-        <v>432</v>
-      </c>
-      <c r="D109" s="34"/>
-      <c r="E109" s="34" t="s">
-        <v>435</v>
-      </c>
-      <c r="F109" s="8"/>
-    </row>
-    <row r="110" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A110" s="34" t="s">
-        <v>827</v>
-      </c>
-      <c r="B110" s="37" t="s">
-        <v>828</v>
-      </c>
-      <c r="C110" s="34" t="s">
-        <v>432</v>
-      </c>
-      <c r="D110" s="34"/>
-      <c r="E110" s="34" t="s">
-        <v>435</v>
-      </c>
-      <c r="F110" s="8"/>
-    </row>
-    <row r="111" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A111" s="34" t="s">
-        <v>438</v>
-      </c>
-      <c r="B111" s="34" t="s">
-        <v>436</v>
-      </c>
-      <c r="C111" s="34" t="s">
-        <v>437</v>
-      </c>
-      <c r="D111" s="34"/>
-      <c r="E111" s="34" t="s">
-        <v>439</v>
-      </c>
-      <c r="F111" s="8"/>
-    </row>
-    <row r="112" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A112" s="34" t="s">
-        <v>829</v>
-      </c>
-      <c r="B112" s="34" t="s">
-        <v>830</v>
-      </c>
-      <c r="C112" s="34" t="s">
-        <v>437</v>
-      </c>
-      <c r="D112" s="34"/>
-      <c r="E112" s="34" t="s">
-        <v>831</v>
-      </c>
-      <c r="F112" s="8"/>
-    </row>
-    <row r="113" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A113" s="34" t="s">
-        <v>832</v>
-      </c>
-      <c r="B113" s="34" t="s">
-        <v>833</v>
-      </c>
-      <c r="C113" s="34" t="s">
-        <v>437</v>
-      </c>
-      <c r="D113" s="34"/>
-      <c r="E113" s="34" t="s">
-        <v>831</v>
-      </c>
-      <c r="F113" s="8"/>
-    </row>
-    <row r="114" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A114" s="34" t="s">
-        <v>443</v>
-      </c>
-      <c r="B114" s="34" t="s">
-        <v>440</v>
-      </c>
-      <c r="C114" s="34" t="s">
-        <v>437</v>
-      </c>
-      <c r="D114" s="34"/>
-      <c r="E114" s="34" t="s">
-        <v>445</v>
-      </c>
-      <c r="F114" s="8"/>
-    </row>
-    <row r="115" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A115" s="34" t="s">
-        <v>834</v>
-      </c>
-      <c r="B115" s="34" t="s">
-        <v>835</v>
-      </c>
-      <c r="C115" s="34" t="s">
-        <v>437</v>
-      </c>
-      <c r="D115" s="34"/>
-      <c r="E115" s="34" t="s">
-        <v>445</v>
-      </c>
-      <c r="F115" s="8"/>
-    </row>
-    <row r="116" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A116" s="34" t="s">
-        <v>444</v>
-      </c>
-      <c r="B116" s="34" t="s">
-        <v>442</v>
-      </c>
-      <c r="C116" s="34" t="s">
-        <v>437</v>
-      </c>
-      <c r="D116" s="34"/>
-      <c r="E116" s="34" t="s">
-        <v>445</v>
-      </c>
-      <c r="F116" s="8"/>
-    </row>
-    <row r="117" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A117" s="34" t="s">
-        <v>473</v>
-      </c>
-      <c r="B117" s="34" t="s">
-        <v>441</v>
-      </c>
-      <c r="C117" s="34" t="s">
-        <v>437</v>
-      </c>
-      <c r="D117" s="34"/>
-      <c r="E117" s="34" t="s">
-        <v>445</v>
-      </c>
-      <c r="F117" s="8"/>
-    </row>
-    <row r="118" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A118" s="34" t="s">
-        <v>454</v>
-      </c>
-      <c r="B118" s="34" t="s">
-        <v>446</v>
-      </c>
-      <c r="C118" s="34" t="s">
-        <v>452</v>
-      </c>
-      <c r="D118" s="34" t="s">
-        <v>847</v>
-      </c>
-      <c r="E118" s="34" t="s">
-        <v>453</v>
-      </c>
-      <c r="F118" s="8"/>
-    </row>
-    <row r="119" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A119" s="34" t="s">
-        <v>455</v>
-      </c>
-      <c r="B119" s="34" t="s">
-        <v>447</v>
-      </c>
-      <c r="C119" s="34" t="s">
-        <v>452</v>
-      </c>
-      <c r="D119" s="34" t="s">
-        <v>847</v>
-      </c>
-      <c r="E119" s="34" t="s">
-        <v>453</v>
-      </c>
-      <c r="F119" s="8"/>
-    </row>
-    <row r="120" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A120" s="34" t="s">
-        <v>456</v>
-      </c>
-      <c r="B120" s="34" t="s">
-        <v>448</v>
-      </c>
-      <c r="C120" s="34" t="s">
-        <v>452</v>
-      </c>
-      <c r="D120" s="34" t="s">
-        <v>847</v>
-      </c>
-      <c r="E120" s="34" t="s">
-        <v>453</v>
-      </c>
-      <c r="F120" s="8"/>
-    </row>
-    <row r="121" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A121" s="34" t="s">
-        <v>457</v>
-      </c>
-      <c r="B121" s="34" t="s">
-        <v>449</v>
-      </c>
-      <c r="C121" s="34" t="s">
-        <v>452</v>
-      </c>
-      <c r="D121" s="34" t="s">
-        <v>847</v>
-      </c>
-      <c r="E121" s="34" t="s">
-        <v>453</v>
-      </c>
-      <c r="F121" s="8"/>
-    </row>
-    <row r="122" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A122" s="34" t="s">
-        <v>458</v>
-      </c>
-      <c r="B122" s="34" t="s">
-        <v>450</v>
-      </c>
-      <c r="C122" s="34" t="s">
-        <v>452</v>
-      </c>
-      <c r="D122" s="34" t="s">
-        <v>847</v>
-      </c>
-      <c r="E122" s="34" t="s">
-        <v>453</v>
-      </c>
-      <c r="F122" s="8"/>
-    </row>
-    <row r="123" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A123" s="34" t="s">
-        <v>459</v>
-      </c>
-      <c r="B123" s="34" t="s">
-        <v>451</v>
-      </c>
-      <c r="C123" s="34" t="s">
-        <v>452</v>
-      </c>
-      <c r="D123" s="34" t="s">
-        <v>847</v>
-      </c>
-      <c r="E123" s="34" t="s">
-        <v>453</v>
-      </c>
-      <c r="F123" s="8"/>
-    </row>
-    <row r="124" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A124" s="34" t="s">
-        <v>463</v>
-      </c>
-      <c r="B124" s="34" t="s">
-        <v>460</v>
-      </c>
-      <c r="C124" s="34" t="s">
-        <v>462</v>
-      </c>
-      <c r="D124" s="34" t="s">
-        <v>847</v>
-      </c>
-      <c r="E124" s="34" t="s">
-        <v>465</v>
-      </c>
-      <c r="F124" s="8"/>
-    </row>
-    <row r="125" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A125" s="34" t="s">
-        <v>464</v>
-      </c>
-      <c r="B125" s="37" t="s">
-        <v>461</v>
-      </c>
-      <c r="C125" s="34" t="s">
-        <v>462</v>
-      </c>
-      <c r="D125" s="34" t="s">
-        <v>847</v>
-      </c>
-      <c r="E125" s="34" t="s">
-        <v>465</v>
-      </c>
-      <c r="F125" s="8"/>
-    </row>
-    <row r="126" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A126" s="34" t="s">
-        <v>469</v>
-      </c>
-      <c r="B126" s="34" t="s">
-        <v>466</v>
-      </c>
-      <c r="C126" s="34" t="s">
-        <v>468</v>
-      </c>
-      <c r="D126" s="34"/>
-      <c r="E126" s="34" t="s">
-        <v>471</v>
-      </c>
-      <c r="F126" s="8"/>
-    </row>
-    <row r="127" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A127" s="34" t="s">
-        <v>470</v>
-      </c>
-      <c r="B127" s="34" t="s">
-        <v>467</v>
-      </c>
-      <c r="C127" s="34" t="s">
-        <v>468</v>
-      </c>
-      <c r="D127" s="34"/>
-      <c r="E127" s="34" t="s">
-        <v>471</v>
-      </c>
-      <c r="F127" s="8"/>
-    </row>
-    <row r="128" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A128" s="34" t="s">
-        <v>836</v>
-      </c>
-      <c r="B128" s="34" t="s">
-        <v>837</v>
-      </c>
-      <c r="C128" s="34" t="s">
-        <v>838</v>
-      </c>
-      <c r="D128" s="34"/>
-      <c r="E128" s="34" t="s">
-        <v>839</v>
-      </c>
-      <c r="F128" s="8"/>
-    </row>
-    <row r="129" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A129" s="34" t="s">
-        <v>840</v>
-      </c>
-      <c r="B129" s="34" t="s">
-        <v>841</v>
-      </c>
-      <c r="C129" s="34" t="s">
-        <v>838</v>
-      </c>
-      <c r="D129" s="34"/>
-      <c r="E129" s="34" t="s">
-        <v>839</v>
-      </c>
-      <c r="F129" s="8"/>
-    </row>
-    <row r="130" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A130" s="34" t="s">
-        <v>842</v>
-      </c>
-      <c r="B130" s="34" t="s">
-        <v>843</v>
-      </c>
-      <c r="C130" s="34" t="s">
-        <v>838</v>
-      </c>
-      <c r="D130" s="34"/>
-      <c r="E130" s="34" t="s">
-        <v>844</v>
-      </c>
-      <c r="F130" s="8"/>
-    </row>
-    <row r="131" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A131" s="34" t="s">
-        <v>845</v>
-      </c>
-      <c r="B131" s="34" t="s">
-        <v>846</v>
-      </c>
-      <c r="C131" s="34" t="s">
-        <v>838</v>
-      </c>
-      <c r="D131" s="34"/>
-      <c r="E131" s="34" t="s">
-        <v>844</v>
-      </c>
-      <c r="F131" s="8"/>
-    </row>
-    <row r="132" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A132" s="32"/>
-      <c r="B132" s="32"/>
-      <c r="C132" s="32"/>
-      <c r="D132" s="32"/>
-      <c r="E132" s="32"/>
-      <c r="F132" s="8"/>
-    </row>
-    <row r="133" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A133" s="32"/>
-      <c r="B133" s="32"/>
-      <c r="C133" s="32"/>
-      <c r="D133" s="32"/>
-      <c r="E133" s="32"/>
-      <c r="F133" s="8"/>
-    </row>
-    <row r="134" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A134" s="32"/>
-      <c r="B134" s="32"/>
-      <c r="C134" s="32"/>
-      <c r="D134" s="32"/>
-      <c r="E134" s="32"/>
-      <c r="F134" s="8"/>
-    </row>
-    <row r="135" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A135" s="32"/>
-      <c r="B135" s="32"/>
-      <c r="C135" s="32"/>
-      <c r="D135" s="33"/>
-      <c r="E135" s="32"/>
-      <c r="F135" s="8"/>
-    </row>
-    <row r="136" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A136" s="32"/>
-      <c r="B136" s="32"/>
-      <c r="C136" s="32"/>
-      <c r="D136" s="32"/>
-      <c r="E136" s="32"/>
-      <c r="F136" s="8"/>
-    </row>
-    <row r="137" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A137" s="32"/>
-      <c r="B137" s="32"/>
-      <c r="C137" s="32"/>
-      <c r="D137" s="32"/>
-      <c r="E137" s="32"/>
-      <c r="F137" s="8"/>
-    </row>
-    <row r="138" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A138" s="32"/>
-      <c r="B138" s="32"/>
-      <c r="C138" s="32"/>
-      <c r="D138" s="32"/>
-      <c r="E138" s="32"/>
-      <c r="F138" s="8"/>
-    </row>
-    <row r="139" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A139" s="32"/>
-      <c r="B139" s="32"/>
-      <c r="C139" s="32"/>
-      <c r="D139" s="32"/>
-      <c r="E139" s="32"/>
-      <c r="F139" s="8"/>
-    </row>
-    <row r="140" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A140" s="32"/>
-      <c r="B140" s="32"/>
-      <c r="C140" s="32"/>
-      <c r="D140" s="32"/>
-      <c r="E140" s="32"/>
-      <c r="F140" s="8"/>
-    </row>
-    <row r="141" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A141" s="32"/>
-      <c r="B141" s="32"/>
-      <c r="C141" s="32"/>
-      <c r="D141" s="32"/>
-      <c r="E141" s="32"/>
-      <c r="F141" s="8"/>
-    </row>
-    <row r="142" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A142" s="32"/>
-      <c r="B142" s="32"/>
-      <c r="C142" s="32"/>
-      <c r="D142" s="32"/>
-      <c r="E142" s="32"/>
-      <c r="F142" s="8"/>
-    </row>
-    <row r="143" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A143" s="32"/>
-      <c r="B143" s="33"/>
-      <c r="C143" s="32"/>
-      <c r="D143" s="32"/>
-      <c r="E143" s="32"/>
-      <c r="F143" s="8"/>
-    </row>
-    <row r="144" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A144" s="1"/>
-      <c r="B144" s="1"/>
-      <c r="C144" s="1"/>
-      <c r="D144" s="1"/>
-      <c r="E144" s="1"/>
-      <c r="F144" s="8"/>
-    </row>
-    <row r="145" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A145" s="25" t="s">
-        <v>776</v>
-      </c>
-      <c r="B145" s="25"/>
-      <c r="C145" s="25"/>
-      <c r="D145" s="25"/>
-      <c r="E145" s="25"/>
-      <c r="F145" s="25"/>
-      <c r="G145" s="25"/>
-      <c r="H145" s="25"/>
-      <c r="I145" s="25"/>
-      <c r="J145" s="25"/>
-      <c r="K145" s="25"/>
-    </row>
-    <row r="146" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A146" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="B146" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="C146" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="D146" s="2" t="s">
-        <v>116</v>
-      </c>
-      <c r="E146" s="2" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="147" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A147" s="9" t="s">
+    <row r="125" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A125" s="9" t="s">
         <v>474</v>
       </c>
-      <c r="B147" s="1"/>
-      <c r="C147" s="1"/>
-      <c r="D147" s="1" t="s">
+      <c r="B125" s="1"/>
+      <c r="C125" s="1"/>
+      <c r="D125" s="1" t="s">
         <v>777</v>
       </c>
-      <c r="E147" s="1"/>
-    </row>
-    <row r="148" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A148" s="1"/>
-      <c r="B148" s="1"/>
-      <c r="C148" s="1"/>
-      <c r="D148" s="1"/>
-      <c r="E148" s="1"/>
-    </row>
-    <row r="149" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A149" s="1"/>
-      <c r="B149" s="1"/>
-      <c r="C149" s="1"/>
-      <c r="D149" s="1"/>
-      <c r="E149" s="1"/>
-    </row>
-    <row r="150" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A150" s="1"/>
-      <c r="B150" s="1"/>
-      <c r="C150" s="1"/>
-      <c r="D150" s="1"/>
-      <c r="E150" s="1"/>
-    </row>
-    <row r="151" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A151" s="1"/>
-      <c r="B151" s="1"/>
-      <c r="C151" s="1"/>
-      <c r="D151" s="1"/>
-      <c r="E151" s="1"/>
-    </row>
-    <row r="152" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A152" s="1"/>
-      <c r="B152" s="1"/>
-      <c r="C152" s="1"/>
-      <c r="D152" s="1"/>
-      <c r="E152" s="1"/>
-    </row>
-    <row r="153" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A153" s="1"/>
-      <c r="B153" s="1"/>
-      <c r="C153" s="1"/>
-      <c r="D153" s="1"/>
-      <c r="E153" s="1"/>
-    </row>
-    <row r="154" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A154" s="1"/>
-      <c r="B154" s="1"/>
-      <c r="C154" s="1"/>
-      <c r="D154" s="1"/>
-      <c r="E154" s="1"/>
+      <c r="E125" s="1"/>
+    </row>
+    <row r="126" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A126" s="1"/>
+      <c r="B126" s="1"/>
+      <c r="C126" s="1"/>
+      <c r="D126" s="1"/>
+      <c r="E126" s="1"/>
+    </row>
+    <row r="127" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A127" s="1"/>
+      <c r="B127" s="1"/>
+      <c r="C127" s="1"/>
+      <c r="D127" s="1"/>
+      <c r="E127" s="1"/>
+    </row>
+    <row r="128" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A128" s="1"/>
+      <c r="B128" s="1"/>
+      <c r="C128" s="1"/>
+      <c r="D128" s="1"/>
+      <c r="E128" s="1"/>
+    </row>
+    <row r="129" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A129" s="1"/>
+      <c r="B129" s="1"/>
+      <c r="C129" s="1"/>
+      <c r="D129" s="1"/>
+      <c r="E129" s="1"/>
+    </row>
+    <row r="130" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A130" s="1"/>
+      <c r="B130" s="1"/>
+      <c r="C130" s="1"/>
+      <c r="D130" s="1"/>
+      <c r="E130" s="1"/>
+    </row>
+    <row r="131" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A131" s="1"/>
+      <c r="B131" s="1"/>
+      <c r="C131" s="1"/>
+      <c r="D131" s="1"/>
+      <c r="E131" s="1"/>
+    </row>
+    <row r="132" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A132" s="1"/>
+      <c r="B132" s="1"/>
+      <c r="C132" s="1"/>
+      <c r="D132" s="1"/>
+      <c r="E132" s="1"/>
     </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A1:K1"/>
-    <mergeCell ref="A72:K72"/>
-    <mergeCell ref="A145:K145"/>
+    <mergeCell ref="A62:K62"/>
+    <mergeCell ref="A123:K123"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -9076,19 +8898,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A1" s="26" t="s">
+      <c r="A1" s="28" t="s">
         <v>111</v>
       </c>
-      <c r="B1" s="26"/>
-      <c r="C1" s="26"/>
-      <c r="D1" s="26"/>
-      <c r="E1" s="26"/>
-      <c r="F1" s="26"/>
-      <c r="G1" s="26"/>
-      <c r="H1" s="26"/>
-      <c r="I1" s="26"/>
-      <c r="J1" s="26"/>
-      <c r="K1" s="26"/>
+      <c r="B1" s="28"/>
+      <c r="C1" s="28"/>
+      <c r="D1" s="28"/>
+      <c r="E1" s="28"/>
+      <c r="F1" s="28"/>
+      <c r="G1" s="28"/>
+      <c r="H1" s="28"/>
+      <c r="I1" s="28"/>
+      <c r="J1" s="28"/>
+      <c r="K1" s="28"/>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
@@ -9129,19 +8951,19 @@
       <c r="E5" s="1"/>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A6" s="27" t="s">
+      <c r="A6" s="29" t="s">
         <v>112</v>
       </c>
-      <c r="B6" s="27"/>
-      <c r="C6" s="27"/>
-      <c r="D6" s="27"/>
-      <c r="E6" s="27"/>
-      <c r="F6" s="27"/>
-      <c r="G6" s="27"/>
-      <c r="H6" s="27"/>
-      <c r="I6" s="27"/>
-      <c r="J6" s="27"/>
-      <c r="K6" s="27"/>
+      <c r="B6" s="29"/>
+      <c r="C6" s="29"/>
+      <c r="D6" s="29"/>
+      <c r="E6" s="29"/>
+      <c r="F6" s="29"/>
+      <c r="G6" s="29"/>
+      <c r="H6" s="29"/>
+      <c r="I6" s="29"/>
+      <c r="J6" s="29"/>
+      <c r="K6" s="29"/>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
@@ -9269,19 +9091,19 @@
       <c r="E15" s="1"/>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A16" s="27" t="s">
+      <c r="A16" s="29" t="s">
         <v>776</v>
       </c>
-      <c r="B16" s="27"/>
-      <c r="C16" s="27"/>
-      <c r="D16" s="27"/>
-      <c r="E16" s="27"/>
-      <c r="F16" s="27"/>
-      <c r="G16" s="27"/>
-      <c r="H16" s="27"/>
-      <c r="I16" s="27"/>
-      <c r="J16" s="27"/>
-      <c r="K16" s="27"/>
+      <c r="B16" s="29"/>
+      <c r="C16" s="29"/>
+      <c r="D16" s="29"/>
+      <c r="E16" s="29"/>
+      <c r="F16" s="29"/>
+      <c r="G16" s="29"/>
+      <c r="H16" s="29"/>
+      <c r="I16" s="29"/>
+      <c r="J16" s="29"/>
+      <c r="K16" s="29"/>
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
@@ -9609,19 +9431,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A1" s="28" t="s">
+      <c r="A1" s="30" t="s">
         <v>111</v>
       </c>
-      <c r="B1" s="28"/>
-      <c r="C1" s="28"/>
-      <c r="D1" s="28"/>
-      <c r="E1" s="28"/>
-      <c r="F1" s="28"/>
-      <c r="G1" s="28"/>
-      <c r="H1" s="28"/>
-      <c r="I1" s="28"/>
-      <c r="J1" s="28"/>
-      <c r="K1" s="28"/>
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
+      <c r="F1" s="30"/>
+      <c r="G1" s="30"/>
+      <c r="H1" s="30"/>
+      <c r="I1" s="30"/>
+      <c r="J1" s="30"/>
+      <c r="K1" s="30"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
@@ -9662,19 +9484,19 @@
       <c r="E5" s="1"/>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A6" s="29" t="s">
+      <c r="A6" s="31" t="s">
         <v>112</v>
       </c>
-      <c r="B6" s="29"/>
-      <c r="C6" s="29"/>
-      <c r="D6" s="29"/>
-      <c r="E6" s="29"/>
-      <c r="F6" s="29"/>
-      <c r="G6" s="29"/>
-      <c r="H6" s="29"/>
-      <c r="I6" s="29"/>
-      <c r="J6" s="29"/>
-      <c r="K6" s="29"/>
+      <c r="B6" s="31"/>
+      <c r="C6" s="31"/>
+      <c r="D6" s="31"/>
+      <c r="E6" s="31"/>
+      <c r="F6" s="31"/>
+      <c r="G6" s="31"/>
+      <c r="H6" s="31"/>
+      <c r="I6" s="31"/>
+      <c r="J6" s="31"/>
+      <c r="K6" s="31"/>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
@@ -10234,19 +10056,19 @@
       </c>
     </row>
     <row r="42" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A42" s="29" t="s">
+      <c r="A42" s="31" t="s">
         <v>776</v>
       </c>
-      <c r="B42" s="29"/>
-      <c r="C42" s="29"/>
-      <c r="D42" s="29"/>
-      <c r="E42" s="29"/>
-      <c r="F42" s="29"/>
-      <c r="G42" s="29"/>
-      <c r="H42" s="29"/>
-      <c r="I42" s="29"/>
-      <c r="J42" s="29"/>
-      <c r="K42" s="29"/>
+      <c r="B42" s="31"/>
+      <c r="C42" s="31"/>
+      <c r="D42" s="31"/>
+      <c r="E42" s="31"/>
+      <c r="F42" s="31"/>
+      <c r="G42" s="31"/>
+      <c r="H42" s="31"/>
+      <c r="I42" s="31"/>
+      <c r="J42" s="31"/>
+      <c r="K42" s="31"/>
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A43" s="2" t="s">
@@ -10311,19 +10133,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A1" s="30" t="s">
+      <c r="A1" s="32" t="s">
         <v>111</v>
       </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="30"/>
-      <c r="D1" s="30"/>
-      <c r="E1" s="30"/>
-      <c r="F1" s="30"/>
-      <c r="G1" s="30"/>
-      <c r="H1" s="30"/>
-      <c r="I1" s="30"/>
-      <c r="J1" s="30"/>
-      <c r="K1" s="30"/>
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
+      <c r="E1" s="32"/>
+      <c r="F1" s="32"/>
+      <c r="G1" s="32"/>
+      <c r="H1" s="32"/>
+      <c r="I1" s="32"/>
+      <c r="J1" s="32"/>
+      <c r="K1" s="32"/>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
@@ -10364,19 +10186,19 @@
       <c r="E5" s="1"/>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A6" s="31" t="s">
+      <c r="A6" s="33" t="s">
         <v>112</v>
       </c>
-      <c r="B6" s="31"/>
-      <c r="C6" s="31"/>
-      <c r="D6" s="31"/>
-      <c r="E6" s="31"/>
-      <c r="F6" s="31"/>
-      <c r="G6" s="31"/>
-      <c r="H6" s="31"/>
-      <c r="I6" s="31"/>
-      <c r="J6" s="31"/>
-      <c r="K6" s="31"/>
+      <c r="B6" s="33"/>
+      <c r="C6" s="33"/>
+      <c r="D6" s="33"/>
+      <c r="E6" s="33"/>
+      <c r="F6" s="33"/>
+      <c r="G6" s="33"/>
+      <c r="H6" s="33"/>
+      <c r="I6" s="33"/>
+      <c r="J6" s="33"/>
+      <c r="K6" s="33"/>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
@@ -10417,19 +10239,19 @@
       <c r="E10" s="1"/>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A11" s="31" t="s">
+      <c r="A11" s="33" t="s">
         <v>776</v>
       </c>
-      <c r="B11" s="31"/>
-      <c r="C11" s="31"/>
-      <c r="D11" s="31"/>
-      <c r="E11" s="31"/>
-      <c r="F11" s="31"/>
-      <c r="G11" s="31"/>
-      <c r="H11" s="31"/>
-      <c r="I11" s="31"/>
-      <c r="J11" s="31"/>
-      <c r="K11" s="31"/>
+      <c r="B11" s="33"/>
+      <c r="C11" s="33"/>
+      <c r="D11" s="33"/>
+      <c r="E11" s="33"/>
+      <c r="F11" s="33"/>
+      <c r="G11" s="33"/>
+      <c r="H11" s="33"/>
+      <c r="I11" s="33"/>
+      <c r="J11" s="33"/>
+      <c r="K11" s="33"/>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">

</xml_diff>

<commit_message>
changes to unlisted proc specialty assignation, and removal of non-cancer tonsillectomies from data. update downloadable codes and phasing tables
</commit_message>
<xml_diff>
--- a/04_reports/management_report/serverless_html/resources/SRASA procedure codes and phasing.xlsx
+++ b/04_reports/management_report/serverless_html/resources/SRASA procedure codes and phasing.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\stats\quality\srasa\(11) Scripts\Bex\snap-srasa\04_reports\management_report\serverless_html\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06063F71-934A-417A-BD71-B137E7F2CFB0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F75EA337-FAE8-4086-A0FF-FBD23FC898D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="4" xr2:uid="{1A0DCE31-DBDB-4A7A-8FC4-F05F39A42CDB}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="3" xr2:uid="{1A0DCE31-DBDB-4A7A-8FC4-F05F39A42CDB}"/>
   </bookViews>
   <sheets>
     <sheet name="Colorectal" sheetId="2" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1878" uniqueCount="856">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1835" uniqueCount="852">
   <si>
     <t>M61 Open excision of prostate</t>
   </si>
@@ -1467,9 +1467,6 @@
     <t>F325</t>
   </si>
   <si>
-    <t>Any rule-of thumb exclusions e.g. paediatric tonsillectomies/adenoidectomies?</t>
-  </si>
-  <si>
     <t>H04</t>
   </si>
   <si>
@@ -2364,9 +2361,6 @@
     <t>M65</t>
   </si>
   <si>
-    <t>With benign neoplasm diagnosis OR anything excluding routine tonsillitis etc OR just the absence of cancer code (can be applied to over 16s only)</t>
-  </si>
-  <si>
     <t>should it just be cancer??</t>
   </si>
   <si>
@@ -2376,9 +2370,6 @@
     <t>Other</t>
   </si>
   <si>
-    <t>Exclude tonsillectomies for non-cancer cases</t>
-  </si>
-  <si>
     <t>E191</t>
   </si>
   <si>
@@ -2608,9 +2599,6 @@
   </si>
   <si>
     <t>Prostatectomy/TURPS</t>
-  </si>
-  <si>
-    <t>REMOVE benign tonsillectomies - TBD</t>
   </si>
 </sst>
 </file>
@@ -2792,7 +2780,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
@@ -2804,7 +2792,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
@@ -2815,6 +2802,9 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -2861,6 +2851,11 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -3444,8 +3439,8 @@
       <c r="E3" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="G3" s="15" t="s">
-        <v>774</v>
+      <c r="G3" s="14" t="s">
+        <v>772</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.3">
@@ -3462,8 +3457,8 @@
       <c r="E4" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="G4" s="15" t="s">
-        <v>775</v>
+      <c r="G4" s="14" t="s">
+        <v>773</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.3">
@@ -3558,124 +3553,124 @@
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="C11" s="1" t="s">
+        <v>503</v>
+      </c>
+      <c r="D11" s="6" t="s">
         <v>504</v>
       </c>
-      <c r="D11" s="6" t="s">
+      <c r="E11" s="1" t="s">
         <v>505</v>
-      </c>
-      <c r="E11" s="1" t="s">
-        <v>506</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="D12" s="1"/>
       <c r="E12" s="1" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="D13" s="1"/>
       <c r="E13" s="1" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="D14" s="1"/>
       <c r="E14" s="1" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="D15" s="1"/>
       <c r="E15" s="1" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="D16" s="1"/>
       <c r="E16" s="1" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="D17" s="1"/>
       <c r="E17" s="1" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="B18" s="1" t="s">
+        <v>502</v>
+      </c>
+      <c r="C18" s="1" t="s">
         <v>503</v>
-      </c>
-      <c r="C18" s="1" t="s">
-        <v>504</v>
       </c>
       <c r="D18" s="1"/>
       <c r="E18" s="1" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.3">
@@ -4094,7 +4089,7 @@
     </row>
     <row r="49" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A49" s="19" t="s">
-        <v>776</v>
+        <v>774</v>
       </c>
       <c r="B49" s="19"/>
       <c r="C49" s="19"/>
@@ -4151,7 +4146,7 @@
       <c r="C52" s="1" t="s">
         <v>172</v>
       </c>
-      <c r="D52" s="13" t="s">
+      <c r="D52" s="12" t="s">
         <v>193</v>
       </c>
       <c r="E52" s="1" t="s">
@@ -4230,7 +4225,7 @@
       <c r="C57" s="1" t="s">
         <v>182</v>
       </c>
-      <c r="D57" s="13" t="s">
+      <c r="D57" s="12" t="s">
         <v>193</v>
       </c>
       <c r="E57" s="1" t="s">
@@ -4339,7 +4334,7 @@
       <c r="C64" s="1" t="s">
         <v>191</v>
       </c>
-      <c r="D64" s="13" t="s">
+      <c r="D64" s="12" t="s">
         <v>193</v>
       </c>
       <c r="E64" s="1" t="s">
@@ -4438,79 +4433,79 @@
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A71" s="1" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="B71" s="1" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
       <c r="C71" s="1" t="s">
+        <v>485</v>
+      </c>
+      <c r="D71" s="6" t="s">
         <v>486</v>
       </c>
-      <c r="D71" s="6" t="s">
-        <v>487</v>
-      </c>
       <c r="E71" s="1" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A72" s="1" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="B72" s="1" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="C72" s="1" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="D72" s="1"/>
       <c r="E72" s="1" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A73" s="1" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="B73" s="1" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="C73" s="1" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="D73" s="1"/>
       <c r="E73" s="1" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A74" s="1" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="B74" s="1" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="C74" s="1" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="D74" s="1"/>
       <c r="E74" s="1" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A75" s="1" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="B75" s="1" t="s">
+        <v>484</v>
+      </c>
+      <c r="C75" s="1" t="s">
         <v>485</v>
-      </c>
-      <c r="C75" s="1" t="s">
-        <v>486</v>
       </c>
       <c r="D75" s="1"/>
       <c r="E75" s="1" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.3">
@@ -4639,7 +4634,7 @@
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B84" s="4" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
     </row>
   </sheetData>
@@ -5117,7 +5112,7 @@
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A30" s="1" t="s">
-        <v>769</v>
+        <v>768</v>
       </c>
       <c r="B30" s="1" t="s">
         <v>31</v>
@@ -5125,7 +5120,7 @@
       <c r="C30" s="1" t="s">
         <v>234</v>
       </c>
-      <c r="D30" s="12" t="s">
+      <c r="D30" s="11" t="s">
         <v>235</v>
       </c>
       <c r="E30" s="1" t="s">
@@ -5134,19 +5129,19 @@
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A31" s="1" t="s">
+        <v>769</v>
+      </c>
+      <c r="B31" s="1" t="s">
         <v>770</v>
       </c>
-      <c r="B31" s="1" t="s">
+      <c r="C31" s="1" t="s">
+        <v>851</v>
+      </c>
+      <c r="D31" s="1" t="s">
+        <v>845</v>
+      </c>
+      <c r="E31" s="1" t="s">
         <v>771</v>
-      </c>
-      <c r="C31" s="1" t="s">
-        <v>854</v>
-      </c>
-      <c r="D31" s="1" t="s">
-        <v>848</v>
-      </c>
-      <c r="E31" s="1" t="s">
-        <v>772</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.3">
@@ -5211,7 +5206,7 @@
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A38" s="21" t="s">
-        <v>776</v>
+        <v>774</v>
       </c>
       <c r="B38" s="21"/>
       <c r="C38" s="21"/>
@@ -5450,7 +5445,7 @@
       <c r="C11" s="1" t="s">
         <v>255</v>
       </c>
-      <c r="D11" s="14" t="s">
+      <c r="D11" s="13" t="s">
         <v>257</v>
       </c>
       <c r="E11" s="1" t="s">
@@ -5594,7 +5589,7 @@
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A25" s="23" t="s">
-        <v>776</v>
+        <v>774</v>
       </c>
       <c r="B25" s="23"/>
       <c r="C25" s="23"/>
@@ -5675,10 +5670,10 @@
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A30" s="1" t="s">
+        <v>507</v>
+      </c>
+      <c r="B30" s="1" t="s">
         <v>508</v>
-      </c>
-      <c r="B30" s="1" t="s">
-        <v>509</v>
       </c>
       <c r="C30" s="1"/>
       <c r="D30" s="1"/>
@@ -5768,185 +5763,185 @@
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>686</v>
+        <v>685</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>697</v>
+        <v>696</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>710</v>
+        <v>709</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>712</v>
-      </c>
-      <c r="F3" s="10" t="s">
-        <v>714</v>
+        <v>711</v>
+      </c>
+      <c r="F3" s="9" t="s">
+        <v>713</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>687</v>
+        <v>686</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>698</v>
+        <v>697</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>710</v>
+        <v>709</v>
       </c>
       <c r="D4" s="1"/>
       <c r="E4" s="1" t="s">
-        <v>712</v>
-      </c>
-      <c r="F4" s="11"/>
+        <v>711</v>
+      </c>
+      <c r="F4" s="10"/>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>710</v>
+        <v>709</v>
       </c>
       <c r="D5" s="1"/>
       <c r="E5" s="1" t="s">
-        <v>712</v>
-      </c>
-      <c r="F5" s="11"/>
+        <v>711</v>
+      </c>
+      <c r="F5" s="10"/>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>689</v>
+        <v>688</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>710</v>
+        <v>709</v>
       </c>
       <c r="D6" s="1"/>
       <c r="E6" s="1" t="s">
-        <v>712</v>
-      </c>
-      <c r="F6" s="11"/>
+        <v>711</v>
+      </c>
+      <c r="F6" s="10"/>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>690</v>
+        <v>689</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>701</v>
+        <v>700</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>710</v>
+        <v>709</v>
       </c>
       <c r="D7" s="1"/>
       <c r="E7" s="1" t="s">
-        <v>712</v>
-      </c>
-      <c r="F7" s="11"/>
+        <v>711</v>
+      </c>
+      <c r="F7" s="10"/>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
-        <v>691</v>
+        <v>690</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>702</v>
+        <v>701</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>710</v>
+        <v>709</v>
       </c>
       <c r="D8" s="1"/>
       <c r="E8" s="1" t="s">
-        <v>712</v>
-      </c>
-      <c r="F8" s="11"/>
+        <v>711</v>
+      </c>
+      <c r="F8" s="10"/>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
-        <v>692</v>
+        <v>691</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>703</v>
+        <v>702</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>711</v>
+        <v>710</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>713</v>
-      </c>
-      <c r="F9" s="11"/>
+        <v>712</v>
+      </c>
+      <c r="F9" s="10"/>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>704</v>
+        <v>703</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>711</v>
+        <v>710</v>
       </c>
       <c r="D10" s="1"/>
       <c r="E10" s="1" t="s">
-        <v>713</v>
-      </c>
-      <c r="F10" s="11"/>
+        <v>712</v>
+      </c>
+      <c r="F10" s="10"/>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>705</v>
+        <v>704</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>711</v>
+        <v>710</v>
       </c>
       <c r="D11" s="1"/>
       <c r="E11" s="1" t="s">
-        <v>713</v>
-      </c>
-      <c r="F11" s="11"/>
+        <v>712</v>
+      </c>
+      <c r="F11" s="10"/>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>706</v>
+        <v>705</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>711</v>
+        <v>710</v>
       </c>
       <c r="D12" s="1"/>
       <c r="E12" s="1" t="s">
-        <v>713</v>
-      </c>
-      <c r="F12" s="11"/>
+        <v>712</v>
+      </c>
+      <c r="F12" s="10"/>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
-        <v>696</v>
+        <v>695</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>707</v>
+        <v>706</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>711</v>
+        <v>710</v>
       </c>
       <c r="D13" s="1"/>
       <c r="E13" s="1" t="s">
-        <v>713</v>
-      </c>
-      <c r="F13" s="11"/>
+        <v>712</v>
+      </c>
+      <c r="F13" s="10"/>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A14" s="1"/>
@@ -5996,221 +5991,221 @@
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
-        <v>686</v>
+        <v>685</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>697</v>
+        <v>696</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>710</v>
+        <v>709</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>712</v>
-      </c>
-      <c r="F18" s="10" t="s">
-        <v>766</v>
+        <v>711</v>
+      </c>
+      <c r="F18" s="9" t="s">
+        <v>765</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
-        <v>687</v>
+        <v>686</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>698</v>
+        <v>697</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>710</v>
+        <v>709</v>
       </c>
       <c r="D19" s="1"/>
       <c r="E19" s="1" t="s">
-        <v>712</v>
-      </c>
-      <c r="F19" s="11"/>
+        <v>711</v>
+      </c>
+      <c r="F19" s="10"/>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>710</v>
+        <v>709</v>
       </c>
       <c r="D20" s="1"/>
       <c r="E20" s="1" t="s">
-        <v>712</v>
-      </c>
-      <c r="F20" s="11"/>
+        <v>711</v>
+      </c>
+      <c r="F20" s="10"/>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
-        <v>689</v>
+        <v>688</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>710</v>
+        <v>709</v>
       </c>
       <c r="D21" s="1"/>
       <c r="E21" s="1" t="s">
-        <v>712</v>
-      </c>
-      <c r="F21" s="11"/>
+        <v>711</v>
+      </c>
+      <c r="F21" s="10"/>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
+        <v>714</v>
+      </c>
+      <c r="B22" s="1" t="s">
         <v>715</v>
       </c>
-      <c r="B22" s="1" t="s">
-        <v>716</v>
-      </c>
       <c r="C22" s="1" t="s">
-        <v>710</v>
+        <v>709</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>712</v>
-      </c>
-      <c r="F22" s="11"/>
+        <v>711</v>
+      </c>
+      <c r="F22" s="10"/>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
-        <v>715</v>
+        <v>714</v>
       </c>
       <c r="B23" s="1" t="s">
+        <v>716</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>709</v>
+      </c>
+      <c r="D23" s="1" t="s">
         <v>717</v>
       </c>
-      <c r="C23" s="1" t="s">
-        <v>710</v>
-      </c>
-      <c r="D23" s="1" t="s">
-        <v>718</v>
-      </c>
       <c r="E23" s="1" t="s">
-        <v>712</v>
-      </c>
-      <c r="F23" s="11"/>
+        <v>711</v>
+      </c>
+      <c r="F23" s="10"/>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
-        <v>690</v>
+        <v>689</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>701</v>
+        <v>700</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>710</v>
+        <v>709</v>
       </c>
       <c r="D24" s="1"/>
       <c r="E24" s="1" t="s">
-        <v>712</v>
-      </c>
-      <c r="F24" s="11"/>
+        <v>711</v>
+      </c>
+      <c r="F24" s="10"/>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25" s="1" t="s">
-        <v>691</v>
+        <v>690</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>702</v>
+        <v>701</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>710</v>
+        <v>709</v>
       </c>
       <c r="D25" s="1"/>
       <c r="E25" s="1" t="s">
-        <v>712</v>
-      </c>
-      <c r="F25" s="11"/>
+        <v>711</v>
+      </c>
+      <c r="F25" s="10"/>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="s">
-        <v>692</v>
+        <v>691</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>703</v>
+        <v>702</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>711</v>
+        <v>710</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>713</v>
-      </c>
-      <c r="F26" s="11"/>
+        <v>712</v>
+      </c>
+      <c r="F26" s="10"/>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A27" s="1" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>704</v>
+        <v>703</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>711</v>
+        <v>710</v>
       </c>
       <c r="D27" s="1"/>
       <c r="E27" s="1" t="s">
-        <v>713</v>
-      </c>
-      <c r="F27" s="11"/>
+        <v>712</v>
+      </c>
+      <c r="F27" s="10"/>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A28" s="1" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>705</v>
+        <v>704</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>711</v>
+        <v>710</v>
       </c>
       <c r="D28" s="1"/>
       <c r="E28" s="1" t="s">
-        <v>713</v>
-      </c>
-      <c r="F28" s="11"/>
+        <v>712</v>
+      </c>
+      <c r="F28" s="10"/>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>706</v>
+        <v>705</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>711</v>
+        <v>710</v>
       </c>
       <c r="D29" s="1"/>
       <c r="E29" s="1" t="s">
-        <v>713</v>
-      </c>
-      <c r="F29" s="11"/>
+        <v>712</v>
+      </c>
+      <c r="F29" s="10"/>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A30" s="1" t="s">
-        <v>696</v>
+        <v>695</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>707</v>
+        <v>706</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>711</v>
+        <v>710</v>
       </c>
       <c r="D30" s="1"/>
       <c r="E30" s="1" t="s">
-        <v>713</v>
-      </c>
-      <c r="F30" s="11"/>
+        <v>712</v>
+      </c>
+      <c r="F30" s="10"/>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A31" s="1"/>
@@ -6228,7 +6223,7 @@
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A33" s="25" t="s">
-        <v>776</v>
+        <v>774</v>
       </c>
       <c r="B33" s="25"/>
       <c r="C33" s="25"/>
@@ -6260,539 +6255,539 @@
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A35" s="1" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>681</v>
+        <v>680</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>729</v>
+        <v>728</v>
       </c>
       <c r="D35" s="1" t="s">
+        <v>683</v>
+      </c>
+      <c r="E35" s="1" t="s">
         <v>684</v>
-      </c>
-      <c r="E35" s="1" t="s">
-        <v>685</v>
       </c>
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A36" s="1" t="s">
-        <v>679</v>
+        <v>678</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>729</v>
+        <v>728</v>
       </c>
       <c r="D36" s="1"/>
       <c r="E36" s="1" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A37" s="1" t="s">
-        <v>680</v>
+        <v>679</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>729</v>
+        <v>728</v>
       </c>
       <c r="D37" s="1"/>
       <c r="E37" s="1" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A38" s="1" t="s">
-        <v>724</v>
+        <v>723</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
       <c r="C38" s="1" t="s">
+        <v>728</v>
+      </c>
+      <c r="D38" s="1" t="s">
         <v>729</v>
       </c>
-      <c r="D38" s="1" t="s">
-        <v>730</v>
-      </c>
       <c r="E38" s="1" t="s">
-        <v>748</v>
+        <v>747</v>
       </c>
     </row>
     <row r="39" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A39" s="1" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>720</v>
+        <v>719</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>729</v>
+        <v>728</v>
       </c>
       <c r="D39" s="1"/>
       <c r="E39" s="1" t="s">
-        <v>748</v>
+        <v>747</v>
       </c>
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A40" s="1" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>729</v>
+        <v>728</v>
       </c>
       <c r="D40" s="1"/>
       <c r="E40" s="1" t="s">
-        <v>748</v>
+        <v>747</v>
       </c>
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A41" s="1" t="s">
-        <v>727</v>
+        <v>726</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>729</v>
+        <v>728</v>
       </c>
       <c r="D41" s="1"/>
       <c r="E41" s="1" t="s">
-        <v>748</v>
+        <v>747</v>
       </c>
     </row>
     <row r="42" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A42" s="1" t="s">
+        <v>727</v>
+      </c>
+      <c r="B42" s="1" t="s">
+        <v>722</v>
+      </c>
+      <c r="C42" s="1" t="s">
         <v>728</v>
-      </c>
-      <c r="B42" s="1" t="s">
-        <v>723</v>
-      </c>
-      <c r="C42" s="1" t="s">
-        <v>729</v>
       </c>
       <c r="D42" s="1"/>
       <c r="E42" s="1" t="s">
-        <v>748</v>
+        <v>747</v>
       </c>
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A43" s="1" t="s">
-        <v>740</v>
+        <v>739</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>731</v>
+        <v>730</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>729</v>
+        <v>728</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>739</v>
+        <v>738</v>
       </c>
       <c r="E43" s="1" t="s">
-        <v>749</v>
+        <v>748</v>
       </c>
     </row>
     <row r="44" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A44" s="1" t="s">
-        <v>741</v>
+        <v>740</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>732</v>
+        <v>731</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>729</v>
+        <v>728</v>
       </c>
       <c r="D44" s="1"/>
       <c r="E44" s="1" t="s">
-        <v>749</v>
+        <v>748</v>
       </c>
     </row>
     <row r="45" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A45" s="1" t="s">
-        <v>742</v>
+        <v>741</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>733</v>
+        <v>732</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>729</v>
+        <v>728</v>
       </c>
       <c r="D45" s="1"/>
       <c r="E45" s="1" t="s">
-        <v>749</v>
+        <v>748</v>
       </c>
     </row>
     <row r="46" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A46" s="1" t="s">
-        <v>743</v>
+        <v>742</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>734</v>
+        <v>733</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>729</v>
+        <v>728</v>
       </c>
       <c r="D46" s="1"/>
       <c r="E46" s="1" t="s">
-        <v>749</v>
+        <v>748</v>
       </c>
     </row>
     <row r="47" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A47" s="1" t="s">
-        <v>744</v>
+        <v>743</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>735</v>
+        <v>734</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>729</v>
+        <v>728</v>
       </c>
       <c r="D47" s="1"/>
       <c r="E47" s="1" t="s">
-        <v>749</v>
+        <v>748</v>
       </c>
     </row>
     <row r="48" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A48" s="1" t="s">
-        <v>745</v>
+        <v>744</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>729</v>
+        <v>728</v>
       </c>
       <c r="D48" s="1"/>
       <c r="E48" s="1" t="s">
-        <v>749</v>
+        <v>748</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A49" s="1" t="s">
-        <v>746</v>
+        <v>745</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>737</v>
+        <v>736</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>729</v>
+        <v>728</v>
       </c>
       <c r="D49" s="1"/>
       <c r="E49" s="1" t="s">
-        <v>749</v>
+        <v>748</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A50" s="1" t="s">
-        <v>747</v>
+        <v>746</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>738</v>
+        <v>737</v>
       </c>
       <c r="C50" s="1" t="s">
-        <v>729</v>
+        <v>728</v>
       </c>
       <c r="D50" s="1"/>
       <c r="E50" s="1" t="s">
-        <v>749</v>
+        <v>748</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A51" s="1" t="s">
-        <v>756</v>
+        <v>755</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>751</v>
+        <v>750</v>
       </c>
       <c r="C51" s="1" t="s">
-        <v>729</v>
+        <v>728</v>
       </c>
       <c r="D51" s="1" t="s">
-        <v>750</v>
+        <v>749</v>
       </c>
       <c r="E51" s="1" t="s">
-        <v>761</v>
+        <v>760</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A52" s="1" t="s">
-        <v>757</v>
+        <v>756</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>752</v>
+        <v>751</v>
       </c>
       <c r="C52" s="1" t="s">
-        <v>729</v>
+        <v>728</v>
       </c>
       <c r="D52" s="1"/>
       <c r="E52" s="1" t="s">
-        <v>761</v>
+        <v>760</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A53" s="1" t="s">
-        <v>758</v>
+        <v>757</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>753</v>
+        <v>752</v>
       </c>
       <c r="C53" s="1" t="s">
-        <v>729</v>
+        <v>728</v>
       </c>
       <c r="D53" s="1"/>
       <c r="E53" s="1" t="s">
-        <v>761</v>
+        <v>760</v>
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A54" s="1" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>754</v>
+        <v>753</v>
       </c>
       <c r="C54" s="1" t="s">
-        <v>729</v>
+        <v>728</v>
       </c>
       <c r="D54" s="1"/>
       <c r="E54" s="1" t="s">
-        <v>761</v>
+        <v>760</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A55" s="1" t="s">
-        <v>760</v>
+        <v>759</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>755</v>
+        <v>754</v>
       </c>
       <c r="C55" s="1" t="s">
-        <v>729</v>
+        <v>728</v>
       </c>
       <c r="D55" s="1"/>
       <c r="E55" s="1" t="s">
-        <v>761</v>
+        <v>760</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A56" s="1" t="s">
-        <v>686</v>
+        <v>685</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>697</v>
+        <v>696</v>
       </c>
       <c r="C56" s="1" t="s">
-        <v>710</v>
+        <v>709</v>
       </c>
       <c r="D56" s="1" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="E56" s="1" t="s">
-        <v>712</v>
-      </c>
-      <c r="F56" s="10" t="s">
-        <v>767</v>
+        <v>711</v>
+      </c>
+      <c r="F56" s="9" t="s">
+        <v>766</v>
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A57" s="1" t="s">
-        <v>687</v>
+        <v>686</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>698</v>
+        <v>697</v>
       </c>
       <c r="C57" s="1" t="s">
-        <v>710</v>
+        <v>709</v>
       </c>
       <c r="D57" s="1"/>
       <c r="E57" s="1" t="s">
-        <v>712</v>
-      </c>
-      <c r="F57" s="11"/>
+        <v>711</v>
+      </c>
+      <c r="F57" s="10"/>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A58" s="1" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
       <c r="C58" s="1" t="s">
-        <v>710</v>
+        <v>709</v>
       </c>
       <c r="D58" s="1"/>
       <c r="E58" s="1" t="s">
-        <v>712</v>
-      </c>
-      <c r="F58" s="11"/>
+        <v>711</v>
+      </c>
+      <c r="F58" s="10"/>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A59" s="1" t="s">
-        <v>689</v>
+        <v>688</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
       <c r="C59" s="1" t="s">
-        <v>710</v>
+        <v>709</v>
       </c>
       <c r="D59" s="1"/>
       <c r="E59" s="1" t="s">
-        <v>712</v>
-      </c>
-      <c r="F59" s="11"/>
+        <v>711</v>
+      </c>
+      <c r="F59" s="10"/>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A60" s="1" t="s">
-        <v>690</v>
+        <v>689</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>701</v>
+        <v>700</v>
       </c>
       <c r="C60" s="1" t="s">
-        <v>710</v>
+        <v>709</v>
       </c>
       <c r="D60" s="1"/>
       <c r="E60" s="1" t="s">
-        <v>712</v>
-      </c>
-      <c r="F60" s="11"/>
+        <v>711</v>
+      </c>
+      <c r="F60" s="10"/>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A61" s="1" t="s">
-        <v>691</v>
+        <v>690</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>702</v>
+        <v>701</v>
       </c>
       <c r="C61" s="1" t="s">
-        <v>710</v>
+        <v>709</v>
       </c>
       <c r="D61" s="1"/>
       <c r="E61" s="1" t="s">
-        <v>712</v>
-      </c>
-      <c r="F61" s="11"/>
+        <v>711</v>
+      </c>
+      <c r="F61" s="10"/>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A62" s="1" t="s">
-        <v>692</v>
+        <v>691</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>703</v>
+        <v>702</v>
       </c>
       <c r="C62" s="1" t="s">
-        <v>711</v>
+        <v>710</v>
       </c>
       <c r="D62" s="1" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
       <c r="E62" s="1" t="s">
-        <v>713</v>
-      </c>
-      <c r="F62" s="11"/>
+        <v>712</v>
+      </c>
+      <c r="F62" s="10"/>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A63" s="1" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>704</v>
+        <v>703</v>
       </c>
       <c r="C63" s="1" t="s">
-        <v>711</v>
+        <v>710</v>
       </c>
       <c r="D63" s="1"/>
       <c r="E63" s="1" t="s">
-        <v>713</v>
-      </c>
-      <c r="F63" s="11"/>
+        <v>712</v>
+      </c>
+      <c r="F63" s="10"/>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A64" s="1" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>705</v>
+        <v>704</v>
       </c>
       <c r="C64" s="1" t="s">
-        <v>711</v>
+        <v>710</v>
       </c>
       <c r="D64" s="1"/>
       <c r="E64" s="1" t="s">
-        <v>713</v>
-      </c>
-      <c r="F64" s="11"/>
+        <v>712</v>
+      </c>
+      <c r="F64" s="10"/>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A65" s="1" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>706</v>
+        <v>705</v>
       </c>
       <c r="C65" s="1" t="s">
-        <v>711</v>
+        <v>710</v>
       </c>
       <c r="D65" s="1"/>
       <c r="E65" s="1" t="s">
-        <v>713</v>
-      </c>
-      <c r="F65" s="11"/>
+        <v>712</v>
+      </c>
+      <c r="F65" s="10"/>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A66" s="1" t="s">
-        <v>696</v>
+        <v>695</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>707</v>
+        <v>706</v>
       </c>
       <c r="C66" s="1" t="s">
-        <v>711</v>
+        <v>710</v>
       </c>
       <c r="D66" s="1"/>
       <c r="E66" s="1" t="s">
-        <v>713</v>
-      </c>
-      <c r="F66" s="11"/>
+        <v>712</v>
+      </c>
+      <c r="F66" s="10"/>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B67" s="4" t="s">
-        <v>762</v>
+        <v>761</v>
       </c>
       <c r="D67" t="s">
-        <v>849</v>
+        <v>846</v>
       </c>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B68" s="4" t="s">
-        <v>763</v>
+        <v>762</v>
       </c>
       <c r="D68" t="s">
-        <v>850</v>
+        <v>847</v>
       </c>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B69" s="4" t="s">
-        <v>764</v>
+        <v>763</v>
       </c>
       <c r="D69" t="s">
-        <v>849</v>
+        <v>846</v>
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B70" s="4" t="s">
-        <v>765</v>
+        <v>764</v>
       </c>
       <c r="D70" t="s">
-        <v>849</v>
+        <v>846</v>
       </c>
     </row>
   </sheetData>
@@ -6808,7 +6803,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{40C4708D-51A9-4027-A13F-C06B96593285}">
-  <dimension ref="A1:K132"/>
+  <dimension ref="A1:L124"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.33203125" bestFit="1" customWidth="1"/>
@@ -6851,19 +6846,19 @@
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>778</v>
+        <v>775</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>779</v>
+        <v>776</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>780</v>
+        <v>777</v>
       </c>
       <c r="D3" s="1"/>
       <c r="E3" s="1" t="s">
         <v>399</v>
       </c>
-      <c r="F3" s="17" t="s">
+      <c r="F3" s="16" t="s">
         <v>415</v>
       </c>
     </row>
@@ -6871,11 +6866,11 @@
       <c r="A4" s="1" t="s">
         <v>393</v>
       </c>
-      <c r="B4" s="16" t="s">
+      <c r="B4" s="15" t="s">
         <v>396</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>780</v>
+        <v>777</v>
       </c>
       <c r="D4" s="1"/>
       <c r="E4" s="1" t="s">
@@ -6887,11 +6882,11 @@
       <c r="A5" s="1" t="s">
         <v>394</v>
       </c>
-      <c r="B5" s="16" t="s">
+      <c r="B5" s="15" t="s">
         <v>397</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>780</v>
+        <v>777</v>
       </c>
       <c r="D5" s="1"/>
       <c r="E5" s="1" t="s">
@@ -6903,14 +6898,14 @@
       <c r="A6" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="B6" s="16" t="s">
+      <c r="B6" s="15" t="s">
         <v>398</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>780</v>
+        <v>777</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>851</v>
+        <v>848</v>
       </c>
       <c r="E6" s="1" t="s">
         <v>399</v>
@@ -6921,7 +6916,7 @@
       <c r="A7" s="1" t="s">
         <v>406</v>
       </c>
-      <c r="B7" s="16" t="s">
+      <c r="B7" s="15" t="s">
         <v>400</v>
       </c>
       <c r="C7" s="1" t="s">
@@ -7015,10 +7010,10 @@
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
-        <v>781</v>
+        <v>778</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>782</v>
+        <v>779</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>412</v>
@@ -7063,289 +7058,289 @@
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
-        <v>783</v>
+        <v>780</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>784</v>
+        <v>781</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>785</v>
+        <v>782</v>
       </c>
       <c r="D16" s="1"/>
       <c r="E16" s="1" t="s">
-        <v>786</v>
+        <v>783</v>
       </c>
       <c r="F16" s="7"/>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
-        <v>787</v>
+        <v>784</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>788</v>
+        <v>785</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>785</v>
+        <v>782</v>
       </c>
       <c r="D17" s="1"/>
       <c r="E17" s="1" t="s">
-        <v>786</v>
+        <v>783</v>
       </c>
       <c r="F17" s="7"/>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
-        <v>789</v>
+        <v>786</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>790</v>
+        <v>787</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>785</v>
+        <v>782</v>
       </c>
       <c r="D18" s="1"/>
       <c r="E18" s="1" t="s">
-        <v>786</v>
+        <v>783</v>
       </c>
       <c r="F18" s="7"/>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
-        <v>791</v>
+        <v>788</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>792</v>
+        <v>789</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>785</v>
+        <v>782</v>
       </c>
       <c r="D19" s="1"/>
       <c r="E19" s="1" t="s">
-        <v>786</v>
+        <v>783</v>
       </c>
       <c r="F19" s="7"/>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
-        <v>793</v>
+        <v>790</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>794</v>
+        <v>791</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>785</v>
+        <v>782</v>
       </c>
       <c r="D20" s="1"/>
       <c r="E20" s="1" t="s">
-        <v>786</v>
+        <v>783</v>
       </c>
       <c r="F20" s="7"/>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
-        <v>795</v>
+        <v>792</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>796</v>
+        <v>793</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>797</v>
+        <v>794</v>
       </c>
       <c r="D21" s="1"/>
       <c r="E21" s="1" t="s">
-        <v>786</v>
+        <v>783</v>
       </c>
       <c r="F21" s="7"/>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
-        <v>798</v>
+        <v>795</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>799</v>
+        <v>796</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>797</v>
+        <v>794</v>
       </c>
       <c r="D22" s="1"/>
       <c r="E22" s="1" t="s">
-        <v>800</v>
+        <v>797</v>
       </c>
       <c r="F22" s="7"/>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
-        <v>801</v>
+        <v>798</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>802</v>
+        <v>799</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>797</v>
+        <v>794</v>
       </c>
       <c r="D23" s="1"/>
       <c r="E23" s="1" t="s">
-        <v>800</v>
+        <v>797</v>
       </c>
       <c r="F23" s="7"/>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
-        <v>803</v>
+        <v>800</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>804</v>
+        <v>801</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>797</v>
+        <v>794</v>
       </c>
       <c r="D24" s="1"/>
       <c r="E24" s="1" t="s">
-        <v>800</v>
+        <v>797</v>
       </c>
       <c r="F24" s="7"/>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25" s="1" t="s">
-        <v>805</v>
+        <v>802</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>806</v>
+        <v>803</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>797</v>
+        <v>794</v>
       </c>
       <c r="D25" s="1"/>
       <c r="E25" s="1" t="s">
-        <v>807</v>
+        <v>804</v>
       </c>
       <c r="F25" s="7"/>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="s">
-        <v>808</v>
+        <v>805</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>809</v>
+        <v>806</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>797</v>
+        <v>794</v>
       </c>
       <c r="D26" s="1"/>
       <c r="E26" s="1" t="s">
-        <v>807</v>
+        <v>804</v>
       </c>
       <c r="F26" s="7"/>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A27" s="1" t="s">
-        <v>810</v>
+        <v>807</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>811</v>
+        <v>808</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>797</v>
+        <v>794</v>
       </c>
       <c r="D27" s="1"/>
       <c r="E27" s="1" t="s">
-        <v>807</v>
+        <v>804</v>
       </c>
       <c r="F27" s="7"/>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A28" s="1" t="s">
-        <v>812</v>
+        <v>809</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>813</v>
+        <v>810</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>797</v>
+        <v>794</v>
       </c>
       <c r="D28" s="1"/>
       <c r="E28" s="1" t="s">
-        <v>814</v>
+        <v>811</v>
       </c>
       <c r="F28" s="7"/>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
-        <v>815</v>
+        <v>812</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>816</v>
+        <v>813</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>797</v>
+        <v>794</v>
       </c>
       <c r="D29" s="1"/>
       <c r="E29" s="1" t="s">
-        <v>814</v>
+        <v>811</v>
       </c>
       <c r="F29" s="7"/>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A30" s="1" t="s">
-        <v>817</v>
+        <v>814</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>818</v>
+        <v>815</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>797</v>
+        <v>794</v>
       </c>
       <c r="D30" s="1"/>
       <c r="E30" s="1" t="s">
-        <v>814</v>
+        <v>811</v>
       </c>
       <c r="F30" s="7"/>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A31" s="1" t="s">
-        <v>819</v>
+        <v>816</v>
       </c>
       <c r="B31" t="s">
-        <v>820</v>
+        <v>817</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>797</v>
+        <v>794</v>
       </c>
       <c r="D31" s="1"/>
       <c r="E31" s="1" t="s">
-        <v>814</v>
+        <v>811</v>
       </c>
       <c r="F31" s="7"/>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A32" s="1" t="s">
-        <v>821</v>
+        <v>818</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>822</v>
+        <v>819</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>823</v>
+        <v>820</v>
       </c>
       <c r="D32" s="1"/>
       <c r="E32" s="1" t="s">
-        <v>824</v>
+        <v>821</v>
       </c>
       <c r="F32" s="7"/>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A33" s="1" t="s">
-        <v>825</v>
+        <v>822</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>826</v>
+        <v>823</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>823</v>
+        <v>820</v>
       </c>
       <c r="D33" s="1"/>
       <c r="E33" s="1" t="s">
-        <v>824</v>
+        <v>821</v>
       </c>
       <c r="F33" s="7"/>
     </row>
@@ -7431,10 +7426,10 @@
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A39" s="1" t="s">
-        <v>827</v>
+        <v>824</v>
       </c>
       <c r="B39" t="s">
-        <v>828</v>
+        <v>825</v>
       </c>
       <c r="C39" s="1" t="s">
         <v>432</v>
@@ -7463,33 +7458,33 @@
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A41" s="1" t="s">
-        <v>829</v>
+        <v>826</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>830</v>
+        <v>827</v>
       </c>
       <c r="C41" s="1" t="s">
         <v>437</v>
       </c>
       <c r="D41" s="1"/>
       <c r="E41" s="1" t="s">
-        <v>831</v>
+        <v>828</v>
       </c>
       <c r="F41" s="7"/>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A42" s="1" t="s">
-        <v>832</v>
+        <v>829</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>833</v>
+        <v>830</v>
       </c>
       <c r="C42" s="1" t="s">
         <v>437</v>
       </c>
       <c r="D42" s="1"/>
       <c r="E42" s="1" t="s">
-        <v>831</v>
+        <v>828</v>
       </c>
       <c r="F42" s="7"/>
     </row>
@@ -7511,10 +7506,10 @@
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A44" s="1" t="s">
-        <v>834</v>
+        <v>831</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>835</v>
+        <v>832</v>
       </c>
       <c r="C44" s="1" t="s">
         <v>437</v>
@@ -7568,7 +7563,7 @@
         <v>452</v>
       </c>
       <c r="D47" s="1" t="s">
-        <v>847</v>
+        <v>844</v>
       </c>
       <c r="E47" s="1" t="s">
         <v>453</v>
@@ -7634,7 +7629,7 @@
         <v>452</v>
       </c>
       <c r="D51" s="1" t="s">
-        <v>852</v>
+        <v>849</v>
       </c>
       <c r="E51" s="1" t="s">
         <v>453</v>
@@ -7652,7 +7647,7 @@
         <v>452</v>
       </c>
       <c r="D52" s="1" t="s">
-        <v>853</v>
+        <v>850</v>
       </c>
       <c r="E52" s="1" t="s">
         <v>453</v>
@@ -7725,65 +7720,65 @@
     </row>
     <row r="57" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A57" s="1" t="s">
-        <v>836</v>
+        <v>833</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>837</v>
+        <v>834</v>
       </c>
       <c r="C57" s="1" t="s">
-        <v>838</v>
+        <v>835</v>
       </c>
       <c r="D57" s="1"/>
       <c r="E57" s="1" t="s">
-        <v>839</v>
+        <v>836</v>
       </c>
       <c r="F57" s="7"/>
     </row>
     <row r="58" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A58" s="1" t="s">
-        <v>840</v>
+        <v>837</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>841</v>
+        <v>838</v>
       </c>
       <c r="C58" s="1" t="s">
-        <v>838</v>
+        <v>835</v>
       </c>
       <c r="D58" s="1"/>
       <c r="E58" s="1" t="s">
-        <v>839</v>
+        <v>836</v>
       </c>
       <c r="F58" s="7"/>
     </row>
     <row r="59" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A59" s="1" t="s">
-        <v>842</v>
+        <v>839</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>843</v>
+        <v>840</v>
       </c>
       <c r="C59" s="1" t="s">
-        <v>838</v>
+        <v>835</v>
       </c>
       <c r="D59" s="1"/>
       <c r="E59" s="1" t="s">
-        <v>844</v>
+        <v>841</v>
       </c>
       <c r="F59" s="7"/>
     </row>
     <row r="60" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A60" s="1" t="s">
-        <v>845</v>
+        <v>842</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>846</v>
+        <v>843</v>
       </c>
       <c r="C60" s="1" t="s">
-        <v>838</v>
+        <v>835</v>
       </c>
       <c r="D60" s="1"/>
       <c r="E60" s="1" t="s">
-        <v>844</v>
+        <v>841</v>
       </c>
       <c r="F60" s="7"/>
     </row>
@@ -7829,13 +7824,13 @@
     </row>
     <row r="64" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A64" s="1" t="s">
-        <v>778</v>
+        <v>775</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>779</v>
+        <v>776</v>
       </c>
       <c r="C64" s="1" t="s">
-        <v>780</v>
+        <v>777</v>
       </c>
       <c r="D64" s="1"/>
       <c r="E64" s="1" t="s">
@@ -7846,11 +7841,11 @@
       <c r="A65" s="1" t="s">
         <v>393</v>
       </c>
-      <c r="B65" s="16" t="s">
+      <c r="B65" s="15" t="s">
         <v>396</v>
       </c>
       <c r="C65" s="1" t="s">
-        <v>780</v>
+        <v>777</v>
       </c>
       <c r="D65" s="1"/>
       <c r="E65" s="1" t="s">
@@ -7864,29 +7859,27 @@
       <c r="A66" s="1" t="s">
         <v>394</v>
       </c>
-      <c r="B66" s="16" t="s">
+      <c r="B66" s="15" t="s">
         <v>397</v>
       </c>
       <c r="C66" s="1" t="s">
-        <v>780</v>
+        <v>777</v>
       </c>
       <c r="D66" s="1"/>
       <c r="E66" s="1" t="s">
         <v>399</v>
       </c>
-      <c r="F66" s="8" t="s">
-        <v>773</v>
-      </c>
+      <c r="F66" s="8"/>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A67" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="B67" s="16" t="s">
+      <c r="B67" s="15" t="s">
         <v>398</v>
       </c>
       <c r="C67" s="1" t="s">
-        <v>780</v>
+        <v>777</v>
       </c>
       <c r="D67" s="1"/>
       <c r="E67" s="1" t="s">
@@ -7898,7 +7891,7 @@
       <c r="A68" s="1" t="s">
         <v>406</v>
       </c>
-      <c r="B68" s="16" t="s">
+      <c r="B68" s="15" t="s">
         <v>400</v>
       </c>
       <c r="C68" s="1" t="s">
@@ -7992,10 +7985,10 @@
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A74" s="1" t="s">
-        <v>781</v>
+        <v>778</v>
       </c>
       <c r="B74" s="1" t="s">
-        <v>782</v>
+        <v>779</v>
       </c>
       <c r="C74" s="1" t="s">
         <v>412</v>
@@ -8040,289 +8033,289 @@
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A77" s="1" t="s">
-        <v>783</v>
+        <v>780</v>
       </c>
       <c r="B77" s="1" t="s">
-        <v>784</v>
+        <v>781</v>
       </c>
       <c r="C77" s="1" t="s">
-        <v>785</v>
+        <v>782</v>
       </c>
       <c r="D77" s="1"/>
       <c r="E77" s="1" t="s">
-        <v>786</v>
+        <v>783</v>
       </c>
       <c r="F77" s="8"/>
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A78" s="1" t="s">
-        <v>787</v>
+        <v>784</v>
       </c>
       <c r="B78" s="1" t="s">
-        <v>788</v>
+        <v>785</v>
       </c>
       <c r="C78" s="1" t="s">
-        <v>785</v>
+        <v>782</v>
       </c>
       <c r="D78" s="1"/>
       <c r="E78" s="1" t="s">
-        <v>786</v>
+        <v>783</v>
       </c>
       <c r="F78" s="8"/>
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A79" s="1" t="s">
-        <v>789</v>
+        <v>786</v>
       </c>
       <c r="B79" s="1" t="s">
-        <v>790</v>
+        <v>787</v>
       </c>
       <c r="C79" s="1" t="s">
-        <v>785</v>
+        <v>782</v>
       </c>
       <c r="D79" s="1"/>
       <c r="E79" s="1" t="s">
-        <v>786</v>
+        <v>783</v>
       </c>
       <c r="F79" s="8"/>
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A80" s="1" t="s">
-        <v>791</v>
+        <v>788</v>
       </c>
       <c r="B80" s="1" t="s">
-        <v>792</v>
+        <v>789</v>
       </c>
       <c r="C80" s="1" t="s">
-        <v>785</v>
+        <v>782</v>
       </c>
       <c r="D80" s="1"/>
       <c r="E80" s="1" t="s">
-        <v>786</v>
+        <v>783</v>
       </c>
       <c r="F80" s="8"/>
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A81" s="1" t="s">
-        <v>793</v>
+        <v>790</v>
       </c>
       <c r="B81" s="1" t="s">
-        <v>794</v>
+        <v>791</v>
       </c>
       <c r="C81" s="1" t="s">
-        <v>785</v>
+        <v>782</v>
       </c>
       <c r="D81" s="1"/>
       <c r="E81" s="1" t="s">
-        <v>786</v>
+        <v>783</v>
       </c>
       <c r="F81" s="8"/>
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A82" s="1" t="s">
-        <v>795</v>
+        <v>792</v>
       </c>
       <c r="B82" s="1" t="s">
-        <v>796</v>
+        <v>793</v>
       </c>
       <c r="C82" s="1" t="s">
-        <v>797</v>
+        <v>794</v>
       </c>
       <c r="D82" s="1"/>
       <c r="E82" s="1" t="s">
-        <v>786</v>
+        <v>783</v>
       </c>
       <c r="F82" s="8"/>
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A83" s="1" t="s">
-        <v>798</v>
+        <v>795</v>
       </c>
       <c r="B83" s="1" t="s">
-        <v>799</v>
+        <v>796</v>
       </c>
       <c r="C83" s="1" t="s">
-        <v>797</v>
+        <v>794</v>
       </c>
       <c r="D83" s="1"/>
       <c r="E83" s="1" t="s">
-        <v>800</v>
+        <v>797</v>
       </c>
       <c r="F83" s="8"/>
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A84" s="1" t="s">
-        <v>801</v>
+        <v>798</v>
       </c>
       <c r="B84" s="1" t="s">
-        <v>802</v>
+        <v>799</v>
       </c>
       <c r="C84" s="1" t="s">
-        <v>797</v>
+        <v>794</v>
       </c>
       <c r="D84" s="1"/>
       <c r="E84" s="1" t="s">
-        <v>800</v>
+        <v>797</v>
       </c>
       <c r="F84" s="8"/>
     </row>
     <row r="85" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A85" s="1" t="s">
-        <v>803</v>
+        <v>800</v>
       </c>
       <c r="B85" s="1" t="s">
-        <v>804</v>
+        <v>801</v>
       </c>
       <c r="C85" s="1" t="s">
-        <v>797</v>
+        <v>794</v>
       </c>
       <c r="D85" s="1"/>
       <c r="E85" s="1" t="s">
-        <v>800</v>
+        <v>797</v>
       </c>
       <c r="F85" s="8"/>
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A86" s="1" t="s">
-        <v>805</v>
+        <v>802</v>
       </c>
       <c r="B86" s="1" t="s">
-        <v>806</v>
+        <v>803</v>
       </c>
       <c r="C86" s="1" t="s">
-        <v>797</v>
+        <v>794</v>
       </c>
       <c r="D86" s="1"/>
       <c r="E86" s="1" t="s">
-        <v>807</v>
+        <v>804</v>
       </c>
       <c r="F86" s="8"/>
     </row>
     <row r="87" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A87" s="1" t="s">
-        <v>808</v>
+        <v>805</v>
       </c>
       <c r="B87" s="1" t="s">
-        <v>809</v>
+        <v>806</v>
       </c>
       <c r="C87" s="1" t="s">
-        <v>797</v>
+        <v>794</v>
       </c>
       <c r="D87" s="1"/>
       <c r="E87" s="1" t="s">
-        <v>807</v>
+        <v>804</v>
       </c>
       <c r="F87" s="8"/>
     </row>
     <row r="88" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A88" s="1" t="s">
-        <v>810</v>
+        <v>807</v>
       </c>
       <c r="B88" s="1" t="s">
-        <v>811</v>
+        <v>808</v>
       </c>
       <c r="C88" s="1" t="s">
-        <v>797</v>
+        <v>794</v>
       </c>
       <c r="D88" s="1"/>
       <c r="E88" s="1" t="s">
-        <v>807</v>
+        <v>804</v>
       </c>
       <c r="F88" s="8"/>
     </row>
     <row r="89" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A89" s="1" t="s">
-        <v>812</v>
+        <v>809</v>
       </c>
       <c r="B89" s="1" t="s">
-        <v>813</v>
+        <v>810</v>
       </c>
       <c r="C89" s="1" t="s">
-        <v>797</v>
+        <v>794</v>
       </c>
       <c r="D89" s="1"/>
       <c r="E89" s="1" t="s">
-        <v>814</v>
+        <v>811</v>
       </c>
       <c r="F89" s="8"/>
     </row>
     <row r="90" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A90" s="1" t="s">
-        <v>815</v>
+        <v>812</v>
       </c>
       <c r="B90" s="1" t="s">
-        <v>816</v>
+        <v>813</v>
       </c>
       <c r="C90" s="1" t="s">
-        <v>797</v>
+        <v>794</v>
       </c>
       <c r="D90" s="1"/>
       <c r="E90" s="1" t="s">
-        <v>814</v>
+        <v>811</v>
       </c>
       <c r="F90" s="8"/>
     </row>
     <row r="91" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A91" s="1" t="s">
-        <v>817</v>
+        <v>814</v>
       </c>
       <c r="B91" s="1" t="s">
-        <v>818</v>
+        <v>815</v>
       </c>
       <c r="C91" s="1" t="s">
-        <v>797</v>
+        <v>794</v>
       </c>
       <c r="D91" s="1"/>
       <c r="E91" s="1" t="s">
-        <v>814</v>
+        <v>811</v>
       </c>
       <c r="F91" s="8"/>
     </row>
     <row r="92" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A92" s="1" t="s">
-        <v>819</v>
+        <v>816</v>
       </c>
       <c r="B92" t="s">
-        <v>820</v>
+        <v>817</v>
       </c>
       <c r="C92" s="1" t="s">
-        <v>797</v>
+        <v>794</v>
       </c>
       <c r="D92" s="1"/>
       <c r="E92" s="1" t="s">
-        <v>814</v>
+        <v>811</v>
       </c>
       <c r="F92" s="8"/>
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A93" s="1" t="s">
-        <v>821</v>
+        <v>818</v>
       </c>
       <c r="B93" s="1" t="s">
-        <v>822</v>
+        <v>819</v>
       </c>
       <c r="C93" s="1" t="s">
-        <v>823</v>
+        <v>820</v>
       </c>
       <c r="D93" s="1"/>
       <c r="E93" s="1" t="s">
-        <v>824</v>
+        <v>821</v>
       </c>
       <c r="F93" s="8"/>
     </row>
     <row r="94" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A94" s="1" t="s">
-        <v>825</v>
+        <v>822</v>
       </c>
       <c r="B94" s="1" t="s">
-        <v>826</v>
+        <v>823</v>
       </c>
       <c r="C94" s="1" t="s">
-        <v>823</v>
+        <v>820</v>
       </c>
       <c r="D94" s="1"/>
       <c r="E94" s="1" t="s">
-        <v>824</v>
+        <v>821</v>
       </c>
       <c r="F94" s="8"/>
     </row>
@@ -8408,10 +8401,10 @@
     </row>
     <row r="100" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A100" s="1" t="s">
-        <v>827</v>
+        <v>824</v>
       </c>
       <c r="B100" t="s">
-        <v>828</v>
+        <v>825</v>
       </c>
       <c r="C100" s="1" t="s">
         <v>432</v>
@@ -8440,33 +8433,33 @@
     </row>
     <row r="102" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A102" s="1" t="s">
-        <v>829</v>
+        <v>826</v>
       </c>
       <c r="B102" s="1" t="s">
-        <v>830</v>
+        <v>827</v>
       </c>
       <c r="C102" s="1" t="s">
         <v>437</v>
       </c>
       <c r="D102" s="1"/>
       <c r="E102" s="1" t="s">
-        <v>831</v>
+        <v>828</v>
       </c>
       <c r="F102" s="8"/>
     </row>
     <row r="103" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A103" s="1" t="s">
-        <v>832</v>
+        <v>829</v>
       </c>
       <c r="B103" s="1" t="s">
-        <v>833</v>
+        <v>830</v>
       </c>
       <c r="C103" s="1" t="s">
         <v>437</v>
       </c>
       <c r="D103" s="1"/>
       <c r="E103" s="1" t="s">
-        <v>831</v>
+        <v>828</v>
       </c>
       <c r="F103" s="8"/>
     </row>
@@ -8488,10 +8481,10 @@
     </row>
     <row r="105" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A105" s="1" t="s">
-        <v>834</v>
+        <v>831</v>
       </c>
       <c r="B105" s="1" t="s">
-        <v>835</v>
+        <v>832</v>
       </c>
       <c r="C105" s="1" t="s">
         <v>437</v>
@@ -8536,349 +8529,216 @@
     </row>
     <row r="108" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A108" s="1" t="s">
-        <v>454</v>
+        <v>469</v>
       </c>
       <c r="B108" s="1" t="s">
-        <v>446</v>
+        <v>466</v>
       </c>
       <c r="C108" s="1" t="s">
-        <v>452</v>
-      </c>
-      <c r="D108" s="1" t="s">
-        <v>855</v>
-      </c>
+        <v>468</v>
+      </c>
+      <c r="D108" s="1"/>
       <c r="E108" s="1" t="s">
-        <v>453</v>
+        <v>471</v>
       </c>
       <c r="F108" s="8"/>
     </row>
     <row r="109" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A109" s="1" t="s">
-        <v>455</v>
+        <v>470</v>
       </c>
       <c r="B109" s="1" t="s">
-        <v>447</v>
+        <v>467</v>
       </c>
       <c r="C109" s="1" t="s">
-        <v>452</v>
-      </c>
-      <c r="D109" s="1" t="s">
-        <v>855</v>
-      </c>
+        <v>468</v>
+      </c>
+      <c r="D109" s="1"/>
       <c r="E109" s="1" t="s">
-        <v>453</v>
+        <v>471</v>
       </c>
       <c r="F109" s="8"/>
     </row>
     <row r="110" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A110" s="1" t="s">
-        <v>456</v>
+        <v>833</v>
       </c>
       <c r="B110" s="1" t="s">
-        <v>448</v>
+        <v>834</v>
       </c>
       <c r="C110" s="1" t="s">
-        <v>452</v>
-      </c>
-      <c r="D110" s="1" t="s">
-        <v>855</v>
-      </c>
+        <v>835</v>
+      </c>
+      <c r="D110" s="1"/>
       <c r="E110" s="1" t="s">
-        <v>453</v>
+        <v>836</v>
       </c>
       <c r="F110" s="8"/>
     </row>
     <row r="111" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A111" s="1" t="s">
-        <v>457</v>
+        <v>837</v>
       </c>
       <c r="B111" s="1" t="s">
-        <v>449</v>
+        <v>838</v>
       </c>
       <c r="C111" s="1" t="s">
-        <v>452</v>
-      </c>
-      <c r="D111" s="1" t="s">
-        <v>855</v>
-      </c>
+        <v>835</v>
+      </c>
+      <c r="D111" s="1"/>
       <c r="E111" s="1" t="s">
-        <v>453</v>
+        <v>836</v>
       </c>
       <c r="F111" s="8"/>
     </row>
     <row r="112" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A112" s="1" t="s">
-        <v>458</v>
+        <v>839</v>
       </c>
       <c r="B112" s="1" t="s">
-        <v>450</v>
+        <v>840</v>
       </c>
       <c r="C112" s="1" t="s">
-        <v>452</v>
-      </c>
-      <c r="D112" s="1" t="s">
-        <v>855</v>
-      </c>
+        <v>835</v>
+      </c>
+      <c r="D112" s="1"/>
       <c r="E112" s="1" t="s">
-        <v>453</v>
+        <v>841</v>
       </c>
       <c r="F112" s="8"/>
     </row>
-    <row r="113" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A113" s="1" t="s">
-        <v>459</v>
+        <v>842</v>
       </c>
       <c r="B113" s="1" t="s">
-        <v>451</v>
+        <v>843</v>
       </c>
       <c r="C113" s="1" t="s">
-        <v>452</v>
-      </c>
-      <c r="D113" s="1" t="s">
-        <v>855</v>
-      </c>
+        <v>835</v>
+      </c>
+      <c r="D113" s="1"/>
       <c r="E113" s="1" t="s">
-        <v>453</v>
+        <v>841</v>
       </c>
       <c r="F113" s="8"/>
     </row>
-    <row r="114" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A114" s="1" t="s">
-        <v>463</v>
-      </c>
-      <c r="B114" s="1" t="s">
-        <v>460</v>
-      </c>
-      <c r="C114" s="1" t="s">
-        <v>462</v>
-      </c>
-      <c r="D114" s="1" t="s">
-        <v>855</v>
-      </c>
-      <c r="E114" s="1" t="s">
-        <v>465</v>
-      </c>
+    <row r="114" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A114" s="1"/>
+      <c r="B114" s="1"/>
+      <c r="C114" s="1"/>
+      <c r="D114" s="1"/>
+      <c r="E114" s="1"/>
       <c r="F114" s="8"/>
     </row>
-    <row r="115" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A115" s="1" t="s">
-        <v>464</v>
-      </c>
-      <c r="B115" t="s">
-        <v>461</v>
-      </c>
-      <c r="C115" s="1" t="s">
-        <v>462</v>
-      </c>
-      <c r="D115" s="1" t="s">
-        <v>855</v>
-      </c>
-      <c r="E115" s="1" t="s">
-        <v>465</v>
-      </c>
-      <c r="F115" s="8"/>
-    </row>
-    <row r="116" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A116" s="1" t="s">
-        <v>469</v>
-      </c>
-      <c r="B116" s="1" t="s">
-        <v>466</v>
-      </c>
-      <c r="C116" s="1" t="s">
-        <v>468</v>
-      </c>
-      <c r="D116" s="1"/>
-      <c r="E116" s="1" t="s">
-        <v>471</v>
-      </c>
-      <c r="F116" s="8"/>
-    </row>
-    <row r="117" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A117" s="1" t="s">
-        <v>470</v>
-      </c>
-      <c r="B117" s="1" t="s">
-        <v>467</v>
-      </c>
-      <c r="C117" s="1" t="s">
-        <v>468</v>
-      </c>
-      <c r="D117" s="1"/>
-      <c r="E117" s="1" t="s">
-        <v>471</v>
-      </c>
-      <c r="F117" s="8"/>
-    </row>
-    <row r="118" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A118" s="1" t="s">
-        <v>836</v>
-      </c>
-      <c r="B118" s="1" t="s">
-        <v>837</v>
-      </c>
-      <c r="C118" s="1" t="s">
-        <v>838</v>
-      </c>
+    <row r="115" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A115" s="17" t="s">
+        <v>774</v>
+      </c>
+      <c r="B115" s="17"/>
+      <c r="C115" s="17"/>
+      <c r="D115" s="17"/>
+      <c r="E115" s="17"/>
+      <c r="F115" s="17"/>
+    </row>
+    <row r="116" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A116" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="B116" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="C116" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="D116" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="E116" s="2" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="117" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A117" s="34"/>
+      <c r="B117" s="34"/>
+      <c r="C117" s="34"/>
+      <c r="D117" s="34"/>
+      <c r="E117" s="1"/>
+    </row>
+    <row r="118" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A118" s="1"/>
+      <c r="B118" s="1"/>
+      <c r="C118" s="1"/>
       <c r="D118" s="1"/>
-      <c r="E118" s="1" t="s">
-        <v>839</v>
-      </c>
-      <c r="F118" s="8"/>
-    </row>
-    <row r="119" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A119" s="1" t="s">
-        <v>840</v>
-      </c>
-      <c r="B119" s="1" t="s">
-        <v>841</v>
-      </c>
-      <c r="C119" s="1" t="s">
-        <v>838</v>
-      </c>
+      <c r="E118" s="1"/>
+    </row>
+    <row r="119" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A119" s="1"/>
+      <c r="B119" s="1"/>
+      <c r="C119" s="1"/>
       <c r="D119" s="1"/>
-      <c r="E119" s="1" t="s">
-        <v>839</v>
-      </c>
-      <c r="F119" s="8"/>
-    </row>
-    <row r="120" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A120" s="1" t="s">
-        <v>842</v>
-      </c>
-      <c r="B120" s="1" t="s">
-        <v>843</v>
-      </c>
-      <c r="C120" s="1" t="s">
-        <v>838</v>
-      </c>
+      <c r="E119" s="1"/>
+    </row>
+    <row r="120" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A120" s="1"/>
+      <c r="B120" s="1"/>
+      <c r="C120" s="1"/>
       <c r="D120" s="1"/>
-      <c r="E120" s="1" t="s">
-        <v>844</v>
-      </c>
-      <c r="F120" s="8"/>
-    </row>
-    <row r="121" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A121" s="1" t="s">
-        <v>845</v>
-      </c>
-      <c r="B121" s="1" t="s">
-        <v>846</v>
-      </c>
-      <c r="C121" s="1" t="s">
-        <v>838</v>
-      </c>
+      <c r="E120" s="1"/>
+    </row>
+    <row r="121" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A121" s="1"/>
+      <c r="B121" s="1"/>
+      <c r="C121" s="1"/>
       <c r="D121" s="1"/>
-      <c r="E121" s="1" t="s">
-        <v>844</v>
-      </c>
-      <c r="F121" s="8"/>
-    </row>
-    <row r="122" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="E121" s="1"/>
+    </row>
+    <row r="122" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A122" s="1"/>
       <c r="B122" s="1"/>
       <c r="C122" s="1"/>
       <c r="D122" s="1"/>
       <c r="E122" s="1"/>
-      <c r="F122" s="8"/>
-    </row>
-    <row r="123" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A123" s="27" t="s">
-        <v>776</v>
-      </c>
-      <c r="B123" s="27"/>
-      <c r="C123" s="27"/>
-      <c r="D123" s="27"/>
-      <c r="E123" s="27"/>
-      <c r="F123" s="27"/>
-      <c r="G123" s="27"/>
-      <c r="H123" s="27"/>
-      <c r="I123" s="27"/>
-      <c r="J123" s="27"/>
-      <c r="K123" s="27"/>
-    </row>
-    <row r="124" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A124" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="B124" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="C124" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="D124" s="2" t="s">
-        <v>116</v>
-      </c>
-      <c r="E124" s="2" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="125" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A125" s="9" t="s">
-        <v>474</v>
-      </c>
-      <c r="B125" s="1"/>
-      <c r="C125" s="1"/>
-      <c r="D125" s="1" t="s">
-        <v>777</v>
-      </c>
-      <c r="E125" s="1"/>
-    </row>
-    <row r="126" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A126" s="1"/>
-      <c r="B126" s="1"/>
-      <c r="C126" s="1"/>
-      <c r="D126" s="1"/>
-      <c r="E126" s="1"/>
-    </row>
-    <row r="127" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A127" s="1"/>
-      <c r="B127" s="1"/>
-      <c r="C127" s="1"/>
-      <c r="D127" s="1"/>
-      <c r="E127" s="1"/>
-    </row>
-    <row r="128" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A128" s="1"/>
-      <c r="B128" s="1"/>
-      <c r="C128" s="1"/>
-      <c r="D128" s="1"/>
-      <c r="E128" s="1"/>
-    </row>
-    <row r="129" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A129" s="1"/>
-      <c r="B129" s="1"/>
-      <c r="C129" s="1"/>
-      <c r="D129" s="1"/>
-      <c r="E129" s="1"/>
-    </row>
-    <row r="130" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A130" s="1"/>
-      <c r="B130" s="1"/>
-      <c r="C130" s="1"/>
-      <c r="D130" s="1"/>
-      <c r="E130" s="1"/>
-    </row>
-    <row r="131" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A131" s="1"/>
-      <c r="B131" s="1"/>
-      <c r="C131" s="1"/>
-      <c r="D131" s="1"/>
-      <c r="E131" s="1"/>
-    </row>
-    <row r="132" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A132" s="1"/>
-      <c r="B132" s="1"/>
-      <c r="C132" s="1"/>
-      <c r="D132" s="1"/>
-      <c r="E132" s="1"/>
+      <c r="F122" s="35"/>
+      <c r="G122" s="35"/>
+      <c r="H122" s="35"/>
+      <c r="I122" s="35"/>
+      <c r="J122" s="35"/>
+      <c r="K122" s="35"/>
+      <c r="L122" s="35"/>
+    </row>
+    <row r="123" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A123" s="1"/>
+      <c r="B123" s="1"/>
+      <c r="C123" s="1"/>
+      <c r="D123" s="1"/>
+      <c r="E123" s="1"/>
+      <c r="F123" s="35"/>
+      <c r="G123" s="36"/>
+      <c r="H123" s="36"/>
+      <c r="I123" s="36"/>
+      <c r="J123" s="36"/>
+      <c r="K123" s="36"/>
+      <c r="L123" s="35"/>
+    </row>
+    <row r="124" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A124" s="1"/>
+      <c r="B124" s="1"/>
+      <c r="C124" s="1"/>
+      <c r="D124" s="1"/>
+      <c r="E124" s="1"/>
+      <c r="F124" s="35"/>
+      <c r="G124" s="35"/>
+      <c r="H124" s="35"/>
+      <c r="I124" s="35"/>
+      <c r="J124" s="35"/>
+      <c r="K124" s="35"/>
+      <c r="L124" s="35"/>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="2">
     <mergeCell ref="A1:K1"/>
     <mergeCell ref="A62:K62"/>
-    <mergeCell ref="A123:K123"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -9092,7 +8952,7 @@
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A16" s="29" t="s">
-        <v>776</v>
+        <v>774</v>
       </c>
       <c r="B16" s="29"/>
       <c r="C16" s="29"/>
@@ -9303,109 +9163,109 @@
     </row>
     <row r="29" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="B29" s="6" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="C29" s="1" t="s">
+        <v>516</v>
+      </c>
+      <c r="D29" s="1" t="s">
         <v>517</v>
       </c>
-      <c r="D29" s="1" t="s">
+      <c r="E29" s="1" t="s">
         <v>518</v>
-      </c>
-      <c r="E29" s="1" t="s">
-        <v>519</v>
       </c>
     </row>
     <row r="30" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A30" s="1" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="B30" s="6" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="D30" s="1"/>
       <c r="E30" s="1" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
     </row>
     <row r="31" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A31" s="1" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="B31" s="6" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="D31" s="1"/>
       <c r="E31" s="1" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
     </row>
     <row r="32" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A32" s="1" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="B32" s="6" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="D32" s="1"/>
       <c r="E32" s="1" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A33" s="1" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
       <c r="B33" s="6" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="D33" s="1"/>
       <c r="E33" s="1" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A34" s="1" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="B34" s="6" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="D34" s="1"/>
       <c r="E34" s="1" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A35" s="1" t="s">
+        <v>515</v>
+      </c>
+      <c r="B35" s="6" t="s">
+        <v>525</v>
+      </c>
+      <c r="C35" s="1" t="s">
         <v>516</v>
-      </c>
-      <c r="B35" s="6" t="s">
-        <v>526</v>
-      </c>
-      <c r="C35" s="1" t="s">
-        <v>517</v>
       </c>
       <c r="D35" s="1"/>
       <c r="E35" s="1" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
     </row>
   </sheetData>
@@ -10057,7 +9917,7 @@
     </row>
     <row r="42" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A42" s="31" t="s">
-        <v>776</v>
+        <v>774</v>
       </c>
       <c r="B42" s="31"/>
       <c r="C42" s="31"/>
@@ -10090,7 +9950,7 @@
     <row r="44" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A44" s="1"/>
       <c r="B44" s="1" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="C44" s="1"/>
       <c r="D44" s="1"/>
@@ -10240,7 +10100,7 @@
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A11" s="33" t="s">
-        <v>776</v>
+        <v>774</v>
       </c>
       <c r="B11" s="33"/>
       <c r="C11" s="33"/>
@@ -10272,971 +10132,971 @@
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>528</v>
+        <v>527</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="D14" s="1"/>
       <c r="E14" s="1" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="D15" s="1"/>
       <c r="E15" s="1" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="D16" s="1"/>
       <c r="E16" s="1" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="D17" s="1"/>
       <c r="E17" s="1" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="D18" s="1"/>
       <c r="E18" s="1" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
-        <v>610</v>
+        <v>609</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>536</v>
+        <v>535</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>668</v>
+        <v>667</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
-        <v>611</v>
+        <v>610</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>538</v>
+        <v>537</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>537</v>
+        <v>536</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="D21" s="1"/>
       <c r="E21" s="1" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>540</v>
+        <v>539</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="D22" s="1"/>
       <c r="E22" s="1" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>541</v>
+        <v>540</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="D23" s="1"/>
       <c r="E23" s="1" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="D24" s="1"/>
       <c r="E24" s="1" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A25" s="1" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>543</v>
+        <v>542</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="D25" s="1"/>
       <c r="E25" s="1" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>545</v>
+        <v>544</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A27" s="1" t="s">
-        <v>618</v>
+        <v>617</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="D27" s="1"/>
       <c r="E27" s="1" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A28" s="1" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>547</v>
+        <v>546</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="D28" s="1"/>
       <c r="E28" s="1" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
-        <v>620</v>
+        <v>619</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="D29" s="1"/>
       <c r="E29" s="1" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A30" s="1" t="s">
-        <v>621</v>
+        <v>620</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>549</v>
+        <v>548</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="D30" s="1"/>
       <c r="E30" s="1" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A31" s="1" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="D31" s="1"/>
       <c r="E31" s="1" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A32" s="1" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>552</v>
+        <v>551</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>671</v>
+        <v>670</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A33" s="1" t="s">
-        <v>624</v>
+        <v>623</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="D33" s="1"/>
       <c r="E33" s="1" t="s">
-        <v>671</v>
+        <v>670</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A34" s="1" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="D34" s="1"/>
       <c r="E34" s="1" t="s">
-        <v>671</v>
+        <v>670</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A35" s="1" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="D35" s="1"/>
       <c r="E35" s="1" t="s">
-        <v>671</v>
+        <v>670</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A36" s="1" t="s">
-        <v>627</v>
+        <v>626</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="D36" s="1"/>
       <c r="E36" s="1" t="s">
-        <v>671</v>
+        <v>670</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A37" s="1" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
       <c r="E37" s="1" t="s">
-        <v>672</v>
+        <v>671</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A38" s="1" t="s">
-        <v>632</v>
+        <v>631</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>559</v>
+        <v>558</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="D38" s="1"/>
       <c r="E38" s="1" t="s">
-        <v>672</v>
+        <v>671</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A39" s="1" t="s">
-        <v>633</v>
+        <v>632</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>560</v>
+        <v>559</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="D39" s="1"/>
       <c r="E39" s="1" t="s">
-        <v>672</v>
+        <v>671</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A40" s="1" t="s">
-        <v>634</v>
+        <v>633</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="D40" s="1"/>
       <c r="E40" s="1" t="s">
-        <v>672</v>
+        <v>671</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A41" s="1" t="s">
-        <v>635</v>
+        <v>634</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="D41" s="1"/>
       <c r="E41" s="1" t="s">
-        <v>672</v>
+        <v>671</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A42" s="1" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="D42" s="1"/>
       <c r="E42" s="1" t="s">
-        <v>672</v>
+        <v>671</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A43" s="1" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="E43" s="1" t="s">
-        <v>673</v>
+        <v>672</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A44" s="1" t="s">
-        <v>630</v>
+        <v>629</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="D44" s="1"/>
       <c r="E44" s="1" t="s">
-        <v>673</v>
+        <v>672</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A45" s="1" t="s">
-        <v>639</v>
+        <v>638</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="D45" s="1"/>
       <c r="E45" s="1" t="s">
-        <v>673</v>
+        <v>672</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A46" s="1" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="D46" s="1"/>
       <c r="E46" s="1" t="s">
-        <v>673</v>
+        <v>672</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A47" s="1" t="s">
-        <v>636</v>
+        <v>635</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="D47" s="1"/>
       <c r="E47" s="1" t="s">
-        <v>673</v>
+        <v>672</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A48" s="1" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="D48" s="1"/>
       <c r="E48" s="1" t="s">
-        <v>673</v>
+        <v>672</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A49" s="1" t="s">
-        <v>638</v>
+        <v>637</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="D49" s="1" t="s">
-        <v>571</v>
+        <v>570</v>
       </c>
       <c r="E49" s="1" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A50" s="1" t="s">
-        <v>641</v>
+        <v>640</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="C50" s="1" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="D50" s="1"/>
       <c r="E50" s="1" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A51" s="1" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="C51" s="1" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="D51" s="1"/>
       <c r="E51" s="1" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A52" s="1" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="C52" s="1" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="D52" s="1"/>
       <c r="E52" s="1" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A53" s="1" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
       <c r="C53" s="1" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="D53" s="1"/>
       <c r="E53" s="1" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A54" s="1" t="s">
-        <v>645</v>
+        <v>644</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="C54" s="1" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="E54" s="1" t="s">
-        <v>675</v>
+        <v>674</v>
       </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A55" s="1" t="s">
-        <v>646</v>
+        <v>645</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="C55" s="1" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="D55" s="1"/>
       <c r="E55" s="1" t="s">
-        <v>675</v>
+        <v>674</v>
       </c>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A56" s="1" t="s">
-        <v>647</v>
+        <v>646</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="C56" s="1" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="D56" s="1"/>
       <c r="E56" s="1" t="s">
-        <v>675</v>
+        <v>674</v>
       </c>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A57" s="1" t="s">
-        <v>648</v>
+        <v>647</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="C57" s="1" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="D57" s="1"/>
       <c r="E57" s="1" t="s">
-        <v>675</v>
+        <v>674</v>
       </c>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A58" s="1" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>582</v>
+        <v>581</v>
       </c>
       <c r="C58" s="1" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="D58" s="1"/>
       <c r="E58" s="1" t="s">
-        <v>675</v>
+        <v>674</v>
       </c>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A59" s="1" t="s">
-        <v>650</v>
+        <v>649</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
       <c r="C59" s="1" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="D59" s="1"/>
       <c r="E59" s="1" t="s">
-        <v>675</v>
+        <v>674</v>
       </c>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A60" s="1" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>585</v>
+        <v>584</v>
       </c>
       <c r="C60" s="1" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="D60" s="1" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="E60" s="1" t="s">
-        <v>768</v>
+        <v>767</v>
       </c>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A61" s="1" t="s">
-        <v>652</v>
+        <v>651</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="C61" s="1" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="D61" s="1"/>
       <c r="E61" s="1" t="s">
-        <v>768</v>
+        <v>767</v>
       </c>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A62" s="1" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="C62" s="1" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="D62" s="1"/>
       <c r="E62" s="1" t="s">
-        <v>768</v>
+        <v>767</v>
       </c>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A63" s="1" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>588</v>
+        <v>587</v>
       </c>
       <c r="C63" s="1" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="D63" s="1"/>
       <c r="E63" s="1" t="s">
-        <v>768</v>
+        <v>767</v>
       </c>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A64" s="1" t="s">
-        <v>655</v>
+        <v>654</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
       <c r="C64" s="1" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="D64" s="1"/>
       <c r="E64" s="1" t="s">
-        <v>768</v>
+        <v>767</v>
       </c>
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A65" s="1" t="s">
-        <v>656</v>
+        <v>655</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="C65" s="1" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="D65" s="1"/>
       <c r="E65" s="1" t="s">
-        <v>768</v>
+        <v>767</v>
       </c>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A66" s="1" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
       <c r="C66" s="1" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="D66" s="1" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="E66" s="1" t="s">
-        <v>676</v>
+        <v>675</v>
       </c>
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A67" s="1" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="B67" s="1" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="C67" s="1" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="D67" s="1"/>
       <c r="E67" s="1" t="s">
-        <v>676</v>
+        <v>675</v>
       </c>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A68" s="1" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>594</v>
+        <v>593</v>
       </c>
       <c r="C68" s="1" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="D68" s="1"/>
       <c r="E68" s="1" t="s">
-        <v>676</v>
+        <v>675</v>
       </c>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A69" s="1" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="B69" s="1" t="s">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="C69" s="1" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="D69" s="1"/>
       <c r="E69" s="1" t="s">
-        <v>676</v>
+        <v>675</v>
       </c>
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A70" s="1" t="s">
-        <v>661</v>
+        <v>660</v>
       </c>
       <c r="B70" s="1" t="s">
-        <v>596</v>
+        <v>595</v>
       </c>
       <c r="C70" s="1" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="D70" s="1"/>
       <c r="E70" s="1" t="s">
-        <v>676</v>
+        <v>675</v>
       </c>
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A71" s="1" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="B71" s="1" t="s">
-        <v>598</v>
+        <v>597</v>
       </c>
       <c r="C71" s="1" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="D71" s="1" t="s">
-        <v>597</v>
+        <v>596</v>
       </c>
       <c r="E71" s="1" t="s">
-        <v>677</v>
+        <v>676</v>
       </c>
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A72" s="1" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
       <c r="B72" s="1" t="s">
-        <v>599</v>
+        <v>598</v>
       </c>
       <c r="C72" s="1" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="D72" s="1"/>
       <c r="E72" s="1" t="s">
-        <v>677</v>
+        <v>676</v>
       </c>
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A73" s="1" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="B73" s="1" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="C73" s="1" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="D73" s="1"/>
       <c r="E73" s="1" t="s">
-        <v>677</v>
+        <v>676</v>
       </c>
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A74" s="1" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="B74" s="1" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="C74" s="1" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="D74" s="1"/>
       <c r="E74" s="1" t="s">
-        <v>677</v>
+        <v>676</v>
       </c>
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A75" s="1" t="s">
-        <v>666</v>
+        <v>665</v>
       </c>
       <c r="B75" s="1" t="s">
+        <v>601</v>
+      </c>
+      <c r="C75" s="1" t="s">
         <v>602</v>
-      </c>
-      <c r="C75" s="1" t="s">
-        <v>603</v>
       </c>
       <c r="D75" s="1"/>
       <c r="E75" s="1" t="s">
-        <v>677</v>
+        <v>676</v>
       </c>
     </row>
   </sheetData>

</xml_diff>